<commit_message>
added excel file to gitignore
</commit_message>
<xml_diff>
--- a/report-vis.xlsx
+++ b/report-vis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\! CS\Y2\AI is taking over\cw\ai-garbage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A8B363-F5F6-4FC7-AE22-87DEC2D22CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D96942-2F04-4413-99B8-843452D433D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{82DBE9BC-AC51-4988-B415-6B972F3134D5}"/>
+    <workbookView xWindow="28680" yWindow="-12645" windowWidth="29040" windowHeight="15840" xr2:uid="{82DBE9BC-AC51-4988-B415-6B972F3134D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1134,103 +1134,79 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1245,13 +1221,13 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1311,73 +1287,97 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -6342,6 +6342,682 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>117</xdr:col>
+      <xdr:colOff>13855</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>41563</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>135</xdr:col>
+      <xdr:colOff>478675</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>20781</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="48" name="Picture 47">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32602446-A3D8-485B-FAE2-7E0F6BA02A9D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="72736364" y="1482436"/>
+          <a:ext cx="11430000" cy="9525000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>135</xdr:col>
+      <xdr:colOff>415637</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>27709</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>154</xdr:col>
+      <xdr:colOff>263237</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>10737</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="53" name="Picture 52">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{951542AB-2907-E09B-8A20-AE4CC8F62BBF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="84110946" y="1468582"/>
+          <a:ext cx="11430000" cy="9525000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>124</xdr:col>
+      <xdr:colOff>332509</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>3463</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>129</xdr:col>
+      <xdr:colOff>526473</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>128155</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="56" name="TextBox 55">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E512BE3A-8B85-88A0-8C07-6848FE46394D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="77351659" y="1527463"/>
+          <a:ext cx="3241964" cy="696192"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2800"/>
+            <a:t>PR Curve (Baseline)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>143</xdr:col>
+      <xdr:colOff>207824</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>9697</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>148</xdr:col>
+      <xdr:colOff>401788</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="57" name="TextBox 56">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B31F4764-D6FD-4C54-AFB3-F21468921FFB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="88809374" y="1533697"/>
+          <a:ext cx="3241964" cy="714203"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2800"/>
+            <a:t>PR Curve (Improved)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>116</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>140</xdr:col>
+      <xdr:colOff>383015</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>25753</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="58" name="Picture 57">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{465CD6EB-85C7-6DA3-8418-4F63A77C3359}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="72713850" y="11620500"/>
+          <a:ext cx="14441915" cy="7078063"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>116</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>133349</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>140</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>133</xdr:row>
+      <xdr:rowOff>99059</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="59" name="Picture 58">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A2B8BF71-A327-5F2D-D449-3030574C348B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="72618600" y="18611849"/>
+          <a:ext cx="14687550" cy="7343775"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>124</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>135</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="60" name="TextBox 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{673ECAEA-1AC0-8504-15C6-96F4598A9014}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="77038200" y="18630900"/>
+          <a:ext cx="6819900" cy="628650"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:sysClr val="window" lastClr="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="3200"/>
+            <a:t>Average</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="3200" baseline="0"/>
+            <a:t> Precision per class  (Improved)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="3200"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>124</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>135</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="61" name="TextBox 60">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2DE14C1-70A6-4823-9197-3AC2B901E8D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="77057250" y="11544300"/>
+          <a:ext cx="6819900" cy="628650"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="3200"/>
+            <a:t>Average</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="3200" baseline="0"/>
+            <a:t> Precision per class  (Baseline)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="3200"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>169</xdr:col>
+      <xdr:colOff>244116</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>69273</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>195</xdr:col>
+      <xdr:colOff>176242</xdr:colOff>
+      <xdr:row>123</xdr:row>
+      <xdr:rowOff>257869</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="62" name="Picture 61">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E198CA6-6ABA-5BED-BA76-452681DF549E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="104118571" y="11170228"/>
+          <a:ext cx="15691671" cy="10943186"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>144</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>66677</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>169</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>123</xdr:row>
+      <xdr:rowOff>200027</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="63" name="Picture 62">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{50708172-EC5E-BC1E-8FE3-21A71BA13214}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="88046379" y="12204248"/>
+          <a:ext cx="14967857" cy="11808279"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>150</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>76202</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>161</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>156212</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="64" name="TextBox 63">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7CB22A2-B04B-4337-97D9-80D7624AC525}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="91371964" y="12213773"/>
+          <a:ext cx="6852557" cy="651510"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="3200"/>
+            <a:t>Confusion Matrix - 100 classes (baseline)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>173</xdr:col>
+      <xdr:colOff>571501</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>12962</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>188</xdr:col>
+      <xdr:colOff>515736</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>25034</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="65" name="TextBox 64">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D41ED4E4-EC38-4713-A8EC-6AAEF1A75ECE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="106870501" y="11287098"/>
+          <a:ext cx="9036280" cy="548936"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="3200"/>
+            <a:t>Confusion Matrix - 100 classes (improved)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -6713,13 +7389,13 @@
       <c r="DL9" s="7"/>
     </row>
     <row r="10" spans="90:116" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="CL10" s="157" t="s">
+      <c r="CL10" s="81" t="s">
         <v>74</v>
       </c>
-      <c r="CM10" s="158" t="s">
+      <c r="CM10" s="82" t="s">
         <v>75</v>
       </c>
-      <c r="DD10" s="162" t="s">
+      <c r="DD10" s="88" t="s">
         <v>76</v>
       </c>
       <c r="DE10" s="7"/>
@@ -6732,10 +7408,10 @@
       <c r="DL10" s="7"/>
     </row>
     <row r="11" spans="90:116" x14ac:dyDescent="0.3">
-      <c r="CL11" s="159">
+      <c r="CL11" s="83">
         <v>100</v>
       </c>
-      <c r="CM11" s="164">
+      <c r="CM11" s="86">
         <v>0.314</v>
       </c>
       <c r="DA11" t="s">
@@ -6744,7 +7420,7 @@
       <c r="DB11" t="s">
         <v>79</v>
       </c>
-      <c r="DD11" s="162"/>
+      <c r="DD11" s="88"/>
       <c r="DE11" s="7"/>
       <c r="DF11" s="7"/>
       <c r="DG11" s="7"/>
@@ -6755,10 +7431,10 @@
       <c r="DL11" s="7"/>
     </row>
     <row r="12" spans="90:116" x14ac:dyDescent="0.3">
-      <c r="CL12" s="160">
+      <c r="CL12" s="84">
         <v>150</v>
       </c>
-      <c r="CM12" s="161">
+      <c r="CM12" s="85">
         <v>0.53400000000000003</v>
       </c>
       <c r="DA12">
@@ -6767,7 +7443,7 @@
       <c r="DB12">
         <v>0.90300000000000002</v>
       </c>
-      <c r="DD12" s="162"/>
+      <c r="DD12" s="88"/>
       <c r="DE12" s="7"/>
       <c r="DF12" s="7"/>
       <c r="DG12" s="7"/>
@@ -6778,10 +7454,10 @@
       <c r="DL12" s="7"/>
     </row>
     <row r="13" spans="90:116" x14ac:dyDescent="0.3">
-      <c r="CL13" s="159">
+      <c r="CL13" s="83">
         <v>200</v>
       </c>
-      <c r="CM13" s="164">
+      <c r="CM13" s="86">
         <v>0.65700000000000003</v>
       </c>
       <c r="DA13">
@@ -6790,7 +7466,7 @@
       <c r="DB13">
         <v>0.90500000000000003</v>
       </c>
-      <c r="DD13" s="162"/>
+      <c r="DD13" s="88"/>
       <c r="DE13" s="7"/>
       <c r="DF13" s="7"/>
       <c r="DG13" s="7"/>
@@ -6801,10 +7477,10 @@
       <c r="DL13" s="7"/>
     </row>
     <row r="14" spans="90:116" x14ac:dyDescent="0.3">
-      <c r="CL14" s="160">
+      <c r="CL14" s="84">
         <v>250</v>
       </c>
-      <c r="CM14" s="161">
+      <c r="CM14" s="85">
         <v>0.754</v>
       </c>
       <c r="DA14">
@@ -6813,7 +7489,7 @@
       <c r="DB14">
         <v>0.90600000000000003</v>
       </c>
-      <c r="DD14" s="162"/>
+      <c r="DD14" s="88"/>
       <c r="DE14" s="7"/>
       <c r="DF14" s="7"/>
       <c r="DG14" s="7"/>
@@ -6824,10 +7500,10 @@
       <c r="DL14" s="7"/>
     </row>
     <row r="15" spans="90:116" x14ac:dyDescent="0.3">
-      <c r="CL15" s="159">
+      <c r="CL15" s="83">
         <v>300</v>
       </c>
-      <c r="CM15" s="164">
+      <c r="CM15" s="86">
         <v>0.81699999999999995</v>
       </c>
       <c r="CO15">
@@ -6848,7 +7524,7 @@
       <c r="DB15">
         <v>0.90900000000000003</v>
       </c>
-      <c r="DD15" s="162"/>
+      <c r="DD15" s="88"/>
       <c r="DE15" s="7"/>
       <c r="DF15" s="7"/>
       <c r="DG15" s="7"/>
@@ -6859,10 +7535,10 @@
       <c r="DL15" s="7"/>
     </row>
     <row r="16" spans="90:116" x14ac:dyDescent="0.3">
-      <c r="CL16" s="160">
+      <c r="CL16" s="84">
         <v>350</v>
       </c>
-      <c r="CM16" s="161">
+      <c r="CM16" s="85">
         <v>0.84899999999999998</v>
       </c>
       <c r="CQ16" s="7"/>
@@ -6880,7 +7556,7 @@
       <c r="DB16">
         <v>0.91</v>
       </c>
-      <c r="DD16" s="162"/>
+      <c r="DD16" s="88"/>
       <c r="DE16" s="7"/>
       <c r="DF16" s="7"/>
       <c r="DG16" s="7"/>
@@ -6891,13 +7567,13 @@
       <c r="DL16" s="7"/>
     </row>
     <row r="17" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL17" s="159">
+      <c r="CL17" s="83">
         <v>400</v>
       </c>
-      <c r="CM17" s="164">
+      <c r="CM17" s="86">
         <v>0.87</v>
       </c>
-      <c r="CQ17" s="162" t="s">
+      <c r="CQ17" s="88" t="s">
         <v>76</v>
       </c>
       <c r="CR17" s="7"/>
@@ -6914,7 +7590,7 @@
       <c r="DB17">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD17" s="162"/>
+      <c r="DD17" s="88"/>
       <c r="DE17" s="7"/>
       <c r="DF17" s="7"/>
       <c r="DG17" s="7"/>
@@ -6925,13 +7601,13 @@
       <c r="DL17" s="7"/>
     </row>
     <row r="18" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL18" s="160">
+      <c r="CL18" s="84">
         <v>450</v>
       </c>
-      <c r="CM18" s="161">
+      <c r="CM18" s="85">
         <v>0.88800000000000001</v>
       </c>
-      <c r="CQ18" s="162"/>
+      <c r="CQ18" s="88"/>
       <c r="CR18" s="7"/>
       <c r="CS18" s="7"/>
       <c r="CT18" s="7"/>
@@ -6946,7 +7622,7 @@
       <c r="DB18">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD18" s="162"/>
+      <c r="DD18" s="88"/>
       <c r="DE18" s="7"/>
       <c r="DF18" s="7"/>
       <c r="DG18" s="7"/>
@@ -6957,13 +7633,13 @@
       <c r="DL18" s="7"/>
     </row>
     <row r="19" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL19" s="159">
+      <c r="CL19" s="83">
         <v>500</v>
       </c>
-      <c r="CM19" s="164">
+      <c r="CM19" s="86">
         <v>0.90100000000000002</v>
       </c>
-      <c r="CQ19" s="162"/>
+      <c r="CQ19" s="88"/>
       <c r="CR19" s="7"/>
       <c r="CS19" s="7"/>
       <c r="CT19" s="7"/>
@@ -6978,7 +7654,7 @@
       <c r="DB19">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD19" s="162"/>
+      <c r="DD19" s="88"/>
       <c r="DE19" s="7"/>
       <c r="DF19" s="7"/>
       <c r="DG19" s="7"/>
@@ -6989,13 +7665,13 @@
       <c r="DL19" s="7"/>
     </row>
     <row r="20" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL20" s="160">
+      <c r="CL20" s="84">
         <v>525</v>
       </c>
-      <c r="CM20" s="161">
+      <c r="CM20" s="85">
         <v>0.90400000000000003</v>
       </c>
-      <c r="CQ20" s="162"/>
+      <c r="CQ20" s="88"/>
       <c r="CR20" s="7"/>
       <c r="CS20" s="7"/>
       <c r="CT20" s="7"/>
@@ -7010,7 +7686,7 @@
       <c r="DB20">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD20" s="162"/>
+      <c r="DD20" s="88"/>
       <c r="DE20" s="7"/>
       <c r="DF20" s="7"/>
       <c r="DG20" s="7"/>
@@ -7021,13 +7697,13 @@
       <c r="DL20" s="7"/>
     </row>
     <row r="21" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL21" s="160">
+      <c r="CL21" s="84">
         <v>550</v>
       </c>
-      <c r="CM21" s="161">
+      <c r="CM21" s="85">
         <v>0.90900000000000003</v>
       </c>
-      <c r="CQ21" s="162"/>
+      <c r="CQ21" s="88"/>
       <c r="CR21" s="7"/>
       <c r="CS21" s="7"/>
       <c r="CT21" s="7"/>
@@ -7042,7 +7718,7 @@
       <c r="DB21">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD21" s="162"/>
+      <c r="DD21" s="88"/>
       <c r="DE21" s="7"/>
       <c r="DF21" s="7"/>
       <c r="DG21" s="7"/>
@@ -7053,13 +7729,13 @@
       <c r="DL21" s="7"/>
     </row>
     <row r="22" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL22" s="160">
+      <c r="CL22" s="84">
         <v>560</v>
       </c>
-      <c r="CM22" s="161">
+      <c r="CM22" s="85">
         <v>0.90900000000000003</v>
       </c>
-      <c r="CQ22" s="162"/>
+      <c r="CQ22" s="88"/>
       <c r="CR22" s="7"/>
       <c r="CS22" s="7"/>
       <c r="CT22" s="7"/>
@@ -7074,7 +7750,7 @@
       <c r="DB22">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD22" s="162"/>
+      <c r="DD22" s="88"/>
       <c r="DE22" s="7"/>
       <c r="DF22" s="7"/>
       <c r="DG22" s="7"/>
@@ -7085,13 +7761,13 @@
       <c r="DL22" s="7"/>
     </row>
     <row r="23" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL23" s="159">
+      <c r="CL23" s="83">
         <v>565</v>
       </c>
-      <c r="CM23" s="164">
+      <c r="CM23" s="86">
         <v>0.91200000000000003</v>
       </c>
-      <c r="CQ23" s="162"/>
+      <c r="CQ23" s="88"/>
       <c r="CR23" s="7"/>
       <c r="CS23" s="7"/>
       <c r="CT23" s="7"/>
@@ -7106,7 +7782,7 @@
       <c r="DB23">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD23" s="162"/>
+      <c r="DD23" s="88"/>
       <c r="DE23" s="7"/>
       <c r="DF23" s="7"/>
       <c r="DG23" s="7"/>
@@ -7117,13 +7793,13 @@
       <c r="DL23" s="7"/>
     </row>
     <row r="24" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL24" s="160">
+      <c r="CL24" s="84">
         <v>570</v>
       </c>
-      <c r="CM24" s="161">
+      <c r="CM24" s="85">
         <v>0.91</v>
       </c>
-      <c r="CQ24" s="162"/>
+      <c r="CQ24" s="88"/>
       <c r="CR24" s="7"/>
       <c r="CS24" s="7"/>
       <c r="CT24" s="7"/>
@@ -7138,7 +7814,7 @@
       <c r="DB24">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD24" s="162"/>
+      <c r="DD24" s="88"/>
       <c r="DE24" s="7"/>
       <c r="DF24" s="7"/>
       <c r="DG24" s="7"/>
@@ -7149,13 +7825,13 @@
       <c r="DL24" s="7"/>
     </row>
     <row r="25" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL25" s="159">
+      <c r="CL25" s="83">
         <v>575</v>
       </c>
-      <c r="CM25" s="164">
+      <c r="CM25" s="86">
         <v>0.91100000000000003</v>
       </c>
-      <c r="CQ25" s="162"/>
+      <c r="CQ25" s="88"/>
       <c r="CR25" s="7"/>
       <c r="CS25" s="7"/>
       <c r="CT25" s="7"/>
@@ -7181,13 +7857,13 @@
       <c r="DL25" s="7"/>
     </row>
     <row r="26" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL26" s="160">
+      <c r="CL26" s="84">
         <v>580</v>
       </c>
-      <c r="CM26" s="161">
+      <c r="CM26" s="85">
         <v>0.91100000000000003</v>
       </c>
-      <c r="CQ26" s="162"/>
+      <c r="CQ26" s="88"/>
       <c r="CR26" s="7"/>
       <c r="CS26" s="7"/>
       <c r="CT26" s="7"/>
@@ -7198,24 +7874,24 @@
       <c r="CY26" s="7"/>
       <c r="DD26" s="7"/>
       <c r="DE26" s="7"/>
-      <c r="DF26" s="163" t="s">
+      <c r="DF26" s="87" t="s">
         <v>80</v>
       </c>
-      <c r="DG26" s="163"/>
-      <c r="DH26" s="163"/>
-      <c r="DI26" s="163"/>
-      <c r="DJ26" s="163"/>
-      <c r="DK26" s="163"/>
+      <c r="DG26" s="87"/>
+      <c r="DH26" s="87"/>
+      <c r="DI26" s="87"/>
+      <c r="DJ26" s="87"/>
+      <c r="DK26" s="87"/>
       <c r="DL26" s="7"/>
     </row>
     <row r="27" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL27" s="160">
+      <c r="CL27" s="84">
         <v>585</v>
       </c>
-      <c r="CM27" s="161">
+      <c r="CM27" s="85">
         <v>0.90900000000000003</v>
       </c>
-      <c r="CQ27" s="162"/>
+      <c r="CQ27" s="88"/>
       <c r="CR27" s="7"/>
       <c r="CS27" s="7"/>
       <c r="CT27" s="7"/>
@@ -7226,22 +7902,22 @@
       <c r="CY27" s="7"/>
       <c r="DD27" s="7"/>
       <c r="DE27" s="7"/>
-      <c r="DF27" s="163"/>
-      <c r="DG27" s="163"/>
-      <c r="DH27" s="163"/>
-      <c r="DI27" s="163"/>
-      <c r="DJ27" s="163"/>
-      <c r="DK27" s="163"/>
+      <c r="DF27" s="87"/>
+      <c r="DG27" s="87"/>
+      <c r="DH27" s="87"/>
+      <c r="DI27" s="87"/>
+      <c r="DJ27" s="87"/>
+      <c r="DK27" s="87"/>
       <c r="DL27" s="7"/>
     </row>
     <row r="28" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL28" s="160">
+      <c r="CL28" s="84">
         <v>590</v>
       </c>
-      <c r="CM28" s="161">
+      <c r="CM28" s="85">
         <v>0.90600000000000003</v>
       </c>
-      <c r="CQ28" s="162"/>
+      <c r="CQ28" s="88"/>
       <c r="CR28" s="7"/>
       <c r="CS28" s="7"/>
       <c r="CT28" s="7"/>
@@ -7252,13 +7928,13 @@
       <c r="CY28" s="7"/>
     </row>
     <row r="29" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL29" s="159">
+      <c r="CL29" s="83">
         <v>600</v>
       </c>
-      <c r="CM29" s="164">
+      <c r="CM29" s="86">
         <v>0.90600000000000003</v>
       </c>
-      <c r="CQ29" s="162"/>
+      <c r="CQ29" s="88"/>
       <c r="CR29" s="7"/>
       <c r="CS29" s="7"/>
       <c r="CT29" s="7"/>
@@ -7269,13 +7945,13 @@
       <c r="CY29" s="7"/>
     </row>
     <row r="30" spans="2:116" x14ac:dyDescent="0.3">
-      <c r="CL30" s="160">
+      <c r="CL30" s="84">
         <v>650</v>
       </c>
-      <c r="CM30" s="161">
+      <c r="CM30" s="85">
         <v>0.90800000000000003</v>
       </c>
-      <c r="CQ30" s="162"/>
+      <c r="CQ30" s="88"/>
       <c r="CR30" s="7"/>
       <c r="CS30" s="7"/>
       <c r="CT30" s="7"/>
@@ -7297,10 +7973,10 @@
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
-      <c r="CL31" s="159">
+      <c r="CL31" s="83">
         <v>700</v>
       </c>
-      <c r="CM31" s="164">
+      <c r="CM31" s="86">
         <v>0.90500000000000003</v>
       </c>
       <c r="CQ31" s="7"/>
@@ -7366,22 +8042,22 @@
       <c r="BA32" s="7"/>
       <c r="BB32" s="7"/>
       <c r="BC32" s="7"/>
-      <c r="CL32" s="160">
+      <c r="CL32" s="84">
         <v>750</v>
       </c>
-      <c r="CM32" s="161">
+      <c r="CM32" s="85">
         <v>0.90800000000000003</v>
       </c>
       <c r="CQ32" s="7"/>
-      <c r="CR32" s="163" t="s">
+      <c r="CR32" s="87" t="s">
         <v>77</v>
       </c>
-      <c r="CS32" s="163"/>
-      <c r="CT32" s="163"/>
-      <c r="CU32" s="163"/>
-      <c r="CV32" s="163"/>
-      <c r="CW32" s="163"/>
-      <c r="CX32" s="163"/>
+      <c r="CS32" s="87"/>
+      <c r="CT32" s="87"/>
+      <c r="CU32" s="87"/>
+      <c r="CV32" s="87"/>
+      <c r="CW32" s="87"/>
+      <c r="CX32" s="87"/>
       <c r="CY32" s="7"/>
     </row>
     <row r="33" spans="2:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7397,11 +8073,11 @@
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
       <c r="M33" s="7"/>
-      <c r="N33" s="91" t="s">
+      <c r="N33" s="144" t="s">
         <v>28</v>
       </c>
-      <c r="O33" s="81"/>
-      <c r="P33" s="81"/>
+      <c r="O33" s="147"/>
+      <c r="P33" s="147"/>
       <c r="Q33" s="7"/>
       <c r="R33" s="7"/>
       <c r="S33" s="7"/>
@@ -7422,13 +8098,13 @@
       <c r="AJ33" s="7"/>
       <c r="AK33" s="7"/>
       <c r="AL33" s="7"/>
-      <c r="AM33" s="91" t="s">
+      <c r="AM33" s="144" t="s">
         <v>48</v>
       </c>
-      <c r="AN33" s="91"/>
-      <c r="AO33" s="91"/>
-      <c r="AP33" s="91"/>
-      <c r="AQ33" s="91"/>
+      <c r="AN33" s="144"/>
+      <c r="AO33" s="144"/>
+      <c r="AP33" s="144"/>
+      <c r="AQ33" s="144"/>
       <c r="AR33" s="7"/>
       <c r="AS33" s="7"/>
       <c r="AT33" s="7"/>
@@ -7441,47 +8117,47 @@
       <c r="BA33" s="7"/>
       <c r="BB33" s="7"/>
       <c r="BC33" s="7"/>
-      <c r="CL33" s="159">
+      <c r="CL33" s="83">
         <v>800</v>
       </c>
-      <c r="CM33" s="164">
+      <c r="CM33" s="86">
         <v>0.90800000000000003</v>
       </c>
       <c r="CQ33" s="7"/>
-      <c r="CR33" s="163"/>
-      <c r="CS33" s="163"/>
-      <c r="CT33" s="163"/>
-      <c r="CU33" s="163"/>
-      <c r="CV33" s="163"/>
-      <c r="CW33" s="163"/>
-      <c r="CX33" s="163"/>
+      <c r="CR33" s="87"/>
+      <c r="CS33" s="87"/>
+      <c r="CT33" s="87"/>
+      <c r="CU33" s="87"/>
+      <c r="CV33" s="87"/>
+      <c r="CW33" s="87"/>
+      <c r="CX33" s="87"/>
       <c r="CY33" s="7"/>
     </row>
     <row r="34" spans="2:103" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
-      <c r="E34" s="89" t="s">
+      <c r="E34" s="156" t="s">
         <v>12</v>
       </c>
-      <c r="F34" s="90"/>
-      <c r="G34" s="90"/>
-      <c r="H34" s="90"/>
-      <c r="I34" s="90"/>
+      <c r="F34" s="150"/>
+      <c r="G34" s="150"/>
+      <c r="H34" s="150"/>
+      <c r="I34" s="150"/>
       <c r="J34" s="7"/>
       <c r="K34" s="7"/>
       <c r="L34" s="7"/>
       <c r="M34" s="7"/>
-      <c r="N34" s="81"/>
-      <c r="O34" s="81"/>
-      <c r="P34" s="81"/>
+      <c r="N34" s="147"/>
+      <c r="O34" s="147"/>
+      <c r="P34" s="147"/>
       <c r="Q34" s="7"/>
       <c r="R34" s="7"/>
-      <c r="S34" s="91" t="s">
+      <c r="S34" s="144" t="s">
         <v>30</v>
       </c>
-      <c r="T34" s="94"/>
-      <c r="U34" s="94"/>
+      <c r="T34" s="158"/>
+      <c r="U34" s="158"/>
       <c r="V34" s="7"/>
       <c r="W34" s="7"/>
       <c r="X34" s="7"/>
@@ -7489,25 +8165,25 @@
       <c r="AB34" s="7"/>
       <c r="AC34" s="7"/>
       <c r="AD34" s="7"/>
-      <c r="AE34" s="89" t="s">
+      <c r="AE34" s="156" t="s">
         <v>12</v>
       </c>
-      <c r="AF34" s="90"/>
-      <c r="AG34" s="90"/>
-      <c r="AH34" s="90"/>
-      <c r="AI34" s="90"/>
+      <c r="AF34" s="150"/>
+      <c r="AG34" s="150"/>
+      <c r="AH34" s="150"/>
+      <c r="AI34" s="150"/>
       <c r="AJ34" s="7"/>
       <c r="AK34" s="7"/>
       <c r="AL34" s="7"/>
-      <c r="AM34" s="91"/>
-      <c r="AN34" s="91"/>
-      <c r="AO34" s="91"/>
-      <c r="AP34" s="91"/>
-      <c r="AQ34" s="91"/>
+      <c r="AM34" s="144"/>
+      <c r="AN34" s="144"/>
+      <c r="AO34" s="144"/>
+      <c r="AP34" s="144"/>
+      <c r="AQ34" s="144"/>
       <c r="AR34" s="7"/>
-      <c r="AS34" s="91"/>
-      <c r="AT34" s="94"/>
-      <c r="AU34" s="94"/>
+      <c r="AS34" s="144"/>
+      <c r="AT34" s="158"/>
+      <c r="AU34" s="158"/>
       <c r="AV34" s="7"/>
       <c r="AW34" s="7"/>
       <c r="AX34" s="7"/>
@@ -7521,11 +8197,11 @@
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="90"/>
-      <c r="F35" s="90"/>
-      <c r="G35" s="90"/>
-      <c r="H35" s="90"/>
-      <c r="I35" s="90"/>
+      <c r="E35" s="150"/>
+      <c r="F35" s="150"/>
+      <c r="G35" s="150"/>
+      <c r="H35" s="150"/>
+      <c r="I35" s="150"/>
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
       <c r="L35" s="7"/>
@@ -7545,11 +8221,11 @@
       <c r="AB35" s="7"/>
       <c r="AC35" s="7"/>
       <c r="AD35" s="7"/>
-      <c r="AE35" s="90"/>
-      <c r="AF35" s="90"/>
-      <c r="AG35" s="90"/>
-      <c r="AH35" s="90"/>
-      <c r="AI35" s="90"/>
+      <c r="AE35" s="150"/>
+      <c r="AF35" s="150"/>
+      <c r="AG35" s="150"/>
+      <c r="AH35" s="150"/>
+      <c r="AI35" s="150"/>
       <c r="AJ35" s="7"/>
       <c r="AK35" s="7"/>
       <c r="AL35" s="7"/>
@@ -7649,10 +8325,10 @@
       <c r="T37" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="U37" s="86" t="s">
+      <c r="U37" s="149" t="s">
         <v>31</v>
       </c>
-      <c r="V37" s="86"/>
+      <c r="V37" s="149"/>
       <c r="W37" s="7"/>
       <c r="X37" s="7"/>
       <c r="Y37" s="7"/>
@@ -7677,8 +8353,8 @@
       <c r="AR37" s="7"/>
       <c r="AS37" s="7"/>
       <c r="AT37" s="7"/>
-      <c r="AU37" s="86"/>
-      <c r="AV37" s="86"/>
+      <c r="AU37" s="149"/>
+      <c r="AV37" s="149"/>
       <c r="AW37" s="7"/>
       <c r="AX37" s="7"/>
       <c r="AY37" s="7"/>
@@ -7716,11 +8392,11 @@
       <c r="Q38" s="7"/>
       <c r="R38" s="7"/>
       <c r="S38" s="7"/>
-      <c r="T38" s="92" t="s">
+      <c r="T38" s="112" t="s">
         <v>13</v>
       </c>
-      <c r="U38" s="86"/>
-      <c r="V38" s="86"/>
+      <c r="U38" s="149"/>
+      <c r="V38" s="149"/>
       <c r="W38" s="7"/>
       <c r="X38" s="7"/>
       <c r="Y38" s="7"/>
@@ -7752,9 +8428,9 @@
       <c r="AQ38" s="7"/>
       <c r="AR38" s="7"/>
       <c r="AS38" s="7"/>
-      <c r="AT38" s="90"/>
-      <c r="AU38" s="86"/>
-      <c r="AV38" s="86"/>
+      <c r="AT38" s="150"/>
+      <c r="AU38" s="149"/>
+      <c r="AV38" s="149"/>
       <c r="AW38" s="7"/>
       <c r="AX38" s="7"/>
       <c r="AY38" s="7"/>
@@ -7782,13 +8458,13 @@
       <c r="Q39" s="7"/>
       <c r="R39" s="7"/>
       <c r="S39" s="7"/>
-      <c r="T39" s="93"/>
-      <c r="U39" s="86"/>
-      <c r="V39" s="86"/>
+      <c r="T39" s="157"/>
+      <c r="U39" s="149"/>
+      <c r="V39" s="149"/>
       <c r="W39" s="7"/>
       <c r="X39" s="7"/>
       <c r="AB39" s="7"/>
-      <c r="AC39" s="110"/>
+      <c r="AC39" s="137"/>
       <c r="AD39" s="6"/>
       <c r="AE39" s="17"/>
       <c r="AF39" s="6"/>
@@ -7796,7 +8472,7 @@
       <c r="AH39" s="6"/>
       <c r="AI39" s="17"/>
       <c r="AJ39" s="6"/>
-      <c r="AK39" s="92"/>
+      <c r="AK39" s="112"/>
       <c r="AL39" s="7"/>
       <c r="AM39" s="7"/>
       <c r="AN39" s="7"/>
@@ -7805,9 +8481,9 @@
       <c r="AQ39" s="7"/>
       <c r="AR39" s="7"/>
       <c r="AS39" s="7"/>
-      <c r="AT39" s="90"/>
-      <c r="AU39" s="86"/>
-      <c r="AV39" s="86"/>
+      <c r="AT39" s="150"/>
+      <c r="AU39" s="149"/>
+      <c r="AV39" s="149"/>
       <c r="AW39" s="7"/>
       <c r="AX39" s="7"/>
       <c r="AY39" s="7"/>
@@ -7837,13 +8513,13 @@
       <c r="Q40" s="7"/>
       <c r="R40" s="7"/>
       <c r="S40" s="7"/>
-      <c r="T40" s="88"/>
-      <c r="U40" s="86"/>
-      <c r="V40" s="86"/>
+      <c r="T40" s="164"/>
+      <c r="U40" s="149"/>
+      <c r="V40" s="149"/>
       <c r="W40" s="7"/>
       <c r="X40" s="7"/>
       <c r="AB40" s="7"/>
-      <c r="AC40" s="110"/>
+      <c r="AC40" s="137"/>
       <c r="AD40" s="6"/>
       <c r="AE40" s="17"/>
       <c r="AF40" s="6"/>
@@ -7851,7 +8527,7 @@
       <c r="AH40" s="6"/>
       <c r="AI40" s="17"/>
       <c r="AJ40" s="6"/>
-      <c r="AK40" s="92"/>
+      <c r="AK40" s="112"/>
       <c r="AL40" s="7"/>
       <c r="AM40" s="7"/>
       <c r="AN40" s="7"/>
@@ -7863,8 +8539,8 @@
       <c r="AR40" s="7"/>
       <c r="AS40" s="7"/>
       <c r="AT40" s="7"/>
-      <c r="AU40" s="86"/>
-      <c r="AV40" s="86"/>
+      <c r="AU40" s="149"/>
+      <c r="AV40" s="149"/>
       <c r="AW40" s="7"/>
       <c r="AX40" s="7"/>
       <c r="AY40" s="7"/>
@@ -7887,14 +8563,14 @@
       <c r="L41" s="7"/>
       <c r="M41" s="7"/>
       <c r="N41" s="7"/>
-      <c r="O41" s="109" t="s">
+      <c r="O41" s="134" t="s">
         <v>15</v>
       </c>
       <c r="P41" s="7"/>
       <c r="Q41" s="7"/>
       <c r="R41" s="7"/>
       <c r="S41" s="7"/>
-      <c r="T41" s="88"/>
+      <c r="T41" s="164"/>
       <c r="U41" s="7"/>
       <c r="V41" s="7"/>
       <c r="W41" s="7"/>
@@ -7912,7 +8588,7 @@
       <c r="AL41" s="7"/>
       <c r="AM41" s="7"/>
       <c r="AN41" s="7"/>
-      <c r="AO41" s="98" t="s">
+      <c r="AO41" s="143" t="s">
         <v>15</v>
       </c>
       <c r="AP41" s="7"/>
@@ -7944,12 +8620,12 @@
       <c r="L42" s="7"/>
       <c r="M42" s="7"/>
       <c r="N42" s="7"/>
-      <c r="O42" s="109"/>
+      <c r="O42" s="134"/>
       <c r="P42" s="7"/>
       <c r="Q42" s="7"/>
       <c r="R42" s="7"/>
       <c r="S42" s="7"/>
-      <c r="T42" s="88"/>
+      <c r="T42" s="164"/>
       <c r="U42" s="7"/>
       <c r="V42" s="7"/>
       <c r="W42" s="7"/>
@@ -7967,7 +8643,7 @@
       <c r="AL42" s="7"/>
       <c r="AM42" s="7"/>
       <c r="AN42" s="7"/>
-      <c r="AO42" s="98"/>
+      <c r="AO42" s="143"/>
       <c r="AP42" s="7"/>
       <c r="AQ42" s="7"/>
       <c r="AR42" s="7"/>
@@ -7997,14 +8673,14 @@
       <c r="L43" s="7"/>
       <c r="M43" s="7"/>
       <c r="N43" s="7"/>
-      <c r="O43" s="103" t="s">
+      <c r="O43" s="139" t="s">
         <v>23</v>
       </c>
       <c r="P43" s="7"/>
       <c r="Q43" s="7"/>
       <c r="R43" s="7"/>
       <c r="S43" s="7"/>
-      <c r="T43" s="88"/>
+      <c r="T43" s="164"/>
       <c r="U43" s="7"/>
       <c r="V43" s="7"/>
       <c r="W43" s="7"/>
@@ -8022,7 +8698,7 @@
       <c r="AL43" s="7"/>
       <c r="AM43" s="7"/>
       <c r="AN43" s="7"/>
-      <c r="AO43" s="107" t="s">
+      <c r="AO43" s="151" t="s">
         <v>23</v>
       </c>
       <c r="AP43" s="7"/>
@@ -8054,18 +8730,18 @@
       <c r="L44" s="7"/>
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
-      <c r="O44" s="104"/>
+      <c r="O44" s="140"/>
       <c r="P44" s="7"/>
       <c r="Q44" s="7"/>
       <c r="R44" s="7"/>
       <c r="S44" s="7"/>
-      <c r="T44" s="88"/>
-      <c r="U44" s="82" t="s">
+      <c r="T44" s="164"/>
+      <c r="U44" s="161" t="s">
         <v>24</v>
       </c>
-      <c r="V44" s="83"/>
-      <c r="W44" s="83"/>
-      <c r="X44" s="83"/>
+      <c r="V44" s="153"/>
+      <c r="W44" s="153"/>
+      <c r="X44" s="153"/>
       <c r="AB44" s="7"/>
       <c r="AC44" s="19"/>
       <c r="AD44" s="6"/>
@@ -8079,16 +8755,16 @@
       <c r="AL44" s="7"/>
       <c r="AM44" s="7"/>
       <c r="AN44" s="7"/>
-      <c r="AO44" s="108"/>
+      <c r="AO44" s="152"/>
       <c r="AP44" s="7"/>
       <c r="AQ44" s="7"/>
       <c r="AR44" s="7"/>
       <c r="AS44" s="7"/>
       <c r="AT44" s="7"/>
-      <c r="AU44" s="83"/>
-      <c r="AV44" s="83"/>
-      <c r="AW44" s="83"/>
-      <c r="AX44" s="83"/>
+      <c r="AU44" s="153"/>
+      <c r="AV44" s="153"/>
+      <c r="AW44" s="153"/>
+      <c r="AX44" s="153"/>
       <c r="AY44" s="7"/>
       <c r="AZ44" s="7"/>
       <c r="BA44" s="7"/>
@@ -8109,18 +8785,18 @@
       <c r="L45" s="7"/>
       <c r="M45" s="7"/>
       <c r="N45" s="7"/>
-      <c r="O45" s="103" t="s">
+      <c r="O45" s="139" t="s">
         <v>22</v>
       </c>
       <c r="P45" s="7"/>
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="7"/>
-      <c r="T45" s="88"/>
-      <c r="U45" s="82"/>
-      <c r="V45" s="83"/>
-      <c r="W45" s="83"/>
-      <c r="X45" s="83"/>
+      <c r="T45" s="164"/>
+      <c r="U45" s="161"/>
+      <c r="V45" s="153"/>
+      <c r="W45" s="153"/>
+      <c r="X45" s="153"/>
       <c r="AB45" s="7"/>
       <c r="AC45" s="19"/>
       <c r="AD45" s="6"/>
@@ -8134,20 +8810,20 @@
       <c r="AL45" s="7"/>
       <c r="AM45" s="7"/>
       <c r="AN45" s="7"/>
-      <c r="AO45" s="107" t="s">
+      <c r="AO45" s="151" t="s">
         <v>22</v>
       </c>
-      <c r="AP45" s="95" t="s">
+      <c r="AP45" s="159" t="s">
         <v>67</v>
       </c>
-      <c r="AQ45" s="96"/>
-      <c r="AR45" s="96"/>
-      <c r="AS45" s="96"/>
-      <c r="AT45" s="96"/>
-      <c r="AU45" s="83"/>
-      <c r="AV45" s="83"/>
-      <c r="AW45" s="83"/>
-      <c r="AX45" s="83"/>
+      <c r="AQ45" s="160"/>
+      <c r="AR45" s="160"/>
+      <c r="AS45" s="160"/>
+      <c r="AT45" s="160"/>
+      <c r="AU45" s="153"/>
+      <c r="AV45" s="153"/>
+      <c r="AW45" s="153"/>
+      <c r="AX45" s="153"/>
       <c r="AY45" s="7"/>
       <c r="AZ45" s="7"/>
       <c r="BA45" s="7"/>
@@ -8178,17 +8854,17 @@
       <c r="L46" s="7"/>
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
-      <c r="O46" s="104"/>
+      <c r="O46" s="140"/>
       <c r="P46" s="7"/>
       <c r="Q46" s="7"/>
       <c r="R46" s="7"/>
       <c r="S46" s="7"/>
-      <c r="T46" s="88"/>
-      <c r="U46" s="87" t="s">
+      <c r="T46" s="164"/>
+      <c r="U46" s="163" t="s">
         <v>32</v>
       </c>
-      <c r="V46" s="81"/>
-      <c r="W46" s="81"/>
+      <c r="V46" s="147"/>
+      <c r="W46" s="147"/>
       <c r="X46" s="7"/>
       <c r="AB46" s="7"/>
       <c r="AC46" s="20">
@@ -8213,15 +8889,15 @@
       <c r="AL46" s="7"/>
       <c r="AM46" s="7"/>
       <c r="AN46" s="7"/>
-      <c r="AO46" s="108"/>
-      <c r="AP46" s="95"/>
-      <c r="AQ46" s="96"/>
-      <c r="AR46" s="96"/>
-      <c r="AS46" s="96"/>
-      <c r="AT46" s="96"/>
-      <c r="AU46" s="81"/>
-      <c r="AV46" s="81"/>
-      <c r="AW46" s="81"/>
+      <c r="AO46" s="152"/>
+      <c r="AP46" s="159"/>
+      <c r="AQ46" s="160"/>
+      <c r="AR46" s="160"/>
+      <c r="AS46" s="160"/>
+      <c r="AT46" s="160"/>
+      <c r="AU46" s="147"/>
+      <c r="AV46" s="147"/>
+      <c r="AW46" s="147"/>
       <c r="AX46" s="7"/>
       <c r="AY46" s="7"/>
       <c r="AZ46" s="7"/>
@@ -8253,14 +8929,14 @@
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
-      <c r="O47" s="109" t="s">
+      <c r="O47" s="134" t="s">
         <v>21</v>
       </c>
       <c r="P47" s="7"/>
       <c r="Q47" s="7"/>
       <c r="R47" s="7"/>
       <c r="S47" s="7"/>
-      <c r="T47" s="88"/>
+      <c r="T47" s="164"/>
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
@@ -8288,7 +8964,7 @@
       <c r="AL47" s="7"/>
       <c r="AM47" s="7"/>
       <c r="AN47" s="7"/>
-      <c r="AO47" s="98" t="s">
+      <c r="AO47" s="143" t="s">
         <v>21</v>
       </c>
       <c r="AP47" s="7"/>
@@ -8330,14 +9006,14 @@
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
-      <c r="O48" s="109"/>
-      <c r="P48" s="85" t="s">
+      <c r="O48" s="134"/>
+      <c r="P48" s="135" t="s">
         <v>27</v>
       </c>
-      <c r="Q48" s="97"/>
-      <c r="R48" s="97"/>
+      <c r="Q48" s="136"/>
+      <c r="R48" s="136"/>
       <c r="S48" s="7"/>
-      <c r="T48" s="88"/>
+      <c r="T48" s="164"/>
       <c r="U48" s="7"/>
       <c r="V48" s="7"/>
       <c r="W48" s="7"/>
@@ -8365,10 +9041,10 @@
       <c r="AL48" s="7"/>
       <c r="AM48" s="7"/>
       <c r="AN48" s="7"/>
-      <c r="AO48" s="98"/>
-      <c r="AP48" s="85"/>
-      <c r="AQ48" s="97"/>
-      <c r="AR48" s="97"/>
+      <c r="AO48" s="143"/>
+      <c r="AP48" s="135"/>
+      <c r="AQ48" s="136"/>
+      <c r="AR48" s="136"/>
       <c r="AS48" s="7"/>
       <c r="AT48" s="7"/>
       <c r="AU48" s="7"/>
@@ -8395,20 +9071,20 @@
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
       <c r="N49" s="7"/>
-      <c r="O49" s="109" t="s">
+      <c r="O49" s="134" t="s">
         <v>19</v>
       </c>
-      <c r="P49" s="97"/>
-      <c r="Q49" s="97"/>
-      <c r="R49" s="97"/>
+      <c r="P49" s="136"/>
+      <c r="Q49" s="136"/>
+      <c r="R49" s="136"/>
       <c r="S49" s="7"/>
-      <c r="T49" s="88"/>
-      <c r="U49" s="84" t="s">
+      <c r="T49" s="164"/>
+      <c r="U49" s="162" t="s">
         <v>25</v>
       </c>
-      <c r="V49" s="85"/>
-      <c r="W49" s="85"/>
-      <c r="X49" s="85"/>
+      <c r="V49" s="135"/>
+      <c r="W49" s="135"/>
+      <c r="X49" s="135"/>
       <c r="AB49" s="7"/>
       <c r="AC49" s="19"/>
       <c r="AD49" s="6"/>
@@ -8422,12 +9098,12 @@
       <c r="AL49" s="7"/>
       <c r="AM49" s="7"/>
       <c r="AN49" s="7"/>
-      <c r="AO49" s="98" t="s">
+      <c r="AO49" s="143" t="s">
         <v>19</v>
       </c>
-      <c r="AP49" s="97"/>
-      <c r="AQ49" s="97"/>
-      <c r="AR49" s="97"/>
+      <c r="AP49" s="136"/>
+      <c r="AQ49" s="136"/>
+      <c r="AR49" s="136"/>
       <c r="AS49" s="7"/>
       <c r="AT49" s="7"/>
       <c r="AU49" s="72"/>
@@ -8454,16 +9130,16 @@
       <c r="L50" s="7"/>
       <c r="M50" s="7"/>
       <c r="N50" s="7"/>
-      <c r="O50" s="109"/>
+      <c r="O50" s="134"/>
       <c r="P50" s="7"/>
       <c r="Q50" s="7"/>
       <c r="R50" s="7"/>
       <c r="S50" s="7"/>
       <c r="T50" s="12"/>
-      <c r="U50" s="84"/>
-      <c r="V50" s="85"/>
-      <c r="W50" s="85"/>
-      <c r="X50" s="85"/>
+      <c r="U50" s="162"/>
+      <c r="V50" s="135"/>
+      <c r="W50" s="135"/>
+      <c r="X50" s="135"/>
       <c r="AB50" s="7"/>
       <c r="AC50" s="19"/>
       <c r="AD50" s="6"/>
@@ -8477,7 +9153,7 @@
       <c r="AL50" s="7"/>
       <c r="AM50" s="7"/>
       <c r="AN50" s="7"/>
-      <c r="AO50" s="98"/>
+      <c r="AO50" s="143"/>
       <c r="AP50" s="7"/>
       <c r="AQ50" s="7"/>
       <c r="AR50" s="7"/>
@@ -8507,18 +9183,18 @@
       <c r="L51" s="7"/>
       <c r="M51" s="7"/>
       <c r="N51" s="7"/>
-      <c r="O51" s="103" t="s">
+      <c r="O51" s="139" t="s">
         <v>20</v>
       </c>
       <c r="P51" s="7"/>
       <c r="Q51" s="7"/>
       <c r="R51" s="7"/>
       <c r="S51" s="7"/>
-      <c r="T51" s="105"/>
-      <c r="U51" s="84"/>
-      <c r="V51" s="85"/>
-      <c r="W51" s="85"/>
-      <c r="X51" s="85"/>
+      <c r="T51" s="141"/>
+      <c r="U51" s="162"/>
+      <c r="V51" s="135"/>
+      <c r="W51" s="135"/>
+      <c r="X51" s="135"/>
       <c r="AB51" s="7"/>
       <c r="AC51" s="19"/>
       <c r="AD51" s="6"/>
@@ -8532,7 +9208,7 @@
       <c r="AL51" s="7"/>
       <c r="AM51" s="7"/>
       <c r="AN51" s="7"/>
-      <c r="AO51" s="111" t="s">
+      <c r="AO51" s="154" t="s">
         <v>20</v>
       </c>
       <c r="AP51" s="7"/>
@@ -8564,18 +9240,18 @@
       <c r="L52" s="7"/>
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
-      <c r="O52" s="104"/>
+      <c r="O52" s="140"/>
       <c r="P52" s="7"/>
       <c r="Q52" s="7"/>
       <c r="R52" s="7"/>
       <c r="S52" s="7"/>
-      <c r="T52" s="105"/>
-      <c r="U52" s="84" t="s">
+      <c r="T52" s="141"/>
+      <c r="U52" s="162" t="s">
         <v>26</v>
       </c>
-      <c r="V52" s="85"/>
-      <c r="W52" s="85"/>
-      <c r="X52" s="85"/>
+      <c r="V52" s="135"/>
+      <c r="W52" s="135"/>
+      <c r="X52" s="135"/>
       <c r="AB52" s="7"/>
       <c r="AC52" s="19"/>
       <c r="AD52" s="6"/>
@@ -8589,15 +9265,15 @@
       <c r="AL52" s="7"/>
       <c r="AM52" s="7"/>
       <c r="AN52" s="7"/>
-      <c r="AO52" s="112"/>
-      <c r="AP52" s="101" t="s">
+      <c r="AO52" s="155"/>
+      <c r="AP52" s="148" t="s">
         <v>65</v>
       </c>
-      <c r="AQ52" s="86"/>
-      <c r="AR52" s="86"/>
-      <c r="AS52" s="86"/>
-      <c r="AT52" s="86"/>
-      <c r="AU52" s="86"/>
+      <c r="AQ52" s="149"/>
+      <c r="AR52" s="149"/>
+      <c r="AS52" s="149"/>
+      <c r="AT52" s="149"/>
+      <c r="AU52" s="149"/>
       <c r="AV52" s="72"/>
       <c r="AW52" s="72"/>
       <c r="AX52" s="72"/>
@@ -8621,18 +9297,18 @@
       <c r="L53" s="7"/>
       <c r="M53" s="7"/>
       <c r="N53" s="7"/>
-      <c r="O53" s="103" t="s">
+      <c r="O53" s="139" t="s">
         <v>16</v>
       </c>
       <c r="P53" s="7"/>
       <c r="Q53" s="7"/>
       <c r="R53" s="7"/>
       <c r="S53" s="7"/>
-      <c r="T53" s="105"/>
-      <c r="U53" s="84"/>
-      <c r="V53" s="85"/>
-      <c r="W53" s="85"/>
-      <c r="X53" s="85"/>
+      <c r="T53" s="141"/>
+      <c r="U53" s="162"/>
+      <c r="V53" s="135"/>
+      <c r="W53" s="135"/>
+      <c r="X53" s="135"/>
       <c r="AB53" s="7"/>
       <c r="AC53" s="19"/>
       <c r="AD53" s="6"/>
@@ -8646,15 +9322,15 @@
       <c r="AL53" s="7"/>
       <c r="AM53" s="7"/>
       <c r="AN53" s="7"/>
-      <c r="AO53" s="111" t="s">
+      <c r="AO53" s="154" t="s">
         <v>16</v>
       </c>
-      <c r="AP53" s="101"/>
-      <c r="AQ53" s="86"/>
-      <c r="AR53" s="86"/>
-      <c r="AS53" s="86"/>
-      <c r="AT53" s="86"/>
-      <c r="AU53" s="86"/>
+      <c r="AP53" s="148"/>
+      <c r="AQ53" s="149"/>
+      <c r="AR53" s="149"/>
+      <c r="AS53" s="149"/>
+      <c r="AT53" s="149"/>
+      <c r="AU53" s="149"/>
       <c r="AV53" s="72"/>
       <c r="AW53" s="72"/>
       <c r="AX53" s="72"/>
@@ -8678,16 +9354,16 @@
       <c r="L54" s="7"/>
       <c r="M54" s="7"/>
       <c r="N54" s="7"/>
-      <c r="O54" s="104"/>
+      <c r="O54" s="140"/>
       <c r="P54" s="7"/>
       <c r="Q54" s="7"/>
       <c r="R54" s="7"/>
       <c r="S54" s="7"/>
-      <c r="T54" s="105"/>
-      <c r="U54" s="84"/>
-      <c r="V54" s="85"/>
-      <c r="W54" s="85"/>
-      <c r="X54" s="85"/>
+      <c r="T54" s="141"/>
+      <c r="U54" s="162"/>
+      <c r="V54" s="135"/>
+      <c r="W54" s="135"/>
+      <c r="X54" s="135"/>
       <c r="AB54" s="7"/>
       <c r="AC54" s="21"/>
       <c r="AD54" s="6"/>
@@ -8701,7 +9377,7 @@
       <c r="AL54" s="7"/>
       <c r="AM54" s="7"/>
       <c r="AN54" s="7"/>
-      <c r="AO54" s="112"/>
+      <c r="AO54" s="155"/>
       <c r="AP54" s="71"/>
       <c r="AQ54" s="70"/>
       <c r="AR54" s="70"/>
@@ -8731,14 +9407,14 @@
       <c r="L55" s="7"/>
       <c r="M55" s="7"/>
       <c r="N55" s="7"/>
-      <c r="O55" s="103" t="s">
+      <c r="O55" s="139" t="s">
         <v>17</v>
       </c>
       <c r="P55" s="7"/>
       <c r="Q55" s="7"/>
       <c r="R55" s="7"/>
       <c r="S55" s="7"/>
-      <c r="T55" s="106"/>
+      <c r="T55" s="142"/>
       <c r="U55" s="7"/>
       <c r="V55" s="7"/>
       <c r="W55" s="7"/>
@@ -8756,7 +9432,7 @@
       <c r="AL55" s="7"/>
       <c r="AM55" s="7"/>
       <c r="AN55" s="7"/>
-      <c r="AO55" s="113" t="s">
+      <c r="AO55" s="106" t="s">
         <v>17</v>
       </c>
       <c r="AP55" s="7"/>
@@ -8788,7 +9464,7 @@
       <c r="L56" s="7"/>
       <c r="M56" s="7"/>
       <c r="N56" s="7"/>
-      <c r="O56" s="104"/>
+      <c r="O56" s="140"/>
       <c r="P56" s="7"/>
       <c r="Q56" s="7"/>
       <c r="R56" s="7"/>
@@ -8811,14 +9487,14 @@
       <c r="AL56" s="7"/>
       <c r="AM56" s="7"/>
       <c r="AN56" s="7"/>
-      <c r="AO56" s="114"/>
-      <c r="AP56" s="101" t="s">
+      <c r="AO56" s="108"/>
+      <c r="AP56" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="AQ56" s="86"/>
-      <c r="AR56" s="86"/>
-      <c r="AS56" s="86"/>
-      <c r="AT56" s="86"/>
+      <c r="AQ56" s="149"/>
+      <c r="AR56" s="149"/>
+      <c r="AS56" s="149"/>
+      <c r="AT56" s="149"/>
       <c r="AU56" s="7"/>
       <c r="AV56" s="7"/>
       <c r="AW56" s="7"/>
@@ -8853,7 +9529,7 @@
       <c r="L57" s="7"/>
       <c r="M57" s="7"/>
       <c r="N57" s="7"/>
-      <c r="O57" s="103" t="s">
+      <c r="O57" s="139" t="s">
         <v>18</v>
       </c>
       <c r="P57" s="7"/>
@@ -8888,14 +9564,14 @@
       <c r="AL57" s="7"/>
       <c r="AM57" s="7"/>
       <c r="AN57" s="7"/>
-      <c r="AO57" s="113" t="s">
+      <c r="AO57" s="106" t="s">
         <v>18</v>
       </c>
-      <c r="AP57" s="101"/>
-      <c r="AQ57" s="86"/>
-      <c r="AR57" s="86"/>
-      <c r="AS57" s="86"/>
-      <c r="AT57" s="86"/>
+      <c r="AP57" s="148"/>
+      <c r="AQ57" s="149"/>
+      <c r="AR57" s="149"/>
+      <c r="AS57" s="149"/>
+      <c r="AT57" s="149"/>
       <c r="AU57" s="7"/>
       <c r="AV57" s="7"/>
       <c r="AW57" s="7"/>
@@ -8920,7 +9596,7 @@
       <c r="L58" s="7"/>
       <c r="M58" s="7"/>
       <c r="N58" s="7"/>
-      <c r="O58" s="104"/>
+      <c r="O58" s="140"/>
       <c r="P58" s="7"/>
       <c r="Q58" s="7"/>
       <c r="R58" s="7"/>
@@ -8943,7 +9619,7 @@
       <c r="AL58" s="7"/>
       <c r="AM58" s="7"/>
       <c r="AN58" s="7"/>
-      <c r="AO58" s="156"/>
+      <c r="AO58" s="107"/>
       <c r="AP58" s="7"/>
       <c r="AQ58" s="7"/>
       <c r="AR58" s="7"/>
@@ -9025,19 +9701,19 @@
       <c r="K60" s="3"/>
       <c r="L60" s="7"/>
       <c r="M60" s="7"/>
-      <c r="N60" s="102" t="s">
+      <c r="N60" s="138" t="s">
         <v>33</v>
       </c>
-      <c r="O60" s="102"/>
-      <c r="P60" s="102"/>
+      <c r="O60" s="138"/>
+      <c r="P60" s="138"/>
       <c r="Q60" s="7"/>
-      <c r="R60" s="102" t="s">
+      <c r="R60" s="138" t="s">
         <v>34</v>
       </c>
-      <c r="S60" s="102"/>
-      <c r="T60" s="102"/>
-      <c r="U60" s="102"/>
-      <c r="V60" s="102"/>
+      <c r="S60" s="138"/>
+      <c r="T60" s="138"/>
+      <c r="U60" s="138"/>
+      <c r="V60" s="138"/>
       <c r="W60" s="7"/>
       <c r="X60" s="7"/>
       <c r="AB60" s="7"/>
@@ -9082,15 +9758,15 @@
       <c r="K61" s="3"/>
       <c r="L61" s="7"/>
       <c r="M61" s="7"/>
-      <c r="N61" s="102"/>
-      <c r="O61" s="102"/>
-      <c r="P61" s="102"/>
+      <c r="N61" s="138"/>
+      <c r="O61" s="138"/>
+      <c r="P61" s="138"/>
       <c r="Q61" s="7"/>
-      <c r="R61" s="102"/>
-      <c r="S61" s="102"/>
-      <c r="T61" s="102"/>
-      <c r="U61" s="102"/>
-      <c r="V61" s="102"/>
+      <c r="R61" s="138"/>
+      <c r="S61" s="138"/>
+      <c r="T61" s="138"/>
+      <c r="U61" s="138"/>
+      <c r="V61" s="138"/>
       <c r="W61" s="7"/>
       <c r="X61" s="7"/>
       <c r="AB61" s="7"/>
@@ -9105,19 +9781,19 @@
       <c r="AK61" s="17"/>
       <c r="AL61" s="7"/>
       <c r="AM61" s="7"/>
-      <c r="AN61" s="150" t="s">
+      <c r="AN61" s="100" t="s">
         <v>37</v>
       </c>
-      <c r="AO61" s="151"/>
-      <c r="AP61" s="151"/>
-      <c r="AQ61" s="151"/>
-      <c r="AR61" s="151"/>
-      <c r="AS61" s="151"/>
-      <c r="AT61" s="151"/>
-      <c r="AU61" s="151"/>
-      <c r="AV61" s="151"/>
-      <c r="AW61" s="151"/>
-      <c r="AX61" s="152"/>
+      <c r="AO61" s="101"/>
+      <c r="AP61" s="101"/>
+      <c r="AQ61" s="101"/>
+      <c r="AR61" s="101"/>
+      <c r="AS61" s="101"/>
+      <c r="AT61" s="101"/>
+      <c r="AU61" s="101"/>
+      <c r="AV61" s="101"/>
+      <c r="AW61" s="101"/>
+      <c r="AX61" s="102"/>
       <c r="AY61" s="7"/>
       <c r="AZ61" s="7"/>
       <c r="BA61" s="7"/>
@@ -9141,13 +9817,13 @@
       <c r="O62" s="7"/>
       <c r="P62" s="7"/>
       <c r="Q62" s="7"/>
-      <c r="R62" s="81" t="s">
+      <c r="R62" s="147" t="s">
         <v>35</v>
       </c>
-      <c r="S62" s="81"/>
-      <c r="T62" s="81"/>
-      <c r="U62" s="81"/>
-      <c r="V62" s="81"/>
+      <c r="S62" s="147"/>
+      <c r="T62" s="147"/>
+      <c r="U62" s="147"/>
+      <c r="V62" s="147"/>
       <c r="W62" s="7"/>
       <c r="X62" s="7"/>
       <c r="AB62" s="7"/>
@@ -9162,17 +9838,17 @@
       <c r="AK62" s="17"/>
       <c r="AL62" s="7"/>
       <c r="AM62" s="7"/>
-      <c r="AN62" s="153"/>
-      <c r="AO62" s="154"/>
-      <c r="AP62" s="154"/>
-      <c r="AQ62" s="154"/>
-      <c r="AR62" s="154"/>
-      <c r="AS62" s="154"/>
-      <c r="AT62" s="154"/>
-      <c r="AU62" s="154"/>
-      <c r="AV62" s="154"/>
-      <c r="AW62" s="154"/>
-      <c r="AX62" s="155"/>
+      <c r="AN62" s="103"/>
+      <c r="AO62" s="104"/>
+      <c r="AP62" s="104"/>
+      <c r="AQ62" s="104"/>
+      <c r="AR62" s="104"/>
+      <c r="AS62" s="104"/>
+      <c r="AT62" s="104"/>
+      <c r="AU62" s="104"/>
+      <c r="AV62" s="104"/>
+      <c r="AW62" s="104"/>
+      <c r="AX62" s="105"/>
       <c r="AY62" s="7"/>
       <c r="AZ62" s="7"/>
       <c r="BA62" s="7"/>
@@ -9215,19 +9891,19 @@
       <c r="AK63" s="17"/>
       <c r="AL63" s="7"/>
       <c r="AM63" s="7"/>
-      <c r="AN63" s="141" t="s">
+      <c r="AN63" s="91" t="s">
         <v>49</v>
       </c>
-      <c r="AO63" s="142"/>
-      <c r="AP63" s="142"/>
-      <c r="AQ63" s="142"/>
-      <c r="AR63" s="142"/>
-      <c r="AS63" s="142"/>
-      <c r="AT63" s="142"/>
-      <c r="AU63" s="142"/>
-      <c r="AV63" s="142"/>
-      <c r="AW63" s="142"/>
-      <c r="AX63" s="143"/>
+      <c r="AO63" s="92"/>
+      <c r="AP63" s="92"/>
+      <c r="AQ63" s="92"/>
+      <c r="AR63" s="92"/>
+      <c r="AS63" s="92"/>
+      <c r="AT63" s="92"/>
+      <c r="AU63" s="92"/>
+      <c r="AV63" s="92"/>
+      <c r="AW63" s="92"/>
+      <c r="AX63" s="93"/>
       <c r="AY63" s="7"/>
       <c r="AZ63" s="7"/>
       <c r="BA63" s="7"/>
@@ -9290,17 +9966,17 @@
       </c>
       <c r="AL64" s="7"/>
       <c r="AM64" s="7"/>
-      <c r="AN64" s="141"/>
-      <c r="AO64" s="142"/>
-      <c r="AP64" s="142"/>
-      <c r="AQ64" s="142"/>
-      <c r="AR64" s="142"/>
-      <c r="AS64" s="142"/>
-      <c r="AT64" s="142"/>
-      <c r="AU64" s="142"/>
-      <c r="AV64" s="142"/>
-      <c r="AW64" s="142"/>
-      <c r="AX64" s="143"/>
+      <c r="AN64" s="91"/>
+      <c r="AO64" s="92"/>
+      <c r="AP64" s="92"/>
+      <c r="AQ64" s="92"/>
+      <c r="AR64" s="92"/>
+      <c r="AS64" s="92"/>
+      <c r="AT64" s="92"/>
+      <c r="AU64" s="92"/>
+      <c r="AV64" s="92"/>
+      <c r="AW64" s="92"/>
+      <c r="AX64" s="93"/>
       <c r="AY64" s="7"/>
       <c r="AZ64" s="7"/>
       <c r="BA64" s="7"/>
@@ -9363,19 +10039,19 @@
       </c>
       <c r="AL65" s="7"/>
       <c r="AM65" s="7"/>
-      <c r="AN65" s="144" t="s">
+      <c r="AN65" s="94" t="s">
         <v>38</v>
       </c>
-      <c r="AO65" s="145"/>
-      <c r="AP65" s="145"/>
-      <c r="AQ65" s="145"/>
-      <c r="AR65" s="145"/>
-      <c r="AS65" s="145"/>
-      <c r="AT65" s="145"/>
-      <c r="AU65" s="145"/>
-      <c r="AV65" s="145"/>
-      <c r="AW65" s="145"/>
-      <c r="AX65" s="146"/>
+      <c r="AO65" s="95"/>
+      <c r="AP65" s="95"/>
+      <c r="AQ65" s="95"/>
+      <c r="AR65" s="95"/>
+      <c r="AS65" s="95"/>
+      <c r="AT65" s="95"/>
+      <c r="AU65" s="95"/>
+      <c r="AV65" s="95"/>
+      <c r="AW65" s="95"/>
+      <c r="AX65" s="96"/>
       <c r="AY65" s="7"/>
       <c r="AZ65" s="7"/>
       <c r="BA65" s="7"/>
@@ -9438,17 +10114,17 @@
       </c>
       <c r="AL66" s="7"/>
       <c r="AM66" s="7"/>
-      <c r="AN66" s="147"/>
-      <c r="AO66" s="148"/>
-      <c r="AP66" s="148"/>
-      <c r="AQ66" s="148"/>
-      <c r="AR66" s="148"/>
-      <c r="AS66" s="148"/>
-      <c r="AT66" s="148"/>
-      <c r="AU66" s="148"/>
-      <c r="AV66" s="148"/>
-      <c r="AW66" s="148"/>
-      <c r="AX66" s="149"/>
+      <c r="AN66" s="97"/>
+      <c r="AO66" s="98"/>
+      <c r="AP66" s="98"/>
+      <c r="AQ66" s="98"/>
+      <c r="AR66" s="98"/>
+      <c r="AS66" s="98"/>
+      <c r="AT66" s="98"/>
+      <c r="AU66" s="98"/>
+      <c r="AV66" s="98"/>
+      <c r="AW66" s="98"/>
+      <c r="AX66" s="99"/>
       <c r="AY66" s="7"/>
       <c r="AZ66" s="7"/>
       <c r="BA66" s="7"/>
@@ -9491,19 +10167,19 @@
       <c r="AK67" s="17"/>
       <c r="AL67" s="7"/>
       <c r="AM67" s="7"/>
-      <c r="AN67" s="99" t="s">
+      <c r="AN67" s="145" t="s">
         <v>64</v>
       </c>
-      <c r="AO67" s="100"/>
-      <c r="AP67" s="100"/>
-      <c r="AQ67" s="100"/>
-      <c r="AR67" s="100"/>
-      <c r="AS67" s="100"/>
-      <c r="AT67" s="100"/>
-      <c r="AU67" s="100"/>
-      <c r="AV67" s="100"/>
-      <c r="AW67" s="100"/>
-      <c r="AX67" s="100"/>
+      <c r="AO67" s="146"/>
+      <c r="AP67" s="146"/>
+      <c r="AQ67" s="146"/>
+      <c r="AR67" s="146"/>
+      <c r="AS67" s="146"/>
+      <c r="AT67" s="146"/>
+      <c r="AU67" s="146"/>
+      <c r="AV67" s="146"/>
+      <c r="AW67" s="146"/>
+      <c r="AX67" s="146"/>
       <c r="AY67" s="7"/>
       <c r="AZ67" s="7"/>
       <c r="BA67" s="7"/>
@@ -9546,17 +10222,17 @@
       <c r="AK68" s="17"/>
       <c r="AL68" s="7"/>
       <c r="AM68" s="7"/>
-      <c r="AN68" s="81"/>
-      <c r="AO68" s="81"/>
-      <c r="AP68" s="81"/>
-      <c r="AQ68" s="81"/>
-      <c r="AR68" s="81"/>
-      <c r="AS68" s="81"/>
-      <c r="AT68" s="81"/>
-      <c r="AU68" s="81"/>
-      <c r="AV68" s="81"/>
-      <c r="AW68" s="81"/>
-      <c r="AX68" s="81"/>
+      <c r="AN68" s="147"/>
+      <c r="AO68" s="147"/>
+      <c r="AP68" s="147"/>
+      <c r="AQ68" s="147"/>
+      <c r="AR68" s="147"/>
+      <c r="AS68" s="147"/>
+      <c r="AT68" s="147"/>
+      <c r="AU68" s="147"/>
+      <c r="AV68" s="147"/>
+      <c r="AW68" s="147"/>
+      <c r="AX68" s="147"/>
       <c r="AY68" s="7"/>
       <c r="AZ68" s="7"/>
       <c r="BA68" s="7"/>
@@ -9928,34 +10604,34 @@
       <c r="BB76" s="7"/>
       <c r="BC76" s="7"/>
       <c r="BG76" s="7"/>
-      <c r="BH76" s="140" t="s">
+      <c r="BH76" s="89" t="s">
         <v>72</v>
       </c>
-      <c r="BI76" s="140"/>
-      <c r="BJ76" s="140"/>
-      <c r="BK76" s="140"/>
-      <c r="BL76" s="140"/>
-      <c r="BM76" s="140"/>
-      <c r="BN76" s="140"/>
-      <c r="BO76" s="140"/>
-      <c r="BP76" s="140"/>
-      <c r="BQ76" s="140"/>
-      <c r="BR76" s="140"/>
-      <c r="BS76" s="140"/>
-      <c r="BT76" s="140"/>
-      <c r="BU76" s="140"/>
-      <c r="BV76" s="140"/>
+      <c r="BI76" s="89"/>
+      <c r="BJ76" s="89"/>
+      <c r="BK76" s="89"/>
+      <c r="BL76" s="89"/>
+      <c r="BM76" s="89"/>
+      <c r="BN76" s="89"/>
+      <c r="BO76" s="89"/>
+      <c r="BP76" s="89"/>
+      <c r="BQ76" s="89"/>
+      <c r="BR76" s="89"/>
+      <c r="BS76" s="89"/>
+      <c r="BT76" s="89"/>
+      <c r="BU76" s="89"/>
+      <c r="BV76" s="89"/>
       <c r="BW76" s="10"/>
       <c r="BX76" s="80"/>
-      <c r="BY76" s="140" t="s">
+      <c r="BY76" s="89" t="s">
         <v>73</v>
       </c>
-      <c r="BZ76" s="140"/>
-      <c r="CA76" s="140"/>
-      <c r="CB76" s="140"/>
-      <c r="CC76" s="140"/>
-      <c r="CD76" s="140"/>
-      <c r="CE76" s="140"/>
+      <c r="BZ76" s="89"/>
+      <c r="CA76" s="89"/>
+      <c r="CB76" s="89"/>
+      <c r="CC76" s="89"/>
+      <c r="CD76" s="89"/>
+      <c r="CE76" s="89"/>
       <c r="CF76" s="80"/>
     </row>
     <row r="77" spans="2:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -9988,30 +10664,30 @@
       <c r="BB77" s="7"/>
       <c r="BC77" s="7"/>
       <c r="BG77" s="7"/>
-      <c r="BH77" s="140"/>
-      <c r="BI77" s="140"/>
-      <c r="BJ77" s="140"/>
-      <c r="BK77" s="140"/>
-      <c r="BL77" s="140"/>
-      <c r="BM77" s="140"/>
-      <c r="BN77" s="140"/>
-      <c r="BO77" s="140"/>
-      <c r="BP77" s="140"/>
-      <c r="BQ77" s="140"/>
-      <c r="BR77" s="140"/>
-      <c r="BS77" s="140"/>
-      <c r="BT77" s="140"/>
-      <c r="BU77" s="140"/>
-      <c r="BV77" s="140"/>
+      <c r="BH77" s="89"/>
+      <c r="BI77" s="89"/>
+      <c r="BJ77" s="89"/>
+      <c r="BK77" s="89"/>
+      <c r="BL77" s="89"/>
+      <c r="BM77" s="89"/>
+      <c r="BN77" s="89"/>
+      <c r="BO77" s="89"/>
+      <c r="BP77" s="89"/>
+      <c r="BQ77" s="89"/>
+      <c r="BR77" s="89"/>
+      <c r="BS77" s="89"/>
+      <c r="BT77" s="89"/>
+      <c r="BU77" s="89"/>
+      <c r="BV77" s="89"/>
       <c r="BW77" s="10"/>
       <c r="BX77" s="80"/>
-      <c r="BY77" s="140"/>
-      <c r="BZ77" s="140"/>
-      <c r="CA77" s="140"/>
-      <c r="CB77" s="140"/>
-      <c r="CC77" s="140"/>
-      <c r="CD77" s="140"/>
-      <c r="CE77" s="140"/>
+      <c r="BY77" s="89"/>
+      <c r="BZ77" s="89"/>
+      <c r="CA77" s="89"/>
+      <c r="CB77" s="89"/>
+      <c r="CC77" s="89"/>
+      <c r="CD77" s="89"/>
+      <c r="CE77" s="89"/>
       <c r="CF77" s="80"/>
     </row>
     <row r="78" spans="2:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -10027,30 +10703,30 @@
       <c r="BB78" s="7"/>
       <c r="BC78" s="7"/>
       <c r="BG78" s="7"/>
-      <c r="BH78" s="140"/>
-      <c r="BI78" s="140"/>
-      <c r="BJ78" s="140"/>
-      <c r="BK78" s="140"/>
-      <c r="BL78" s="140"/>
-      <c r="BM78" s="140"/>
-      <c r="BN78" s="140"/>
-      <c r="BO78" s="140"/>
-      <c r="BP78" s="140"/>
-      <c r="BQ78" s="140"/>
-      <c r="BR78" s="140"/>
-      <c r="BS78" s="140"/>
-      <c r="BT78" s="140"/>
-      <c r="BU78" s="140"/>
-      <c r="BV78" s="140"/>
+      <c r="BH78" s="89"/>
+      <c r="BI78" s="89"/>
+      <c r="BJ78" s="89"/>
+      <c r="BK78" s="89"/>
+      <c r="BL78" s="89"/>
+      <c r="BM78" s="89"/>
+      <c r="BN78" s="89"/>
+      <c r="BO78" s="89"/>
+      <c r="BP78" s="89"/>
+      <c r="BQ78" s="89"/>
+      <c r="BR78" s="89"/>
+      <c r="BS78" s="89"/>
+      <c r="BT78" s="89"/>
+      <c r="BU78" s="89"/>
+      <c r="BV78" s="89"/>
       <c r="BW78" s="10"/>
       <c r="BX78" s="80"/>
-      <c r="BY78" s="140"/>
-      <c r="BZ78" s="140"/>
-      <c r="CA78" s="140"/>
-      <c r="CB78" s="140"/>
-      <c r="CC78" s="140"/>
-      <c r="CD78" s="140"/>
-      <c r="CE78" s="140"/>
+      <c r="BY78" s="89"/>
+      <c r="BZ78" s="89"/>
+      <c r="CA78" s="89"/>
+      <c r="CB78" s="89"/>
+      <c r="CC78" s="89"/>
+      <c r="CD78" s="89"/>
+      <c r="CE78" s="89"/>
       <c r="CF78" s="80"/>
     </row>
     <row r="79" spans="2:84" x14ac:dyDescent="0.3">
@@ -10078,13 +10754,13 @@
       <c r="BV79" s="7"/>
       <c r="BW79" s="10"/>
       <c r="BX79" s="7"/>
-      <c r="BY79" s="140"/>
-      <c r="BZ79" s="140"/>
-      <c r="CA79" s="140"/>
-      <c r="CB79" s="140"/>
-      <c r="CC79" s="140"/>
-      <c r="CD79" s="140"/>
-      <c r="CE79" s="140"/>
+      <c r="BY79" s="89"/>
+      <c r="BZ79" s="89"/>
+      <c r="CA79" s="89"/>
+      <c r="CB79" s="89"/>
+      <c r="CC79" s="89"/>
+      <c r="CD79" s="89"/>
+      <c r="CE79" s="89"/>
       <c r="CF79" s="7"/>
     </row>
     <row r="80" spans="2:84" x14ac:dyDescent="0.3">
@@ -10170,7 +10846,7 @@
       <c r="BI82" s="6"/>
       <c r="BJ82" s="17"/>
       <c r="BK82" s="6"/>
-      <c r="BL82" s="92"/>
+      <c r="BL82" s="112"/>
       <c r="BM82" s="7"/>
       <c r="BN82" s="17"/>
       <c r="BO82" s="6"/>
@@ -10186,7 +10862,7 @@
       <c r="BY82" s="7"/>
       <c r="BZ82" s="7"/>
       <c r="CA82" s="69"/>
-      <c r="CB82" s="118"/>
+      <c r="CB82" s="113"/>
       <c r="CC82" s="7"/>
       <c r="CD82" s="7"/>
       <c r="CE82" s="7"/>
@@ -10199,7 +10875,7 @@
       <c r="BI83" s="6"/>
       <c r="BJ83" s="17"/>
       <c r="BK83" s="6"/>
-      <c r="BL83" s="92"/>
+      <c r="BL83" s="112"/>
       <c r="BM83" s="7"/>
       <c r="BN83" s="17"/>
       <c r="BO83" s="6"/>
@@ -10215,7 +10891,7 @@
       <c r="BY83" s="7"/>
       <c r="BZ83" s="7"/>
       <c r="CA83" s="69"/>
-      <c r="CB83" s="118"/>
+      <c r="CB83" s="113"/>
       <c r="CC83" s="7"/>
       <c r="CD83" s="7"/>
       <c r="CE83" s="7"/>
@@ -10301,10 +10977,10 @@
       <c r="BW86" s="10"/>
       <c r="BX86" s="17"/>
       <c r="BY86" s="7"/>
-      <c r="BZ86" s="121" t="s">
+      <c r="BZ86" s="115" t="s">
         <v>62</v>
       </c>
-      <c r="CA86" s="122"/>
+      <c r="CA86" s="116"/>
       <c r="CB86" s="32"/>
       <c r="CC86" s="7"/>
       <c r="CD86" s="7"/>
@@ -10332,8 +11008,8 @@
       <c r="BW87" s="10"/>
       <c r="BX87" s="17"/>
       <c r="BY87" s="7"/>
-      <c r="BZ87" s="121"/>
-      <c r="CA87" s="122"/>
+      <c r="BZ87" s="115"/>
+      <c r="CA87" s="116"/>
       <c r="CB87" s="32"/>
       <c r="CC87" s="7"/>
       <c r="CD87" s="7"/>
@@ -10364,10 +11040,10 @@
       <c r="BZ88" s="7"/>
       <c r="CA88" s="69"/>
       <c r="CB88" s="2"/>
-      <c r="CC88" s="123" t="s">
+      <c r="CC88" s="117" t="s">
         <v>63</v>
       </c>
-      <c r="CD88" s="124"/>
+      <c r="CD88" s="118"/>
       <c r="CE88" s="7"/>
       <c r="CF88" s="7"/>
     </row>
@@ -10395,8 +11071,8 @@
       <c r="BZ89" s="7"/>
       <c r="CA89" s="69"/>
       <c r="CB89" s="3"/>
-      <c r="CC89" s="125"/>
-      <c r="CD89" s="124"/>
+      <c r="CC89" s="119"/>
+      <c r="CD89" s="118"/>
       <c r="CE89" s="7"/>
       <c r="CF89" s="7"/>
       <c r="CJ89" t="s">
@@ -10638,23 +11314,23 @@
     <row r="98" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG98" s="7"/>
       <c r="BH98" s="39"/>
-      <c r="BI98" s="119" t="s">
+      <c r="BI98" s="114" t="s">
         <v>40</v>
       </c>
-      <c r="BJ98" s="119"/>
-      <c r="BK98" s="119"/>
-      <c r="BL98" s="119"/>
-      <c r="BM98" s="119"/>
-      <c r="BN98" s="119"/>
-      <c r="BO98" s="119"/>
-      <c r="BP98" s="119"/>
-      <c r="BQ98" s="119"/>
-      <c r="BR98" s="119"/>
-      <c r="BS98" s="119"/>
-      <c r="BT98" s="119"/>
-      <c r="BU98" s="119"/>
-      <c r="BV98" s="119"/>
-      <c r="BW98" s="119"/>
+      <c r="BJ98" s="114"/>
+      <c r="BK98" s="114"/>
+      <c r="BL98" s="114"/>
+      <c r="BM98" s="114"/>
+      <c r="BN98" s="114"/>
+      <c r="BO98" s="114"/>
+      <c r="BP98" s="114"/>
+      <c r="BQ98" s="114"/>
+      <c r="BR98" s="114"/>
+      <c r="BS98" s="114"/>
+      <c r="BT98" s="114"/>
+      <c r="BU98" s="114"/>
+      <c r="BV98" s="114"/>
+      <c r="BW98" s="114"/>
       <c r="BX98" s="40"/>
       <c r="BY98" s="7"/>
       <c r="BZ98" s="7"/>
@@ -10668,21 +11344,21 @@
     <row r="99" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG99" s="7"/>
       <c r="BH99" s="39"/>
-      <c r="BI99" s="119"/>
-      <c r="BJ99" s="119"/>
-      <c r="BK99" s="119"/>
-      <c r="BL99" s="119"/>
-      <c r="BM99" s="119"/>
-      <c r="BN99" s="119"/>
-      <c r="BO99" s="119"/>
-      <c r="BP99" s="119"/>
-      <c r="BQ99" s="119"/>
-      <c r="BR99" s="119"/>
-      <c r="BS99" s="119"/>
-      <c r="BT99" s="119"/>
-      <c r="BU99" s="119"/>
-      <c r="BV99" s="119"/>
-      <c r="BW99" s="119"/>
+      <c r="BI99" s="114"/>
+      <c r="BJ99" s="114"/>
+      <c r="BK99" s="114"/>
+      <c r="BL99" s="114"/>
+      <c r="BM99" s="114"/>
+      <c r="BN99" s="114"/>
+      <c r="BO99" s="114"/>
+      <c r="BP99" s="114"/>
+      <c r="BQ99" s="114"/>
+      <c r="BR99" s="114"/>
+      <c r="BS99" s="114"/>
+      <c r="BT99" s="114"/>
+      <c r="BU99" s="114"/>
+      <c r="BV99" s="114"/>
+      <c r="BW99" s="114"/>
       <c r="BX99" s="40"/>
       <c r="BY99" s="7"/>
       <c r="BZ99" s="7"/>
@@ -10696,21 +11372,21 @@
     <row r="100" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG100" s="7"/>
       <c r="BH100" s="39"/>
-      <c r="BI100" s="119"/>
-      <c r="BJ100" s="119"/>
-      <c r="BK100" s="119"/>
-      <c r="BL100" s="119"/>
-      <c r="BM100" s="119"/>
-      <c r="BN100" s="119"/>
-      <c r="BO100" s="119"/>
-      <c r="BP100" s="119"/>
-      <c r="BQ100" s="119"/>
-      <c r="BR100" s="119"/>
-      <c r="BS100" s="119"/>
-      <c r="BT100" s="119"/>
-      <c r="BU100" s="119"/>
-      <c r="BV100" s="119"/>
-      <c r="BW100" s="119"/>
+      <c r="BI100" s="114"/>
+      <c r="BJ100" s="114"/>
+      <c r="BK100" s="114"/>
+      <c r="BL100" s="114"/>
+      <c r="BM100" s="114"/>
+      <c r="BN100" s="114"/>
+      <c r="BO100" s="114"/>
+      <c r="BP100" s="114"/>
+      <c r="BQ100" s="114"/>
+      <c r="BR100" s="114"/>
+      <c r="BS100" s="114"/>
+      <c r="BT100" s="114"/>
+      <c r="BU100" s="114"/>
+      <c r="BV100" s="114"/>
+      <c r="BW100" s="114"/>
       <c r="BX100" s="40"/>
       <c r="BY100" s="7"/>
       <c r="BZ100" s="7"/>
@@ -10724,21 +11400,21 @@
     <row r="101" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG101" s="7"/>
       <c r="BH101" s="39"/>
-      <c r="BI101" s="119"/>
-      <c r="BJ101" s="119"/>
-      <c r="BK101" s="119"/>
-      <c r="BL101" s="119"/>
-      <c r="BM101" s="119"/>
-      <c r="BN101" s="119"/>
-      <c r="BO101" s="119"/>
-      <c r="BP101" s="119"/>
-      <c r="BQ101" s="119"/>
-      <c r="BR101" s="119"/>
-      <c r="BS101" s="119"/>
-      <c r="BT101" s="119"/>
-      <c r="BU101" s="119"/>
-      <c r="BV101" s="119"/>
-      <c r="BW101" s="119"/>
+      <c r="BI101" s="114"/>
+      <c r="BJ101" s="114"/>
+      <c r="BK101" s="114"/>
+      <c r="BL101" s="114"/>
+      <c r="BM101" s="114"/>
+      <c r="BN101" s="114"/>
+      <c r="BO101" s="114"/>
+      <c r="BP101" s="114"/>
+      <c r="BQ101" s="114"/>
+      <c r="BR101" s="114"/>
+      <c r="BS101" s="114"/>
+      <c r="BT101" s="114"/>
+      <c r="BU101" s="114"/>
+      <c r="BV101" s="114"/>
+      <c r="BW101" s="114"/>
       <c r="BX101" s="40"/>
       <c r="BY101" s="7"/>
       <c r="BZ101" s="7"/>
@@ -10752,21 +11428,21 @@
     <row r="102" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG102" s="7"/>
       <c r="BH102" s="39"/>
-      <c r="BI102" s="119"/>
-      <c r="BJ102" s="119"/>
-      <c r="BK102" s="119"/>
-      <c r="BL102" s="119"/>
-      <c r="BM102" s="119"/>
-      <c r="BN102" s="119"/>
-      <c r="BO102" s="119"/>
-      <c r="BP102" s="119"/>
-      <c r="BQ102" s="119"/>
-      <c r="BR102" s="119"/>
-      <c r="BS102" s="119"/>
-      <c r="BT102" s="119"/>
-      <c r="BU102" s="119"/>
-      <c r="BV102" s="119"/>
-      <c r="BW102" s="119"/>
+      <c r="BI102" s="114"/>
+      <c r="BJ102" s="114"/>
+      <c r="BK102" s="114"/>
+      <c r="BL102" s="114"/>
+      <c r="BM102" s="114"/>
+      <c r="BN102" s="114"/>
+      <c r="BO102" s="114"/>
+      <c r="BP102" s="114"/>
+      <c r="BQ102" s="114"/>
+      <c r="BR102" s="114"/>
+      <c r="BS102" s="114"/>
+      <c r="BT102" s="114"/>
+      <c r="BU102" s="114"/>
+      <c r="BV102" s="114"/>
+      <c r="BW102" s="114"/>
       <c r="BX102" s="40"/>
       <c r="BY102" s="7"/>
       <c r="BZ102" s="7"/>
@@ -11011,15 +11687,15 @@
       <c r="BM111" s="45"/>
       <c r="BN111" s="45"/>
       <c r="BO111" s="45"/>
-      <c r="BP111" s="139" t="s">
+      <c r="BP111" s="133" t="s">
         <v>41</v>
       </c>
-      <c r="BQ111" s="139"/>
-      <c r="BR111" s="139"/>
-      <c r="BS111" s="139"/>
-      <c r="BT111" s="139"/>
-      <c r="BU111" s="139"/>
-      <c r="BV111" s="139"/>
+      <c r="BQ111" s="133"/>
+      <c r="BR111" s="133"/>
+      <c r="BS111" s="133"/>
+      <c r="BT111" s="133"/>
+      <c r="BU111" s="133"/>
+      <c r="BV111" s="133"/>
       <c r="BW111" s="56"/>
       <c r="BX111" s="11"/>
       <c r="BY111" s="45"/>
@@ -11041,13 +11717,13 @@
       <c r="BM112" s="45"/>
       <c r="BN112" s="45"/>
       <c r="BO112" s="45"/>
-      <c r="BP112" s="139"/>
-      <c r="BQ112" s="139"/>
-      <c r="BR112" s="139"/>
-      <c r="BS112" s="139"/>
-      <c r="BT112" s="139"/>
-      <c r="BU112" s="139"/>
-      <c r="BV112" s="139"/>
+      <c r="BP112" s="133"/>
+      <c r="BQ112" s="133"/>
+      <c r="BR112" s="133"/>
+      <c r="BS112" s="133"/>
+      <c r="BT112" s="133"/>
+      <c r="BU112" s="133"/>
+      <c r="BV112" s="133"/>
       <c r="BW112" s="56"/>
       <c r="BX112" s="11"/>
       <c r="BY112" s="45"/>
@@ -11069,13 +11745,13 @@
       <c r="BM113" s="45"/>
       <c r="BN113" s="45"/>
       <c r="BO113" s="45"/>
-      <c r="BP113" s="139"/>
-      <c r="BQ113" s="139"/>
-      <c r="BR113" s="139"/>
-      <c r="BS113" s="139"/>
-      <c r="BT113" s="139"/>
-      <c r="BU113" s="139"/>
-      <c r="BV113" s="139"/>
+      <c r="BP113" s="133"/>
+      <c r="BQ113" s="133"/>
+      <c r="BR113" s="133"/>
+      <c r="BS113" s="133"/>
+      <c r="BT113" s="133"/>
+      <c r="BU113" s="133"/>
+      <c r="BV113" s="133"/>
       <c r="BW113" s="56"/>
       <c r="BX113" s="11"/>
       <c r="BY113" s="45"/>
@@ -11097,13 +11773,13 @@
       <c r="BM114" s="45"/>
       <c r="BN114" s="45"/>
       <c r="BO114" s="45"/>
-      <c r="BP114" s="139"/>
-      <c r="BQ114" s="139"/>
-      <c r="BR114" s="139"/>
-      <c r="BS114" s="139"/>
-      <c r="BT114" s="139"/>
-      <c r="BU114" s="139"/>
-      <c r="BV114" s="139"/>
+      <c r="BP114" s="133"/>
+      <c r="BQ114" s="133"/>
+      <c r="BR114" s="133"/>
+      <c r="BS114" s="133"/>
+      <c r="BT114" s="133"/>
+      <c r="BU114" s="133"/>
+      <c r="BV114" s="133"/>
       <c r="BW114" s="56"/>
       <c r="BX114" s="11"/>
       <c r="BY114" s="45"/>
@@ -11125,13 +11801,13 @@
       <c r="BM115" s="45"/>
       <c r="BN115" s="45"/>
       <c r="BO115" s="45"/>
-      <c r="BP115" s="139"/>
-      <c r="BQ115" s="139"/>
-      <c r="BR115" s="139"/>
-      <c r="BS115" s="139"/>
-      <c r="BT115" s="139"/>
-      <c r="BU115" s="139"/>
-      <c r="BV115" s="139"/>
+      <c r="BP115" s="133"/>
+      <c r="BQ115" s="133"/>
+      <c r="BR115" s="133"/>
+      <c r="BS115" s="133"/>
+      <c r="BT115" s="133"/>
+      <c r="BU115" s="133"/>
+      <c r="BV115" s="133"/>
       <c r="BW115" s="56"/>
       <c r="BX115" s="11"/>
       <c r="BY115" s="45"/>
@@ -11341,15 +12017,15 @@
     </row>
     <row r="123" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG123" s="7"/>
-      <c r="BH123" s="120" t="s">
+      <c r="BH123" s="90" t="s">
         <v>43</v>
       </c>
       <c r="BI123" s="6"/>
-      <c r="BJ123" s="120" t="s">
+      <c r="BJ123" s="90" t="s">
         <v>44</v>
       </c>
       <c r="BK123" s="6"/>
-      <c r="BL123" s="120" t="s">
+      <c r="BL123" s="90" t="s">
         <v>51</v>
       </c>
       <c r="BM123" s="7"/>
@@ -11359,15 +12035,15 @@
       <c r="BQ123" s="6"/>
       <c r="BR123" s="17"/>
       <c r="BS123" s="6"/>
-      <c r="BT123" s="120" t="s">
+      <c r="BT123" s="90" t="s">
         <v>45</v>
       </c>
       <c r="BU123" s="6"/>
-      <c r="BV123" s="120" t="s">
+      <c r="BV123" s="90" t="s">
         <v>46</v>
       </c>
       <c r="BW123" s="10"/>
-      <c r="BX123" s="120" t="s">
+      <c r="BX123" s="90" t="s">
         <v>50</v>
       </c>
       <c r="BY123" s="7"/>
@@ -11381,11 +12057,11 @@
     </row>
     <row r="124" spans="59:84" ht="25.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="BG124" s="7"/>
-      <c r="BH124" s="120"/>
+      <c r="BH124" s="90"/>
       <c r="BI124" s="6"/>
-      <c r="BJ124" s="120"/>
+      <c r="BJ124" s="90"/>
       <c r="BK124" s="6"/>
-      <c r="BL124" s="120"/>
+      <c r="BL124" s="90"/>
       <c r="BM124" s="34"/>
       <c r="BN124" s="17"/>
       <c r="BP124" s="79" t="s">
@@ -11394,11 +12070,11 @@
       <c r="BQ124" s="6"/>
       <c r="BR124" s="17"/>
       <c r="BS124" s="6"/>
-      <c r="BT124" s="120"/>
+      <c r="BT124" s="90"/>
       <c r="BU124" s="6"/>
-      <c r="BV124" s="120"/>
+      <c r="BV124" s="90"/>
       <c r="BW124" s="10"/>
-      <c r="BX124" s="120"/>
+      <c r="BX124" s="90"/>
       <c r="BY124" s="7"/>
       <c r="BZ124" s="7"/>
       <c r="CA124" s="69"/>
@@ -11410,11 +12086,11 @@
     </row>
     <row r="125" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG125" s="7"/>
-      <c r="BH125" s="120"/>
+      <c r="BH125" s="90"/>
       <c r="BI125" s="6"/>
-      <c r="BJ125" s="120"/>
+      <c r="BJ125" s="90"/>
       <c r="BK125" s="6"/>
-      <c r="BL125" s="120"/>
+      <c r="BL125" s="90"/>
       <c r="BM125" s="7"/>
       <c r="BN125" s="17"/>
       <c r="BO125" s="6"/>
@@ -11422,11 +12098,11 @@
       <c r="BQ125" s="6"/>
       <c r="BR125" s="17"/>
       <c r="BS125" s="6"/>
-      <c r="BT125" s="120"/>
+      <c r="BT125" s="90"/>
       <c r="BU125" s="6"/>
-      <c r="BV125" s="120"/>
+      <c r="BV125" s="90"/>
       <c r="BW125" s="10"/>
-      <c r="BX125" s="120"/>
+      <c r="BX125" s="90"/>
       <c r="BY125" s="7"/>
       <c r="BZ125" s="7"/>
       <c r="CA125" s="69"/>
@@ -11595,11 +12271,11 @@
       <c r="BV131" s="7"/>
       <c r="BW131" s="10"/>
       <c r="BX131" s="7"/>
-      <c r="BY131" s="130" t="s">
+      <c r="BY131" s="124" t="s">
         <v>52</v>
       </c>
-      <c r="BZ131" s="131"/>
-      <c r="CA131" s="132"/>
+      <c r="BZ131" s="125"/>
+      <c r="CA131" s="126"/>
       <c r="CB131" s="69"/>
       <c r="CC131" s="60"/>
       <c r="CD131" s="61"/>
@@ -11614,28 +12290,28 @@
       <c r="BK132" s="7"/>
       <c r="BL132" s="7"/>
       <c r="BM132" s="7"/>
-      <c r="BN132" s="126" t="s">
+      <c r="BN132" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="BO132" s="127"/>
-      <c r="BP132" s="127"/>
-      <c r="BQ132" s="127"/>
-      <c r="BR132" s="128"/>
+      <c r="BO132" s="121"/>
+      <c r="BP132" s="121"/>
+      <c r="BQ132" s="121"/>
+      <c r="BR132" s="122"/>
       <c r="BS132" s="7"/>
       <c r="BT132" s="7"/>
       <c r="BU132" s="7"/>
       <c r="BV132" s="7"/>
       <c r="BW132" s="10"/>
       <c r="BX132" s="7"/>
-      <c r="BY132" s="133"/>
-      <c r="BZ132" s="134"/>
-      <c r="CA132" s="135"/>
+      <c r="BY132" s="127"/>
+      <c r="BZ132" s="128"/>
+      <c r="CA132" s="129"/>
       <c r="CB132" s="69"/>
-      <c r="CC132" s="115" t="s">
+      <c r="CC132" s="109" t="s">
         <v>47</v>
       </c>
-      <c r="CD132" s="116"/>
-      <c r="CE132" s="117"/>
+      <c r="CD132" s="110"/>
+      <c r="CE132" s="111"/>
       <c r="CF132" s="7"/>
     </row>
     <row r="133" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -11646,24 +12322,24 @@
       <c r="BK133" s="7"/>
       <c r="BL133" s="7"/>
       <c r="BM133" s="7"/>
-      <c r="BN133" s="129"/>
-      <c r="BO133" s="127"/>
-      <c r="BP133" s="127"/>
-      <c r="BQ133" s="127"/>
-      <c r="BR133" s="128"/>
+      <c r="BN133" s="123"/>
+      <c r="BO133" s="121"/>
+      <c r="BP133" s="121"/>
+      <c r="BQ133" s="121"/>
+      <c r="BR133" s="122"/>
       <c r="BS133" s="7"/>
       <c r="BT133" s="7"/>
       <c r="BU133" s="7"/>
       <c r="BV133" s="7"/>
       <c r="BW133" s="10"/>
       <c r="BX133" s="7"/>
-      <c r="BY133" s="133"/>
-      <c r="BZ133" s="134"/>
-      <c r="CA133" s="135"/>
+      <c r="BY133" s="127"/>
+      <c r="BZ133" s="128"/>
+      <c r="CA133" s="129"/>
       <c r="CB133" s="69"/>
-      <c r="CC133" s="115"/>
-      <c r="CD133" s="116"/>
-      <c r="CE133" s="117"/>
+      <c r="CC133" s="109"/>
+      <c r="CD133" s="110"/>
+      <c r="CE133" s="111"/>
       <c r="CF133" s="7"/>
     </row>
     <row r="134" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -11674,24 +12350,24 @@
       <c r="BK134" s="7"/>
       <c r="BL134" s="7"/>
       <c r="BM134" s="7"/>
-      <c r="BN134" s="129"/>
-      <c r="BO134" s="127"/>
-      <c r="BP134" s="127"/>
-      <c r="BQ134" s="127"/>
-      <c r="BR134" s="128"/>
+      <c r="BN134" s="123"/>
+      <c r="BO134" s="121"/>
+      <c r="BP134" s="121"/>
+      <c r="BQ134" s="121"/>
+      <c r="BR134" s="122"/>
       <c r="BS134" s="7"/>
       <c r="BT134" s="7"/>
       <c r="BU134" s="7"/>
       <c r="BV134" s="7"/>
       <c r="BW134" s="10"/>
       <c r="BX134" s="7"/>
-      <c r="BY134" s="133"/>
-      <c r="BZ134" s="134"/>
-      <c r="CA134" s="135"/>
+      <c r="BY134" s="127"/>
+      <c r="BZ134" s="128"/>
+      <c r="CA134" s="129"/>
       <c r="CB134" s="69"/>
-      <c r="CC134" s="115"/>
-      <c r="CD134" s="116"/>
-      <c r="CE134" s="117"/>
+      <c r="CC134" s="109"/>
+      <c r="CD134" s="110"/>
+      <c r="CE134" s="111"/>
       <c r="CF134" s="7"/>
     </row>
     <row r="135" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -11702,24 +12378,24 @@
       <c r="BK135" s="7"/>
       <c r="BL135" s="7"/>
       <c r="BM135" s="7"/>
-      <c r="BN135" s="129"/>
-      <c r="BO135" s="127"/>
-      <c r="BP135" s="127"/>
-      <c r="BQ135" s="127"/>
-      <c r="BR135" s="128"/>
+      <c r="BN135" s="123"/>
+      <c r="BO135" s="121"/>
+      <c r="BP135" s="121"/>
+      <c r="BQ135" s="121"/>
+      <c r="BR135" s="122"/>
       <c r="BS135" s="7"/>
       <c r="BT135" s="7"/>
       <c r="BU135" s="7"/>
       <c r="BV135" s="7"/>
       <c r="BW135" s="10"/>
       <c r="BX135" s="7"/>
-      <c r="BY135" s="133"/>
-      <c r="BZ135" s="134"/>
-      <c r="CA135" s="135"/>
+      <c r="BY135" s="127"/>
+      <c r="BZ135" s="128"/>
+      <c r="CA135" s="129"/>
       <c r="CB135" s="69"/>
-      <c r="CC135" s="115"/>
-      <c r="CD135" s="116"/>
-      <c r="CE135" s="117"/>
+      <c r="CC135" s="109"/>
+      <c r="CD135" s="110"/>
+      <c r="CE135" s="111"/>
       <c r="CF135" s="7"/>
     </row>
     <row r="136" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -11730,24 +12406,24 @@
       <c r="BK136" s="7"/>
       <c r="BL136" s="7"/>
       <c r="BM136" s="7"/>
-      <c r="BN136" s="129"/>
-      <c r="BO136" s="127"/>
-      <c r="BP136" s="127"/>
-      <c r="BQ136" s="127"/>
-      <c r="BR136" s="128"/>
+      <c r="BN136" s="123"/>
+      <c r="BO136" s="121"/>
+      <c r="BP136" s="121"/>
+      <c r="BQ136" s="121"/>
+      <c r="BR136" s="122"/>
       <c r="BS136" s="7"/>
       <c r="BT136" s="7"/>
       <c r="BU136" s="7"/>
       <c r="BV136" s="7"/>
       <c r="BW136" s="10"/>
       <c r="BX136" s="7"/>
-      <c r="BY136" s="133"/>
-      <c r="BZ136" s="134"/>
-      <c r="CA136" s="135"/>
+      <c r="BY136" s="127"/>
+      <c r="BZ136" s="128"/>
+      <c r="CA136" s="129"/>
       <c r="CB136" s="69"/>
-      <c r="CC136" s="115"/>
-      <c r="CD136" s="116"/>
-      <c r="CE136" s="117"/>
+      <c r="CC136" s="109"/>
+      <c r="CD136" s="110"/>
+      <c r="CE136" s="111"/>
       <c r="CF136" s="7"/>
     </row>
     <row r="137" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -11769,9 +12445,9 @@
       <c r="BV137" s="7"/>
       <c r="BW137" s="10"/>
       <c r="BX137" s="7"/>
-      <c r="BY137" s="136"/>
-      <c r="BZ137" s="137"/>
-      <c r="CA137" s="138"/>
+      <c r="BY137" s="130"/>
+      <c r="BZ137" s="131"/>
+      <c r="CA137" s="132"/>
       <c r="CB137" s="69"/>
       <c r="CC137" s="63"/>
       <c r="CD137" s="64"/>
@@ -11945,16 +12621,51 @@
     </row>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="CR32:CX33"/>
-    <mergeCell ref="DD10:DD24"/>
-    <mergeCell ref="DF26:DK27"/>
-    <mergeCell ref="CQ17:CQ30"/>
-    <mergeCell ref="BY76:CE79"/>
-    <mergeCell ref="BH123:BH125"/>
-    <mergeCell ref="AN63:AX64"/>
-    <mergeCell ref="AN65:AX66"/>
-    <mergeCell ref="AN61:AX62"/>
-    <mergeCell ref="AO57:AO58"/>
+    <mergeCell ref="R62:V62"/>
+    <mergeCell ref="U44:X45"/>
+    <mergeCell ref="U49:X51"/>
+    <mergeCell ref="U52:X54"/>
+    <mergeCell ref="U37:V40"/>
+    <mergeCell ref="U46:W46"/>
+    <mergeCell ref="T40:T49"/>
+    <mergeCell ref="E34:I35"/>
+    <mergeCell ref="N33:P34"/>
+    <mergeCell ref="T38:T39"/>
+    <mergeCell ref="S34:U34"/>
+    <mergeCell ref="AP45:AT46"/>
+    <mergeCell ref="AE34:AI35"/>
+    <mergeCell ref="O45:O46"/>
+    <mergeCell ref="O41:O42"/>
+    <mergeCell ref="O43:O44"/>
+    <mergeCell ref="AS34:AU34"/>
+    <mergeCell ref="AP48:AR49"/>
+    <mergeCell ref="AO49:AO50"/>
+    <mergeCell ref="AM33:AQ34"/>
+    <mergeCell ref="AN67:AX68"/>
+    <mergeCell ref="AP56:AT57"/>
+    <mergeCell ref="AP52:AU53"/>
+    <mergeCell ref="AU37:AV40"/>
+    <mergeCell ref="AT38:AT39"/>
+    <mergeCell ref="AO41:AO42"/>
+    <mergeCell ref="AO43:AO44"/>
+    <mergeCell ref="AU44:AX45"/>
+    <mergeCell ref="AO45:AO46"/>
+    <mergeCell ref="AU46:AW46"/>
+    <mergeCell ref="AO47:AO48"/>
+    <mergeCell ref="AO51:AO52"/>
+    <mergeCell ref="AO53:AO54"/>
+    <mergeCell ref="N60:P61"/>
+    <mergeCell ref="R60:V61"/>
+    <mergeCell ref="O55:O56"/>
+    <mergeCell ref="O57:O58"/>
+    <mergeCell ref="T51:T55"/>
+    <mergeCell ref="O51:O52"/>
+    <mergeCell ref="O53:O54"/>
+    <mergeCell ref="O47:O48"/>
+    <mergeCell ref="O49:O50"/>
+    <mergeCell ref="P48:R49"/>
+    <mergeCell ref="AC39:AC40"/>
+    <mergeCell ref="AK39:AK40"/>
     <mergeCell ref="AO55:AO56"/>
     <mergeCell ref="CC132:CE136"/>
     <mergeCell ref="BL82:BL83"/>
@@ -11971,51 +12682,16 @@
     <mergeCell ref="BY131:CA137"/>
     <mergeCell ref="BP111:BV115"/>
     <mergeCell ref="BH76:BV78"/>
-    <mergeCell ref="O47:O48"/>
-    <mergeCell ref="O49:O50"/>
-    <mergeCell ref="P48:R49"/>
-    <mergeCell ref="AC39:AC40"/>
-    <mergeCell ref="AK39:AK40"/>
-    <mergeCell ref="N60:P61"/>
-    <mergeCell ref="R60:V61"/>
-    <mergeCell ref="O55:O56"/>
-    <mergeCell ref="O57:O58"/>
-    <mergeCell ref="T51:T55"/>
-    <mergeCell ref="O51:O52"/>
-    <mergeCell ref="O53:O54"/>
-    <mergeCell ref="AP48:AR49"/>
-    <mergeCell ref="AO49:AO50"/>
-    <mergeCell ref="AM33:AQ34"/>
-    <mergeCell ref="AN67:AX68"/>
-    <mergeCell ref="AP56:AT57"/>
-    <mergeCell ref="AP52:AU53"/>
-    <mergeCell ref="AU37:AV40"/>
-    <mergeCell ref="AT38:AT39"/>
-    <mergeCell ref="AO41:AO42"/>
-    <mergeCell ref="AO43:AO44"/>
-    <mergeCell ref="AU44:AX45"/>
-    <mergeCell ref="AO45:AO46"/>
-    <mergeCell ref="AU46:AW46"/>
-    <mergeCell ref="AO47:AO48"/>
-    <mergeCell ref="AO51:AO52"/>
-    <mergeCell ref="AO53:AO54"/>
-    <mergeCell ref="E34:I35"/>
-    <mergeCell ref="N33:P34"/>
-    <mergeCell ref="T38:T39"/>
-    <mergeCell ref="S34:U34"/>
-    <mergeCell ref="AP45:AT46"/>
-    <mergeCell ref="AE34:AI35"/>
-    <mergeCell ref="O45:O46"/>
-    <mergeCell ref="O41:O42"/>
-    <mergeCell ref="O43:O44"/>
-    <mergeCell ref="AS34:AU34"/>
-    <mergeCell ref="R62:V62"/>
-    <mergeCell ref="U44:X45"/>
-    <mergeCell ref="U49:X51"/>
-    <mergeCell ref="U52:X54"/>
-    <mergeCell ref="U37:V40"/>
-    <mergeCell ref="U46:W46"/>
-    <mergeCell ref="T40:T49"/>
+    <mergeCell ref="BH123:BH125"/>
+    <mergeCell ref="AN63:AX64"/>
+    <mergeCell ref="AN65:AX66"/>
+    <mergeCell ref="AN61:AX62"/>
+    <mergeCell ref="AO57:AO58"/>
+    <mergeCell ref="CR32:CX33"/>
+    <mergeCell ref="DD10:DD24"/>
+    <mergeCell ref="DF26:DK27"/>
+    <mergeCell ref="CQ17:CQ30"/>
+    <mergeCell ref="BY76:CE79"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
thats enough of this :)
</commit_message>
<xml_diff>
--- a/report-vis.xlsx
+++ b/report-vis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\! CS\Y2\AI is taking over\cw\ai-garbage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D96942-2F04-4413-99B8-843452D433D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D671CB22-4633-4DCE-818E-3D99FFDF49A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-12645" windowWidth="29040" windowHeight="15840" xr2:uid="{82DBE9BC-AC51-4988-B415-6B972F3134D5}"/>
   </bookViews>
@@ -167,18 +167,6 @@
     <t>Fit Subject-Specific Classifiers</t>
   </si>
   <si>
-    <t>W1</t>
-  </si>
-  <si>
-    <t>W2</t>
-  </si>
-  <si>
-    <t>W7</t>
-  </si>
-  <si>
-    <t>W8</t>
-  </si>
-  <si>
     <t>Test Final Model</t>
   </si>
   <si>
@@ -186,12 +174,6 @@
   </si>
   <si>
     <t>FINE TUNING is performed using the FINE TUNING SAMPLES from the TEST SUBJECT</t>
-  </si>
-  <si>
-    <t>W9</t>
-  </si>
-  <si>
-    <t>W3</t>
   </si>
   <si>
     <t>Fine-Tuning:
@@ -253,36 +235,6 @@
     <t>ST</t>
   </si>
   <si>
-    <r>
-      <t>Initialise Generalised Classifier
-with</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="18"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> W</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>general</t>
-    </r>
-  </si>
-  <si>
     <t>TRAINING (SOURCE) SUBJECTS</t>
   </si>
   <si>
@@ -337,12 +289,48 @@
       <t xml:space="preserve">α </t>
     </r>
   </si>
+  <si>
+    <t>M1</t>
+  </si>
+  <si>
+    <t>M2</t>
+  </si>
+  <si>
+    <t>M3</t>
+  </si>
+  <si>
+    <t>M7</t>
+  </si>
+  <si>
+    <t>M8</t>
+  </si>
+  <si>
+    <t>M9</t>
+  </si>
+  <si>
+    <r>
+      <t>Initialise Generalised Classifier
+M</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>general</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -443,15 +431,6 @@
       <b/>
       <u/>
       <sz val="26"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="18"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -1146,67 +1125,103 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1221,13 +1236,13 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1287,98 +1302,62 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7390,13 +7369,13 @@
     </row>
     <row r="10" spans="90:116" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="CL10" s="81" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="CM10" s="82" t="s">
-        <v>75</v>
-      </c>
-      <c r="DD10" s="88" t="s">
-        <v>76</v>
+        <v>68</v>
+      </c>
+      <c r="DD10" s="164" t="s">
+        <v>69</v>
       </c>
       <c r="DE10" s="7"/>
       <c r="DF10" s="7"/>
@@ -7415,12 +7394,12 @@
         <v>0.314</v>
       </c>
       <c r="DA11" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="DB11" t="s">
-        <v>79</v>
-      </c>
-      <c r="DD11" s="88"/>
+        <v>72</v>
+      </c>
+      <c r="DD11" s="164"/>
       <c r="DE11" s="7"/>
       <c r="DF11" s="7"/>
       <c r="DG11" s="7"/>
@@ -7443,7 +7422,7 @@
       <c r="DB12">
         <v>0.90300000000000002</v>
       </c>
-      <c r="DD12" s="88"/>
+      <c r="DD12" s="164"/>
       <c r="DE12" s="7"/>
       <c r="DF12" s="7"/>
       <c r="DG12" s="7"/>
@@ -7466,7 +7445,7 @@
       <c r="DB13">
         <v>0.90500000000000003</v>
       </c>
-      <c r="DD13" s="88"/>
+      <c r="DD13" s="164"/>
       <c r="DE13" s="7"/>
       <c r="DF13" s="7"/>
       <c r="DG13" s="7"/>
@@ -7489,7 +7468,7 @@
       <c r="DB14">
         <v>0.90600000000000003</v>
       </c>
-      <c r="DD14" s="88"/>
+      <c r="DD14" s="164"/>
       <c r="DE14" s="7"/>
       <c r="DF14" s="7"/>
       <c r="DG14" s="7"/>
@@ -7524,7 +7503,7 @@
       <c r="DB15">
         <v>0.90900000000000003</v>
       </c>
-      <c r="DD15" s="88"/>
+      <c r="DD15" s="164"/>
       <c r="DE15" s="7"/>
       <c r="DF15" s="7"/>
       <c r="DG15" s="7"/>
@@ -7556,7 +7535,7 @@
       <c r="DB16">
         <v>0.91</v>
       </c>
-      <c r="DD16" s="88"/>
+      <c r="DD16" s="164"/>
       <c r="DE16" s="7"/>
       <c r="DF16" s="7"/>
       <c r="DG16" s="7"/>
@@ -7573,8 +7552,8 @@
       <c r="CM17" s="86">
         <v>0.87</v>
       </c>
-      <c r="CQ17" s="88" t="s">
-        <v>76</v>
+      <c r="CQ17" s="164" t="s">
+        <v>69</v>
       </c>
       <c r="CR17" s="7"/>
       <c r="CS17" s="7"/>
@@ -7590,7 +7569,7 @@
       <c r="DB17">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD17" s="88"/>
+      <c r="DD17" s="164"/>
       <c r="DE17" s="7"/>
       <c r="DF17" s="7"/>
       <c r="DG17" s="7"/>
@@ -7607,7 +7586,7 @@
       <c r="CM18" s="85">
         <v>0.88800000000000001</v>
       </c>
-      <c r="CQ18" s="88"/>
+      <c r="CQ18" s="164"/>
       <c r="CR18" s="7"/>
       <c r="CS18" s="7"/>
       <c r="CT18" s="7"/>
@@ -7622,7 +7601,7 @@
       <c r="DB18">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD18" s="88"/>
+      <c r="DD18" s="164"/>
       <c r="DE18" s="7"/>
       <c r="DF18" s="7"/>
       <c r="DG18" s="7"/>
@@ -7639,7 +7618,7 @@
       <c r="CM19" s="86">
         <v>0.90100000000000002</v>
       </c>
-      <c r="CQ19" s="88"/>
+      <c r="CQ19" s="164"/>
       <c r="CR19" s="7"/>
       <c r="CS19" s="7"/>
       <c r="CT19" s="7"/>
@@ -7654,7 +7633,7 @@
       <c r="DB19">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD19" s="88"/>
+      <c r="DD19" s="164"/>
       <c r="DE19" s="7"/>
       <c r="DF19" s="7"/>
       <c r="DG19" s="7"/>
@@ -7671,7 +7650,7 @@
       <c r="CM20" s="85">
         <v>0.90400000000000003</v>
       </c>
-      <c r="CQ20" s="88"/>
+      <c r="CQ20" s="164"/>
       <c r="CR20" s="7"/>
       <c r="CS20" s="7"/>
       <c r="CT20" s="7"/>
@@ -7686,7 +7665,7 @@
       <c r="DB20">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD20" s="88"/>
+      <c r="DD20" s="164"/>
       <c r="DE20" s="7"/>
       <c r="DF20" s="7"/>
       <c r="DG20" s="7"/>
@@ -7703,7 +7682,7 @@
       <c r="CM21" s="85">
         <v>0.90900000000000003</v>
       </c>
-      <c r="CQ21" s="88"/>
+      <c r="CQ21" s="164"/>
       <c r="CR21" s="7"/>
       <c r="CS21" s="7"/>
       <c r="CT21" s="7"/>
@@ -7718,7 +7697,7 @@
       <c r="DB21">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD21" s="88"/>
+      <c r="DD21" s="164"/>
       <c r="DE21" s="7"/>
       <c r="DF21" s="7"/>
       <c r="DG21" s="7"/>
@@ -7735,7 +7714,7 @@
       <c r="CM22" s="85">
         <v>0.90900000000000003</v>
       </c>
-      <c r="CQ22" s="88"/>
+      <c r="CQ22" s="164"/>
       <c r="CR22" s="7"/>
       <c r="CS22" s="7"/>
       <c r="CT22" s="7"/>
@@ -7750,7 +7729,7 @@
       <c r="DB22">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD22" s="88"/>
+      <c r="DD22" s="164"/>
       <c r="DE22" s="7"/>
       <c r="DF22" s="7"/>
       <c r="DG22" s="7"/>
@@ -7767,7 +7746,7 @@
       <c r="CM23" s="86">
         <v>0.91200000000000003</v>
       </c>
-      <c r="CQ23" s="88"/>
+      <c r="CQ23" s="164"/>
       <c r="CR23" s="7"/>
       <c r="CS23" s="7"/>
       <c r="CT23" s="7"/>
@@ -7782,7 +7761,7 @@
       <c r="DB23">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD23" s="88"/>
+      <c r="DD23" s="164"/>
       <c r="DE23" s="7"/>
       <c r="DF23" s="7"/>
       <c r="DG23" s="7"/>
@@ -7799,7 +7778,7 @@
       <c r="CM24" s="85">
         <v>0.91</v>
       </c>
-      <c r="CQ24" s="88"/>
+      <c r="CQ24" s="164"/>
       <c r="CR24" s="7"/>
       <c r="CS24" s="7"/>
       <c r="CT24" s="7"/>
@@ -7814,7 +7793,7 @@
       <c r="DB24">
         <v>0.91200000000000003</v>
       </c>
-      <c r="DD24" s="88"/>
+      <c r="DD24" s="164"/>
       <c r="DE24" s="7"/>
       <c r="DF24" s="7"/>
       <c r="DG24" s="7"/>
@@ -7831,7 +7810,7 @@
       <c r="CM25" s="86">
         <v>0.91100000000000003</v>
       </c>
-      <c r="CQ25" s="88"/>
+      <c r="CQ25" s="164"/>
       <c r="CR25" s="7"/>
       <c r="CS25" s="7"/>
       <c r="CT25" s="7"/>
@@ -7863,7 +7842,7 @@
       <c r="CM26" s="85">
         <v>0.91100000000000003</v>
       </c>
-      <c r="CQ26" s="88"/>
+      <c r="CQ26" s="164"/>
       <c r="CR26" s="7"/>
       <c r="CS26" s="7"/>
       <c r="CT26" s="7"/>
@@ -7874,14 +7853,14 @@
       <c r="CY26" s="7"/>
       <c r="DD26" s="7"/>
       <c r="DE26" s="7"/>
-      <c r="DF26" s="87" t="s">
-        <v>80</v>
-      </c>
-      <c r="DG26" s="87"/>
-      <c r="DH26" s="87"/>
-      <c r="DI26" s="87"/>
-      <c r="DJ26" s="87"/>
-      <c r="DK26" s="87"/>
+      <c r="DF26" s="163" t="s">
+        <v>73</v>
+      </c>
+      <c r="DG26" s="163"/>
+      <c r="DH26" s="163"/>
+      <c r="DI26" s="163"/>
+      <c r="DJ26" s="163"/>
+      <c r="DK26" s="163"/>
       <c r="DL26" s="7"/>
     </row>
     <row r="27" spans="2:116" x14ac:dyDescent="0.3">
@@ -7891,7 +7870,7 @@
       <c r="CM27" s="85">
         <v>0.90900000000000003</v>
       </c>
-      <c r="CQ27" s="88"/>
+      <c r="CQ27" s="164"/>
       <c r="CR27" s="7"/>
       <c r="CS27" s="7"/>
       <c r="CT27" s="7"/>
@@ -7902,12 +7881,12 @@
       <c r="CY27" s="7"/>
       <c r="DD27" s="7"/>
       <c r="DE27" s="7"/>
-      <c r="DF27" s="87"/>
-      <c r="DG27" s="87"/>
-      <c r="DH27" s="87"/>
-      <c r="DI27" s="87"/>
-      <c r="DJ27" s="87"/>
-      <c r="DK27" s="87"/>
+      <c r="DF27" s="163"/>
+      <c r="DG27" s="163"/>
+      <c r="DH27" s="163"/>
+      <c r="DI27" s="163"/>
+      <c r="DJ27" s="163"/>
+      <c r="DK27" s="163"/>
       <c r="DL27" s="7"/>
     </row>
     <row r="28" spans="2:116" x14ac:dyDescent="0.3">
@@ -7917,7 +7896,7 @@
       <c r="CM28" s="85">
         <v>0.90600000000000003</v>
       </c>
-      <c r="CQ28" s="88"/>
+      <c r="CQ28" s="164"/>
       <c r="CR28" s="7"/>
       <c r="CS28" s="7"/>
       <c r="CT28" s="7"/>
@@ -7934,7 +7913,7 @@
       <c r="CM29" s="86">
         <v>0.90600000000000003</v>
       </c>
-      <c r="CQ29" s="88"/>
+      <c r="CQ29" s="164"/>
       <c r="CR29" s="7"/>
       <c r="CS29" s="7"/>
       <c r="CT29" s="7"/>
@@ -7951,7 +7930,7 @@
       <c r="CM30" s="85">
         <v>0.90800000000000003</v>
       </c>
-      <c r="CQ30" s="88"/>
+      <c r="CQ30" s="164"/>
       <c r="CR30" s="7"/>
       <c r="CS30" s="7"/>
       <c r="CT30" s="7"/>
@@ -8049,15 +8028,15 @@
         <v>0.90800000000000003</v>
       </c>
       <c r="CQ32" s="7"/>
-      <c r="CR32" s="87" t="s">
-        <v>77</v>
-      </c>
-      <c r="CS32" s="87"/>
-      <c r="CT32" s="87"/>
-      <c r="CU32" s="87"/>
-      <c r="CV32" s="87"/>
-      <c r="CW32" s="87"/>
-      <c r="CX32" s="87"/>
+      <c r="CR32" s="163" t="s">
+        <v>70</v>
+      </c>
+      <c r="CS32" s="163"/>
+      <c r="CT32" s="163"/>
+      <c r="CU32" s="163"/>
+      <c r="CV32" s="163"/>
+      <c r="CW32" s="163"/>
+      <c r="CX32" s="163"/>
       <c r="CY32" s="7"/>
     </row>
     <row r="33" spans="2:103" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8073,11 +8052,11 @@
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
       <c r="M33" s="7"/>
-      <c r="N33" s="144" t="s">
+      <c r="N33" s="97" t="s">
         <v>28</v>
       </c>
-      <c r="O33" s="147"/>
-      <c r="P33" s="147"/>
+      <c r="O33" s="87"/>
+      <c r="P33" s="87"/>
       <c r="Q33" s="7"/>
       <c r="R33" s="7"/>
       <c r="S33" s="7"/>
@@ -8098,13 +8077,13 @@
       <c r="AJ33" s="7"/>
       <c r="AK33" s="7"/>
       <c r="AL33" s="7"/>
-      <c r="AM33" s="144" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN33" s="144"/>
-      <c r="AO33" s="144"/>
-      <c r="AP33" s="144"/>
-      <c r="AQ33" s="144"/>
+      <c r="AM33" s="97" t="s">
+        <v>44</v>
+      </c>
+      <c r="AN33" s="97"/>
+      <c r="AO33" s="97"/>
+      <c r="AP33" s="97"/>
+      <c r="AQ33" s="97"/>
       <c r="AR33" s="7"/>
       <c r="AS33" s="7"/>
       <c r="AT33" s="7"/>
@@ -8124,40 +8103,40 @@
         <v>0.90800000000000003</v>
       </c>
       <c r="CQ33" s="7"/>
-      <c r="CR33" s="87"/>
-      <c r="CS33" s="87"/>
-      <c r="CT33" s="87"/>
-      <c r="CU33" s="87"/>
-      <c r="CV33" s="87"/>
-      <c r="CW33" s="87"/>
-      <c r="CX33" s="87"/>
+      <c r="CR33" s="163"/>
+      <c r="CS33" s="163"/>
+      <c r="CT33" s="163"/>
+      <c r="CU33" s="163"/>
+      <c r="CV33" s="163"/>
+      <c r="CW33" s="163"/>
+      <c r="CX33" s="163"/>
       <c r="CY33" s="7"/>
     </row>
     <row r="34" spans="2:103" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
-      <c r="E34" s="156" t="s">
+      <c r="E34" s="95" t="s">
         <v>12</v>
       </c>
-      <c r="F34" s="150"/>
-      <c r="G34" s="150"/>
-      <c r="H34" s="150"/>
-      <c r="I34" s="150"/>
+      <c r="F34" s="96"/>
+      <c r="G34" s="96"/>
+      <c r="H34" s="96"/>
+      <c r="I34" s="96"/>
       <c r="J34" s="7"/>
       <c r="K34" s="7"/>
       <c r="L34" s="7"/>
       <c r="M34" s="7"/>
-      <c r="N34" s="147"/>
-      <c r="O34" s="147"/>
-      <c r="P34" s="147"/>
+      <c r="N34" s="87"/>
+      <c r="O34" s="87"/>
+      <c r="P34" s="87"/>
       <c r="Q34" s="7"/>
       <c r="R34" s="7"/>
-      <c r="S34" s="144" t="s">
+      <c r="S34" s="97" t="s">
         <v>30</v>
       </c>
-      <c r="T34" s="158"/>
-      <c r="U34" s="158"/>
+      <c r="T34" s="100"/>
+      <c r="U34" s="100"/>
       <c r="V34" s="7"/>
       <c r="W34" s="7"/>
       <c r="X34" s="7"/>
@@ -8165,25 +8144,25 @@
       <c r="AB34" s="7"/>
       <c r="AC34" s="7"/>
       <c r="AD34" s="7"/>
-      <c r="AE34" s="156" t="s">
+      <c r="AE34" s="95" t="s">
         <v>12</v>
       </c>
-      <c r="AF34" s="150"/>
-      <c r="AG34" s="150"/>
-      <c r="AH34" s="150"/>
-      <c r="AI34" s="150"/>
+      <c r="AF34" s="96"/>
+      <c r="AG34" s="96"/>
+      <c r="AH34" s="96"/>
+      <c r="AI34" s="96"/>
       <c r="AJ34" s="7"/>
       <c r="AK34" s="7"/>
       <c r="AL34" s="7"/>
-      <c r="AM34" s="144"/>
-      <c r="AN34" s="144"/>
-      <c r="AO34" s="144"/>
-      <c r="AP34" s="144"/>
-      <c r="AQ34" s="144"/>
+      <c r="AM34" s="97"/>
+      <c r="AN34" s="97"/>
+      <c r="AO34" s="97"/>
+      <c r="AP34" s="97"/>
+      <c r="AQ34" s="97"/>
       <c r="AR34" s="7"/>
-      <c r="AS34" s="144"/>
-      <c r="AT34" s="158"/>
-      <c r="AU34" s="158"/>
+      <c r="AS34" s="97"/>
+      <c r="AT34" s="100"/>
+      <c r="AU34" s="100"/>
       <c r="AV34" s="7"/>
       <c r="AW34" s="7"/>
       <c r="AX34" s="7"/>
@@ -8197,11 +8176,11 @@
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="150"/>
-      <c r="F35" s="150"/>
-      <c r="G35" s="150"/>
-      <c r="H35" s="150"/>
-      <c r="I35" s="150"/>
+      <c r="E35" s="96"/>
+      <c r="F35" s="96"/>
+      <c r="G35" s="96"/>
+      <c r="H35" s="96"/>
+      <c r="I35" s="96"/>
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
       <c r="L35" s="7"/>
@@ -8221,11 +8200,11 @@
       <c r="AB35" s="7"/>
       <c r="AC35" s="7"/>
       <c r="AD35" s="7"/>
-      <c r="AE35" s="150"/>
-      <c r="AF35" s="150"/>
-      <c r="AG35" s="150"/>
-      <c r="AH35" s="150"/>
-      <c r="AI35" s="150"/>
+      <c r="AE35" s="96"/>
+      <c r="AF35" s="96"/>
+      <c r="AG35" s="96"/>
+      <c r="AH35" s="96"/>
+      <c r="AI35" s="96"/>
       <c r="AJ35" s="7"/>
       <c r="AK35" s="7"/>
       <c r="AL35" s="7"/>
@@ -8325,10 +8304,10 @@
       <c r="T37" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="U37" s="149" t="s">
+      <c r="U37" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="V37" s="149"/>
+      <c r="V37" s="92"/>
       <c r="W37" s="7"/>
       <c r="X37" s="7"/>
       <c r="Y37" s="7"/>
@@ -8353,8 +8332,8 @@
       <c r="AR37" s="7"/>
       <c r="AS37" s="7"/>
       <c r="AT37" s="7"/>
-      <c r="AU37" s="149"/>
-      <c r="AV37" s="149"/>
+      <c r="AU37" s="92"/>
+      <c r="AV37" s="92"/>
       <c r="AW37" s="7"/>
       <c r="AX37" s="7"/>
       <c r="AY37" s="7"/>
@@ -8392,33 +8371,33 @@
       <c r="Q38" s="7"/>
       <c r="R38" s="7"/>
       <c r="S38" s="7"/>
-      <c r="T38" s="112" t="s">
+      <c r="T38" s="98" t="s">
         <v>13</v>
       </c>
-      <c r="U38" s="149"/>
-      <c r="V38" s="149"/>
+      <c r="U38" s="92"/>
+      <c r="V38" s="92"/>
       <c r="W38" s="7"/>
       <c r="X38" s="7"/>
       <c r="Y38" s="7"/>
       <c r="AB38" s="7"/>
       <c r="AC38" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="AD38" s="6"/>
       <c r="AE38" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="AF38" s="6"/>
       <c r="AG38" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="AH38" s="6"/>
       <c r="AI38" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="AJ38" s="6"/>
       <c r="AK38" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="AL38" s="7"/>
       <c r="AM38" s="7"/>
@@ -8428,9 +8407,9 @@
       <c r="AQ38" s="7"/>
       <c r="AR38" s="7"/>
       <c r="AS38" s="7"/>
-      <c r="AT38" s="150"/>
-      <c r="AU38" s="149"/>
-      <c r="AV38" s="149"/>
+      <c r="AT38" s="96"/>
+      <c r="AU38" s="92"/>
+      <c r="AV38" s="92"/>
       <c r="AW38" s="7"/>
       <c r="AX38" s="7"/>
       <c r="AY38" s="7"/>
@@ -8458,13 +8437,13 @@
       <c r="Q39" s="7"/>
       <c r="R39" s="7"/>
       <c r="S39" s="7"/>
-      <c r="T39" s="157"/>
-      <c r="U39" s="149"/>
-      <c r="V39" s="149"/>
+      <c r="T39" s="99"/>
+      <c r="U39" s="92"/>
+      <c r="V39" s="92"/>
       <c r="W39" s="7"/>
       <c r="X39" s="7"/>
       <c r="AB39" s="7"/>
-      <c r="AC39" s="137"/>
+      <c r="AC39" s="118"/>
       <c r="AD39" s="6"/>
       <c r="AE39" s="17"/>
       <c r="AF39" s="6"/>
@@ -8472,7 +8451,7 @@
       <c r="AH39" s="6"/>
       <c r="AI39" s="17"/>
       <c r="AJ39" s="6"/>
-      <c r="AK39" s="112"/>
+      <c r="AK39" s="98"/>
       <c r="AL39" s="7"/>
       <c r="AM39" s="7"/>
       <c r="AN39" s="7"/>
@@ -8481,9 +8460,9 @@
       <c r="AQ39" s="7"/>
       <c r="AR39" s="7"/>
       <c r="AS39" s="7"/>
-      <c r="AT39" s="150"/>
-      <c r="AU39" s="149"/>
-      <c r="AV39" s="149"/>
+      <c r="AT39" s="96"/>
+      <c r="AU39" s="92"/>
+      <c r="AV39" s="92"/>
       <c r="AW39" s="7"/>
       <c r="AX39" s="7"/>
       <c r="AY39" s="7"/>
@@ -8513,13 +8492,13 @@
       <c r="Q40" s="7"/>
       <c r="R40" s="7"/>
       <c r="S40" s="7"/>
-      <c r="T40" s="164"/>
-      <c r="U40" s="149"/>
-      <c r="V40" s="149"/>
+      <c r="T40" s="94"/>
+      <c r="U40" s="92"/>
+      <c r="V40" s="92"/>
       <c r="W40" s="7"/>
       <c r="X40" s="7"/>
       <c r="AB40" s="7"/>
-      <c r="AC40" s="137"/>
+      <c r="AC40" s="118"/>
       <c r="AD40" s="6"/>
       <c r="AE40" s="17"/>
       <c r="AF40" s="6"/>
@@ -8527,7 +8506,7 @@
       <c r="AH40" s="6"/>
       <c r="AI40" s="17"/>
       <c r="AJ40" s="6"/>
-      <c r="AK40" s="112"/>
+      <c r="AK40" s="98"/>
       <c r="AL40" s="7"/>
       <c r="AM40" s="7"/>
       <c r="AN40" s="7"/>
@@ -8539,8 +8518,8 @@
       <c r="AR40" s="7"/>
       <c r="AS40" s="7"/>
       <c r="AT40" s="7"/>
-      <c r="AU40" s="149"/>
-      <c r="AV40" s="149"/>
+      <c r="AU40" s="92"/>
+      <c r="AV40" s="92"/>
       <c r="AW40" s="7"/>
       <c r="AX40" s="7"/>
       <c r="AY40" s="7"/>
@@ -8563,14 +8542,14 @@
       <c r="L41" s="7"/>
       <c r="M41" s="7"/>
       <c r="N41" s="7"/>
-      <c r="O41" s="134" t="s">
+      <c r="O41" s="105" t="s">
         <v>15</v>
       </c>
       <c r="P41" s="7"/>
       <c r="Q41" s="7"/>
       <c r="R41" s="7"/>
       <c r="S41" s="7"/>
-      <c r="T41" s="164"/>
+      <c r="T41" s="94"/>
       <c r="U41" s="7"/>
       <c r="V41" s="7"/>
       <c r="W41" s="7"/>
@@ -8588,7 +8567,7 @@
       <c r="AL41" s="7"/>
       <c r="AM41" s="7"/>
       <c r="AN41" s="7"/>
-      <c r="AO41" s="143" t="s">
+      <c r="AO41" s="107" t="s">
         <v>15</v>
       </c>
       <c r="AP41" s="7"/>
@@ -8620,12 +8599,12 @@
       <c r="L42" s="7"/>
       <c r="M42" s="7"/>
       <c r="N42" s="7"/>
-      <c r="O42" s="134"/>
+      <c r="O42" s="105"/>
       <c r="P42" s="7"/>
       <c r="Q42" s="7"/>
       <c r="R42" s="7"/>
       <c r="S42" s="7"/>
-      <c r="T42" s="164"/>
+      <c r="T42" s="94"/>
       <c r="U42" s="7"/>
       <c r="V42" s="7"/>
       <c r="W42" s="7"/>
@@ -8643,7 +8622,7 @@
       <c r="AL42" s="7"/>
       <c r="AM42" s="7"/>
       <c r="AN42" s="7"/>
-      <c r="AO42" s="143"/>
+      <c r="AO42" s="107"/>
       <c r="AP42" s="7"/>
       <c r="AQ42" s="7"/>
       <c r="AR42" s="7"/>
@@ -8673,14 +8652,14 @@
       <c r="L43" s="7"/>
       <c r="M43" s="7"/>
       <c r="N43" s="7"/>
-      <c r="O43" s="139" t="s">
+      <c r="O43" s="103" t="s">
         <v>23</v>
       </c>
       <c r="P43" s="7"/>
       <c r="Q43" s="7"/>
       <c r="R43" s="7"/>
       <c r="S43" s="7"/>
-      <c r="T43" s="164"/>
+      <c r="T43" s="94"/>
       <c r="U43" s="7"/>
       <c r="V43" s="7"/>
       <c r="W43" s="7"/>
@@ -8698,7 +8677,7 @@
       <c r="AL43" s="7"/>
       <c r="AM43" s="7"/>
       <c r="AN43" s="7"/>
-      <c r="AO43" s="151" t="s">
+      <c r="AO43" s="111" t="s">
         <v>23</v>
       </c>
       <c r="AP43" s="7"/>
@@ -8730,18 +8709,18 @@
       <c r="L44" s="7"/>
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
-      <c r="O44" s="140"/>
+      <c r="O44" s="104"/>
       <c r="P44" s="7"/>
       <c r="Q44" s="7"/>
       <c r="R44" s="7"/>
       <c r="S44" s="7"/>
-      <c r="T44" s="164"/>
-      <c r="U44" s="161" t="s">
+      <c r="T44" s="94"/>
+      <c r="U44" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="V44" s="153"/>
-      <c r="W44" s="153"/>
-      <c r="X44" s="153"/>
+      <c r="V44" s="89"/>
+      <c r="W44" s="89"/>
+      <c r="X44" s="89"/>
       <c r="AB44" s="7"/>
       <c r="AC44" s="19"/>
       <c r="AD44" s="6"/>
@@ -8755,16 +8734,16 @@
       <c r="AL44" s="7"/>
       <c r="AM44" s="7"/>
       <c r="AN44" s="7"/>
-      <c r="AO44" s="152"/>
+      <c r="AO44" s="112"/>
       <c r="AP44" s="7"/>
       <c r="AQ44" s="7"/>
       <c r="AR44" s="7"/>
       <c r="AS44" s="7"/>
       <c r="AT44" s="7"/>
-      <c r="AU44" s="153"/>
-      <c r="AV44" s="153"/>
-      <c r="AW44" s="153"/>
-      <c r="AX44" s="153"/>
+      <c r="AU44" s="89"/>
+      <c r="AV44" s="89"/>
+      <c r="AW44" s="89"/>
+      <c r="AX44" s="89"/>
       <c r="AY44" s="7"/>
       <c r="AZ44" s="7"/>
       <c r="BA44" s="7"/>
@@ -8785,18 +8764,18 @@
       <c r="L45" s="7"/>
       <c r="M45" s="7"/>
       <c r="N45" s="7"/>
-      <c r="O45" s="139" t="s">
+      <c r="O45" s="103" t="s">
         <v>22</v>
       </c>
       <c r="P45" s="7"/>
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="7"/>
-      <c r="T45" s="164"/>
-      <c r="U45" s="161"/>
-      <c r="V45" s="153"/>
-      <c r="W45" s="153"/>
-      <c r="X45" s="153"/>
+      <c r="T45" s="94"/>
+      <c r="U45" s="88"/>
+      <c r="V45" s="89"/>
+      <c r="W45" s="89"/>
+      <c r="X45" s="89"/>
       <c r="AB45" s="7"/>
       <c r="AC45" s="19"/>
       <c r="AD45" s="6"/>
@@ -8810,20 +8789,20 @@
       <c r="AL45" s="7"/>
       <c r="AM45" s="7"/>
       <c r="AN45" s="7"/>
-      <c r="AO45" s="151" t="s">
+      <c r="AO45" s="111" t="s">
         <v>22</v>
       </c>
-      <c r="AP45" s="159" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ45" s="160"/>
-      <c r="AR45" s="160"/>
-      <c r="AS45" s="160"/>
-      <c r="AT45" s="160"/>
-      <c r="AU45" s="153"/>
-      <c r="AV45" s="153"/>
-      <c r="AW45" s="153"/>
-      <c r="AX45" s="153"/>
+      <c r="AP45" s="101" t="s">
+        <v>61</v>
+      </c>
+      <c r="AQ45" s="102"/>
+      <c r="AR45" s="102"/>
+      <c r="AS45" s="102"/>
+      <c r="AT45" s="102"/>
+      <c r="AU45" s="89"/>
+      <c r="AV45" s="89"/>
+      <c r="AW45" s="89"/>
+      <c r="AX45" s="89"/>
       <c r="AY45" s="7"/>
       <c r="AZ45" s="7"/>
       <c r="BA45" s="7"/>
@@ -8854,17 +8833,17 @@
       <c r="L46" s="7"/>
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
-      <c r="O46" s="140"/>
+      <c r="O46" s="104"/>
       <c r="P46" s="7"/>
       <c r="Q46" s="7"/>
       <c r="R46" s="7"/>
       <c r="S46" s="7"/>
-      <c r="T46" s="164"/>
-      <c r="U46" s="163" t="s">
+      <c r="T46" s="94"/>
+      <c r="U46" s="93" t="s">
         <v>32</v>
       </c>
-      <c r="V46" s="147"/>
-      <c r="W46" s="147"/>
+      <c r="V46" s="87"/>
+      <c r="W46" s="87"/>
       <c r="X46" s="7"/>
       <c r="AB46" s="7"/>
       <c r="AC46" s="20">
@@ -8889,15 +8868,15 @@
       <c r="AL46" s="7"/>
       <c r="AM46" s="7"/>
       <c r="AN46" s="7"/>
-      <c r="AO46" s="152"/>
-      <c r="AP46" s="159"/>
-      <c r="AQ46" s="160"/>
-      <c r="AR46" s="160"/>
-      <c r="AS46" s="160"/>
-      <c r="AT46" s="160"/>
-      <c r="AU46" s="147"/>
-      <c r="AV46" s="147"/>
-      <c r="AW46" s="147"/>
+      <c r="AO46" s="112"/>
+      <c r="AP46" s="101"/>
+      <c r="AQ46" s="102"/>
+      <c r="AR46" s="102"/>
+      <c r="AS46" s="102"/>
+      <c r="AT46" s="102"/>
+      <c r="AU46" s="87"/>
+      <c r="AV46" s="87"/>
+      <c r="AW46" s="87"/>
       <c r="AX46" s="7"/>
       <c r="AY46" s="7"/>
       <c r="AZ46" s="7"/>
@@ -8929,14 +8908,14 @@
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
-      <c r="O47" s="134" t="s">
+      <c r="O47" s="105" t="s">
         <v>21</v>
       </c>
       <c r="P47" s="7"/>
       <c r="Q47" s="7"/>
       <c r="R47" s="7"/>
       <c r="S47" s="7"/>
-      <c r="T47" s="164"/>
+      <c r="T47" s="94"/>
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
@@ -8964,7 +8943,7 @@
       <c r="AL47" s="7"/>
       <c r="AM47" s="7"/>
       <c r="AN47" s="7"/>
-      <c r="AO47" s="143" t="s">
+      <c r="AO47" s="107" t="s">
         <v>21</v>
       </c>
       <c r="AP47" s="7"/>
@@ -9006,14 +8985,14 @@
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
-      <c r="O48" s="134"/>
-      <c r="P48" s="135" t="s">
+      <c r="O48" s="105"/>
+      <c r="P48" s="91" t="s">
         <v>27</v>
       </c>
-      <c r="Q48" s="136"/>
-      <c r="R48" s="136"/>
+      <c r="Q48" s="106"/>
+      <c r="R48" s="106"/>
       <c r="S48" s="7"/>
-      <c r="T48" s="164"/>
+      <c r="T48" s="94"/>
       <c r="U48" s="7"/>
       <c r="V48" s="7"/>
       <c r="W48" s="7"/>
@@ -9041,10 +9020,10 @@
       <c r="AL48" s="7"/>
       <c r="AM48" s="7"/>
       <c r="AN48" s="7"/>
-      <c r="AO48" s="143"/>
-      <c r="AP48" s="135"/>
-      <c r="AQ48" s="136"/>
-      <c r="AR48" s="136"/>
+      <c r="AO48" s="107"/>
+      <c r="AP48" s="91"/>
+      <c r="AQ48" s="106"/>
+      <c r="AR48" s="106"/>
       <c r="AS48" s="7"/>
       <c r="AT48" s="7"/>
       <c r="AU48" s="7"/>
@@ -9071,20 +9050,20 @@
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
       <c r="N49" s="7"/>
-      <c r="O49" s="134" t="s">
+      <c r="O49" s="105" t="s">
         <v>19</v>
       </c>
-      <c r="P49" s="136"/>
-      <c r="Q49" s="136"/>
-      <c r="R49" s="136"/>
+      <c r="P49" s="106"/>
+      <c r="Q49" s="106"/>
+      <c r="R49" s="106"/>
       <c r="S49" s="7"/>
-      <c r="T49" s="164"/>
-      <c r="U49" s="162" t="s">
+      <c r="T49" s="94"/>
+      <c r="U49" s="90" t="s">
         <v>25</v>
       </c>
-      <c r="V49" s="135"/>
-      <c r="W49" s="135"/>
-      <c r="X49" s="135"/>
+      <c r="V49" s="91"/>
+      <c r="W49" s="91"/>
+      <c r="X49" s="91"/>
       <c r="AB49" s="7"/>
       <c r="AC49" s="19"/>
       <c r="AD49" s="6"/>
@@ -9098,12 +9077,12 @@
       <c r="AL49" s="7"/>
       <c r="AM49" s="7"/>
       <c r="AN49" s="7"/>
-      <c r="AO49" s="143" t="s">
+      <c r="AO49" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="AP49" s="136"/>
-      <c r="AQ49" s="136"/>
-      <c r="AR49" s="136"/>
+      <c r="AP49" s="106"/>
+      <c r="AQ49" s="106"/>
+      <c r="AR49" s="106"/>
       <c r="AS49" s="7"/>
       <c r="AT49" s="7"/>
       <c r="AU49" s="72"/>
@@ -9130,16 +9109,16 @@
       <c r="L50" s="7"/>
       <c r="M50" s="7"/>
       <c r="N50" s="7"/>
-      <c r="O50" s="134"/>
+      <c r="O50" s="105"/>
       <c r="P50" s="7"/>
       <c r="Q50" s="7"/>
       <c r="R50" s="7"/>
       <c r="S50" s="7"/>
       <c r="T50" s="12"/>
-      <c r="U50" s="162"/>
-      <c r="V50" s="135"/>
-      <c r="W50" s="135"/>
-      <c r="X50" s="135"/>
+      <c r="U50" s="90"/>
+      <c r="V50" s="91"/>
+      <c r="W50" s="91"/>
+      <c r="X50" s="91"/>
       <c r="AB50" s="7"/>
       <c r="AC50" s="19"/>
       <c r="AD50" s="6"/>
@@ -9153,7 +9132,7 @@
       <c r="AL50" s="7"/>
       <c r="AM50" s="7"/>
       <c r="AN50" s="7"/>
-      <c r="AO50" s="143"/>
+      <c r="AO50" s="107"/>
       <c r="AP50" s="7"/>
       <c r="AQ50" s="7"/>
       <c r="AR50" s="7"/>
@@ -9183,18 +9162,18 @@
       <c r="L51" s="7"/>
       <c r="M51" s="7"/>
       <c r="N51" s="7"/>
-      <c r="O51" s="139" t="s">
+      <c r="O51" s="103" t="s">
         <v>20</v>
       </c>
       <c r="P51" s="7"/>
       <c r="Q51" s="7"/>
       <c r="R51" s="7"/>
       <c r="S51" s="7"/>
-      <c r="T51" s="141"/>
-      <c r="U51" s="162"/>
-      <c r="V51" s="135"/>
-      <c r="W51" s="135"/>
-      <c r="X51" s="135"/>
+      <c r="T51" s="116"/>
+      <c r="U51" s="90"/>
+      <c r="V51" s="91"/>
+      <c r="W51" s="91"/>
+      <c r="X51" s="91"/>
       <c r="AB51" s="7"/>
       <c r="AC51" s="19"/>
       <c r="AD51" s="6"/>
@@ -9208,7 +9187,7 @@
       <c r="AL51" s="7"/>
       <c r="AM51" s="7"/>
       <c r="AN51" s="7"/>
-      <c r="AO51" s="154" t="s">
+      <c r="AO51" s="113" t="s">
         <v>20</v>
       </c>
       <c r="AP51" s="7"/>
@@ -9240,18 +9219,18 @@
       <c r="L52" s="7"/>
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
-      <c r="O52" s="140"/>
+      <c r="O52" s="104"/>
       <c r="P52" s="7"/>
       <c r="Q52" s="7"/>
       <c r="R52" s="7"/>
       <c r="S52" s="7"/>
-      <c r="T52" s="141"/>
-      <c r="U52" s="162" t="s">
+      <c r="T52" s="116"/>
+      <c r="U52" s="90" t="s">
         <v>26</v>
       </c>
-      <c r="V52" s="135"/>
-      <c r="W52" s="135"/>
-      <c r="X52" s="135"/>
+      <c r="V52" s="91"/>
+      <c r="W52" s="91"/>
+      <c r="X52" s="91"/>
       <c r="AB52" s="7"/>
       <c r="AC52" s="19"/>
       <c r="AD52" s="6"/>
@@ -9265,15 +9244,15 @@
       <c r="AL52" s="7"/>
       <c r="AM52" s="7"/>
       <c r="AN52" s="7"/>
-      <c r="AO52" s="155"/>
-      <c r="AP52" s="148" t="s">
-        <v>65</v>
-      </c>
-      <c r="AQ52" s="149"/>
-      <c r="AR52" s="149"/>
-      <c r="AS52" s="149"/>
-      <c r="AT52" s="149"/>
-      <c r="AU52" s="149"/>
+      <c r="AO52" s="114"/>
+      <c r="AP52" s="110" t="s">
+        <v>59</v>
+      </c>
+      <c r="AQ52" s="92"/>
+      <c r="AR52" s="92"/>
+      <c r="AS52" s="92"/>
+      <c r="AT52" s="92"/>
+      <c r="AU52" s="92"/>
       <c r="AV52" s="72"/>
       <c r="AW52" s="72"/>
       <c r="AX52" s="72"/>
@@ -9297,18 +9276,18 @@
       <c r="L53" s="7"/>
       <c r="M53" s="7"/>
       <c r="N53" s="7"/>
-      <c r="O53" s="139" t="s">
+      <c r="O53" s="103" t="s">
         <v>16</v>
       </c>
       <c r="P53" s="7"/>
       <c r="Q53" s="7"/>
       <c r="R53" s="7"/>
       <c r="S53" s="7"/>
-      <c r="T53" s="141"/>
-      <c r="U53" s="162"/>
-      <c r="V53" s="135"/>
-      <c r="W53" s="135"/>
-      <c r="X53" s="135"/>
+      <c r="T53" s="116"/>
+      <c r="U53" s="90"/>
+      <c r="V53" s="91"/>
+      <c r="W53" s="91"/>
+      <c r="X53" s="91"/>
       <c r="AB53" s="7"/>
       <c r="AC53" s="19"/>
       <c r="AD53" s="6"/>
@@ -9322,15 +9301,15 @@
       <c r="AL53" s="7"/>
       <c r="AM53" s="7"/>
       <c r="AN53" s="7"/>
-      <c r="AO53" s="154" t="s">
+      <c r="AO53" s="113" t="s">
         <v>16</v>
       </c>
-      <c r="AP53" s="148"/>
-      <c r="AQ53" s="149"/>
-      <c r="AR53" s="149"/>
-      <c r="AS53" s="149"/>
-      <c r="AT53" s="149"/>
-      <c r="AU53" s="149"/>
+      <c r="AP53" s="110"/>
+      <c r="AQ53" s="92"/>
+      <c r="AR53" s="92"/>
+      <c r="AS53" s="92"/>
+      <c r="AT53" s="92"/>
+      <c r="AU53" s="92"/>
       <c r="AV53" s="72"/>
       <c r="AW53" s="72"/>
       <c r="AX53" s="72"/>
@@ -9354,16 +9333,16 @@
       <c r="L54" s="7"/>
       <c r="M54" s="7"/>
       <c r="N54" s="7"/>
-      <c r="O54" s="140"/>
+      <c r="O54" s="104"/>
       <c r="P54" s="7"/>
       <c r="Q54" s="7"/>
       <c r="R54" s="7"/>
       <c r="S54" s="7"/>
-      <c r="T54" s="141"/>
-      <c r="U54" s="162"/>
-      <c r="V54" s="135"/>
-      <c r="W54" s="135"/>
-      <c r="X54" s="135"/>
+      <c r="T54" s="116"/>
+      <c r="U54" s="90"/>
+      <c r="V54" s="91"/>
+      <c r="W54" s="91"/>
+      <c r="X54" s="91"/>
       <c r="AB54" s="7"/>
       <c r="AC54" s="21"/>
       <c r="AD54" s="6"/>
@@ -9377,7 +9356,7 @@
       <c r="AL54" s="7"/>
       <c r="AM54" s="7"/>
       <c r="AN54" s="7"/>
-      <c r="AO54" s="155"/>
+      <c r="AO54" s="114"/>
       <c r="AP54" s="71"/>
       <c r="AQ54" s="70"/>
       <c r="AR54" s="70"/>
@@ -9407,14 +9386,14 @@
       <c r="L55" s="7"/>
       <c r="M55" s="7"/>
       <c r="N55" s="7"/>
-      <c r="O55" s="139" t="s">
+      <c r="O55" s="103" t="s">
         <v>17</v>
       </c>
       <c r="P55" s="7"/>
       <c r="Q55" s="7"/>
       <c r="R55" s="7"/>
       <c r="S55" s="7"/>
-      <c r="T55" s="142"/>
+      <c r="T55" s="117"/>
       <c r="U55" s="7"/>
       <c r="V55" s="7"/>
       <c r="W55" s="7"/>
@@ -9432,7 +9411,7 @@
       <c r="AL55" s="7"/>
       <c r="AM55" s="7"/>
       <c r="AN55" s="7"/>
-      <c r="AO55" s="106" t="s">
+      <c r="AO55" s="119" t="s">
         <v>17</v>
       </c>
       <c r="AP55" s="7"/>
@@ -9464,7 +9443,7 @@
       <c r="L56" s="7"/>
       <c r="M56" s="7"/>
       <c r="N56" s="7"/>
-      <c r="O56" s="140"/>
+      <c r="O56" s="104"/>
       <c r="P56" s="7"/>
       <c r="Q56" s="7"/>
       <c r="R56" s="7"/>
@@ -9487,14 +9466,14 @@
       <c r="AL56" s="7"/>
       <c r="AM56" s="7"/>
       <c r="AN56" s="7"/>
-      <c r="AO56" s="108"/>
-      <c r="AP56" s="148" t="s">
-        <v>66</v>
-      </c>
-      <c r="AQ56" s="149"/>
-      <c r="AR56" s="149"/>
-      <c r="AS56" s="149"/>
-      <c r="AT56" s="149"/>
+      <c r="AO56" s="120"/>
+      <c r="AP56" s="110" t="s">
+        <v>60</v>
+      </c>
+      <c r="AQ56" s="92"/>
+      <c r="AR56" s="92"/>
+      <c r="AS56" s="92"/>
+      <c r="AT56" s="92"/>
       <c r="AU56" s="7"/>
       <c r="AV56" s="7"/>
       <c r="AW56" s="7"/>
@@ -9529,7 +9508,7 @@
       <c r="L57" s="7"/>
       <c r="M57" s="7"/>
       <c r="N57" s="7"/>
-      <c r="O57" s="139" t="s">
+      <c r="O57" s="103" t="s">
         <v>18</v>
       </c>
       <c r="P57" s="7"/>
@@ -9543,35 +9522,35 @@
       <c r="X57" s="7"/>
       <c r="AB57" s="7"/>
       <c r="AC57" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="AD57" s="6"/>
       <c r="AE57" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="AF57" s="6"/>
       <c r="AG57" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="AH57" s="6"/>
       <c r="AI57" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="AJ57" s="6"/>
       <c r="AK57" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="AL57" s="7"/>
       <c r="AM57" s="7"/>
       <c r="AN57" s="7"/>
-      <c r="AO57" s="106" t="s">
+      <c r="AO57" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="AP57" s="148"/>
-      <c r="AQ57" s="149"/>
-      <c r="AR57" s="149"/>
-      <c r="AS57" s="149"/>
-      <c r="AT57" s="149"/>
+      <c r="AP57" s="110"/>
+      <c r="AQ57" s="92"/>
+      <c r="AR57" s="92"/>
+      <c r="AS57" s="92"/>
+      <c r="AT57" s="92"/>
       <c r="AU57" s="7"/>
       <c r="AV57" s="7"/>
       <c r="AW57" s="7"/>
@@ -9596,7 +9575,7 @@
       <c r="L58" s="7"/>
       <c r="M58" s="7"/>
       <c r="N58" s="7"/>
-      <c r="O58" s="140"/>
+      <c r="O58" s="104"/>
       <c r="P58" s="7"/>
       <c r="Q58" s="7"/>
       <c r="R58" s="7"/>
@@ -9619,7 +9598,7 @@
       <c r="AL58" s="7"/>
       <c r="AM58" s="7"/>
       <c r="AN58" s="7"/>
-      <c r="AO58" s="107"/>
+      <c r="AO58" s="162"/>
       <c r="AP58" s="7"/>
       <c r="AQ58" s="7"/>
       <c r="AR58" s="7"/>
@@ -9701,19 +9680,19 @@
       <c r="K60" s="3"/>
       <c r="L60" s="7"/>
       <c r="M60" s="7"/>
-      <c r="N60" s="138" t="s">
+      <c r="N60" s="115" t="s">
         <v>33</v>
       </c>
-      <c r="O60" s="138"/>
-      <c r="P60" s="138"/>
+      <c r="O60" s="115"/>
+      <c r="P60" s="115"/>
       <c r="Q60" s="7"/>
-      <c r="R60" s="138" t="s">
+      <c r="R60" s="115" t="s">
         <v>34</v>
       </c>
-      <c r="S60" s="138"/>
-      <c r="T60" s="138"/>
-      <c r="U60" s="138"/>
-      <c r="V60" s="138"/>
+      <c r="S60" s="115"/>
+      <c r="T60" s="115"/>
+      <c r="U60" s="115"/>
+      <c r="V60" s="115"/>
       <c r="W60" s="7"/>
       <c r="X60" s="7"/>
       <c r="AB60" s="7"/>
@@ -9758,15 +9737,15 @@
       <c r="K61" s="3"/>
       <c r="L61" s="7"/>
       <c r="M61" s="7"/>
-      <c r="N61" s="138"/>
-      <c r="O61" s="138"/>
-      <c r="P61" s="138"/>
+      <c r="N61" s="115"/>
+      <c r="O61" s="115"/>
+      <c r="P61" s="115"/>
       <c r="Q61" s="7"/>
-      <c r="R61" s="138"/>
-      <c r="S61" s="138"/>
-      <c r="T61" s="138"/>
-      <c r="U61" s="138"/>
-      <c r="V61" s="138"/>
+      <c r="R61" s="115"/>
+      <c r="S61" s="115"/>
+      <c r="T61" s="115"/>
+      <c r="U61" s="115"/>
+      <c r="V61" s="115"/>
       <c r="W61" s="7"/>
       <c r="X61" s="7"/>
       <c r="AB61" s="7"/>
@@ -9781,19 +9760,19 @@
       <c r="AK61" s="17"/>
       <c r="AL61" s="7"/>
       <c r="AM61" s="7"/>
-      <c r="AN61" s="100" t="s">
+      <c r="AN61" s="156" t="s">
         <v>37</v>
       </c>
-      <c r="AO61" s="101"/>
-      <c r="AP61" s="101"/>
-      <c r="AQ61" s="101"/>
-      <c r="AR61" s="101"/>
-      <c r="AS61" s="101"/>
-      <c r="AT61" s="101"/>
-      <c r="AU61" s="101"/>
-      <c r="AV61" s="101"/>
-      <c r="AW61" s="101"/>
-      <c r="AX61" s="102"/>
+      <c r="AO61" s="157"/>
+      <c r="AP61" s="157"/>
+      <c r="AQ61" s="157"/>
+      <c r="AR61" s="157"/>
+      <c r="AS61" s="157"/>
+      <c r="AT61" s="157"/>
+      <c r="AU61" s="157"/>
+      <c r="AV61" s="157"/>
+      <c r="AW61" s="157"/>
+      <c r="AX61" s="158"/>
       <c r="AY61" s="7"/>
       <c r="AZ61" s="7"/>
       <c r="BA61" s="7"/>
@@ -9817,13 +9796,13 @@
       <c r="O62" s="7"/>
       <c r="P62" s="7"/>
       <c r="Q62" s="7"/>
-      <c r="R62" s="147" t="s">
+      <c r="R62" s="87" t="s">
         <v>35</v>
       </c>
-      <c r="S62" s="147"/>
-      <c r="T62" s="147"/>
-      <c r="U62" s="147"/>
-      <c r="V62" s="147"/>
+      <c r="S62" s="87"/>
+      <c r="T62" s="87"/>
+      <c r="U62" s="87"/>
+      <c r="V62" s="87"/>
       <c r="W62" s="7"/>
       <c r="X62" s="7"/>
       <c r="AB62" s="7"/>
@@ -9838,17 +9817,17 @@
       <c r="AK62" s="17"/>
       <c r="AL62" s="7"/>
       <c r="AM62" s="7"/>
-      <c r="AN62" s="103"/>
-      <c r="AO62" s="104"/>
-      <c r="AP62" s="104"/>
-      <c r="AQ62" s="104"/>
-      <c r="AR62" s="104"/>
-      <c r="AS62" s="104"/>
-      <c r="AT62" s="104"/>
-      <c r="AU62" s="104"/>
-      <c r="AV62" s="104"/>
-      <c r="AW62" s="104"/>
-      <c r="AX62" s="105"/>
+      <c r="AN62" s="159"/>
+      <c r="AO62" s="160"/>
+      <c r="AP62" s="160"/>
+      <c r="AQ62" s="160"/>
+      <c r="AR62" s="160"/>
+      <c r="AS62" s="160"/>
+      <c r="AT62" s="160"/>
+      <c r="AU62" s="160"/>
+      <c r="AV62" s="160"/>
+      <c r="AW62" s="160"/>
+      <c r="AX62" s="161"/>
       <c r="AY62" s="7"/>
       <c r="AZ62" s="7"/>
       <c r="BA62" s="7"/>
@@ -9891,19 +9870,19 @@
       <c r="AK63" s="17"/>
       <c r="AL63" s="7"/>
       <c r="AM63" s="7"/>
-      <c r="AN63" s="91" t="s">
-        <v>49</v>
-      </c>
-      <c r="AO63" s="92"/>
-      <c r="AP63" s="92"/>
-      <c r="AQ63" s="92"/>
-      <c r="AR63" s="92"/>
-      <c r="AS63" s="92"/>
-      <c r="AT63" s="92"/>
-      <c r="AU63" s="92"/>
-      <c r="AV63" s="92"/>
-      <c r="AW63" s="92"/>
-      <c r="AX63" s="93"/>
+      <c r="AN63" s="147" t="s">
+        <v>45</v>
+      </c>
+      <c r="AO63" s="148"/>
+      <c r="AP63" s="148"/>
+      <c r="AQ63" s="148"/>
+      <c r="AR63" s="148"/>
+      <c r="AS63" s="148"/>
+      <c r="AT63" s="148"/>
+      <c r="AU63" s="148"/>
+      <c r="AV63" s="148"/>
+      <c r="AW63" s="148"/>
+      <c r="AX63" s="149"/>
       <c r="AY63" s="7"/>
       <c r="AZ63" s="7"/>
       <c r="BA63" s="7"/>
@@ -9966,17 +9945,17 @@
       </c>
       <c r="AL64" s="7"/>
       <c r="AM64" s="7"/>
-      <c r="AN64" s="91"/>
-      <c r="AO64" s="92"/>
-      <c r="AP64" s="92"/>
-      <c r="AQ64" s="92"/>
-      <c r="AR64" s="92"/>
-      <c r="AS64" s="92"/>
-      <c r="AT64" s="92"/>
-      <c r="AU64" s="92"/>
-      <c r="AV64" s="92"/>
-      <c r="AW64" s="92"/>
-      <c r="AX64" s="93"/>
+      <c r="AN64" s="147"/>
+      <c r="AO64" s="148"/>
+      <c r="AP64" s="148"/>
+      <c r="AQ64" s="148"/>
+      <c r="AR64" s="148"/>
+      <c r="AS64" s="148"/>
+      <c r="AT64" s="148"/>
+      <c r="AU64" s="148"/>
+      <c r="AV64" s="148"/>
+      <c r="AW64" s="148"/>
+      <c r="AX64" s="149"/>
       <c r="AY64" s="7"/>
       <c r="AZ64" s="7"/>
       <c r="BA64" s="7"/>
@@ -10039,19 +10018,19 @@
       </c>
       <c r="AL65" s="7"/>
       <c r="AM65" s="7"/>
-      <c r="AN65" s="94" t="s">
+      <c r="AN65" s="150" t="s">
         <v>38</v>
       </c>
-      <c r="AO65" s="95"/>
-      <c r="AP65" s="95"/>
-      <c r="AQ65" s="95"/>
-      <c r="AR65" s="95"/>
-      <c r="AS65" s="95"/>
-      <c r="AT65" s="95"/>
-      <c r="AU65" s="95"/>
-      <c r="AV65" s="95"/>
-      <c r="AW65" s="95"/>
-      <c r="AX65" s="96"/>
+      <c r="AO65" s="151"/>
+      <c r="AP65" s="151"/>
+      <c r="AQ65" s="151"/>
+      <c r="AR65" s="151"/>
+      <c r="AS65" s="151"/>
+      <c r="AT65" s="151"/>
+      <c r="AU65" s="151"/>
+      <c r="AV65" s="151"/>
+      <c r="AW65" s="151"/>
+      <c r="AX65" s="152"/>
       <c r="AY65" s="7"/>
       <c r="AZ65" s="7"/>
       <c r="BA65" s="7"/>
@@ -10114,17 +10093,17 @@
       </c>
       <c r="AL66" s="7"/>
       <c r="AM66" s="7"/>
-      <c r="AN66" s="97"/>
-      <c r="AO66" s="98"/>
-      <c r="AP66" s="98"/>
-      <c r="AQ66" s="98"/>
-      <c r="AR66" s="98"/>
-      <c r="AS66" s="98"/>
-      <c r="AT66" s="98"/>
-      <c r="AU66" s="98"/>
-      <c r="AV66" s="98"/>
-      <c r="AW66" s="98"/>
-      <c r="AX66" s="99"/>
+      <c r="AN66" s="153"/>
+      <c r="AO66" s="154"/>
+      <c r="AP66" s="154"/>
+      <c r="AQ66" s="154"/>
+      <c r="AR66" s="154"/>
+      <c r="AS66" s="154"/>
+      <c r="AT66" s="154"/>
+      <c r="AU66" s="154"/>
+      <c r="AV66" s="154"/>
+      <c r="AW66" s="154"/>
+      <c r="AX66" s="155"/>
       <c r="AY66" s="7"/>
       <c r="AZ66" s="7"/>
       <c r="BA66" s="7"/>
@@ -10167,19 +10146,19 @@
       <c r="AK67" s="17"/>
       <c r="AL67" s="7"/>
       <c r="AM67" s="7"/>
-      <c r="AN67" s="145" t="s">
-        <v>64</v>
-      </c>
-      <c r="AO67" s="146"/>
-      <c r="AP67" s="146"/>
-      <c r="AQ67" s="146"/>
-      <c r="AR67" s="146"/>
-      <c r="AS67" s="146"/>
-      <c r="AT67" s="146"/>
-      <c r="AU67" s="146"/>
-      <c r="AV67" s="146"/>
-      <c r="AW67" s="146"/>
-      <c r="AX67" s="146"/>
+      <c r="AN67" s="108" t="s">
+        <v>58</v>
+      </c>
+      <c r="AO67" s="109"/>
+      <c r="AP67" s="109"/>
+      <c r="AQ67" s="109"/>
+      <c r="AR67" s="109"/>
+      <c r="AS67" s="109"/>
+      <c r="AT67" s="109"/>
+      <c r="AU67" s="109"/>
+      <c r="AV67" s="109"/>
+      <c r="AW67" s="109"/>
+      <c r="AX67" s="109"/>
       <c r="AY67" s="7"/>
       <c r="AZ67" s="7"/>
       <c r="BA67" s="7"/>
@@ -10222,17 +10201,17 @@
       <c r="AK68" s="17"/>
       <c r="AL68" s="7"/>
       <c r="AM68" s="7"/>
-      <c r="AN68" s="147"/>
-      <c r="AO68" s="147"/>
-      <c r="AP68" s="147"/>
-      <c r="AQ68" s="147"/>
-      <c r="AR68" s="147"/>
-      <c r="AS68" s="147"/>
-      <c r="AT68" s="147"/>
-      <c r="AU68" s="147"/>
-      <c r="AV68" s="147"/>
-      <c r="AW68" s="147"/>
-      <c r="AX68" s="147"/>
+      <c r="AN68" s="87"/>
+      <c r="AO68" s="87"/>
+      <c r="AP68" s="87"/>
+      <c r="AQ68" s="87"/>
+      <c r="AR68" s="87"/>
+      <c r="AS68" s="87"/>
+      <c r="AT68" s="87"/>
+      <c r="AU68" s="87"/>
+      <c r="AV68" s="87"/>
+      <c r="AW68" s="87"/>
+      <c r="AX68" s="87"/>
       <c r="AY68" s="7"/>
       <c r="AZ68" s="7"/>
       <c r="BA68" s="7"/>
@@ -10544,7 +10523,7 @@
       <c r="AB75" s="7"/>
       <c r="AC75" s="23"/>
       <c r="AD75" s="16" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="AE75" s="16"/>
       <c r="AF75" s="27"/>
@@ -10576,7 +10555,7 @@
       <c r="AB76" s="7"/>
       <c r="AC76" s="24"/>
       <c r="AD76" s="28" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="AE76" s="28"/>
       <c r="AF76" s="29"/>
@@ -10604,34 +10583,34 @@
       <c r="BB76" s="7"/>
       <c r="BC76" s="7"/>
       <c r="BG76" s="7"/>
-      <c r="BH76" s="89" t="s">
-        <v>72</v>
-      </c>
-      <c r="BI76" s="89"/>
-      <c r="BJ76" s="89"/>
-      <c r="BK76" s="89"/>
-      <c r="BL76" s="89"/>
-      <c r="BM76" s="89"/>
-      <c r="BN76" s="89"/>
-      <c r="BO76" s="89"/>
-      <c r="BP76" s="89"/>
-      <c r="BQ76" s="89"/>
-      <c r="BR76" s="89"/>
-      <c r="BS76" s="89"/>
-      <c r="BT76" s="89"/>
-      <c r="BU76" s="89"/>
-      <c r="BV76" s="89"/>
+      <c r="BH76" s="146" t="s">
+        <v>65</v>
+      </c>
+      <c r="BI76" s="146"/>
+      <c r="BJ76" s="146"/>
+      <c r="BK76" s="146"/>
+      <c r="BL76" s="146"/>
+      <c r="BM76" s="146"/>
+      <c r="BN76" s="146"/>
+      <c r="BO76" s="146"/>
+      <c r="BP76" s="146"/>
+      <c r="BQ76" s="146"/>
+      <c r="BR76" s="146"/>
+      <c r="BS76" s="146"/>
+      <c r="BT76" s="146"/>
+      <c r="BU76" s="146"/>
+      <c r="BV76" s="146"/>
       <c r="BW76" s="10"/>
       <c r="BX76" s="80"/>
-      <c r="BY76" s="89" t="s">
-        <v>73</v>
-      </c>
-      <c r="BZ76" s="89"/>
-      <c r="CA76" s="89"/>
-      <c r="CB76" s="89"/>
-      <c r="CC76" s="89"/>
-      <c r="CD76" s="89"/>
-      <c r="CE76" s="89"/>
+      <c r="BY76" s="146" t="s">
+        <v>66</v>
+      </c>
+      <c r="BZ76" s="146"/>
+      <c r="CA76" s="146"/>
+      <c r="CB76" s="146"/>
+      <c r="CC76" s="146"/>
+      <c r="CD76" s="146"/>
+      <c r="CE76" s="146"/>
       <c r="CF76" s="80"/>
     </row>
     <row r="77" spans="2:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -10664,30 +10643,30 @@
       <c r="BB77" s="7"/>
       <c r="BC77" s="7"/>
       <c r="BG77" s="7"/>
-      <c r="BH77" s="89"/>
-      <c r="BI77" s="89"/>
-      <c r="BJ77" s="89"/>
-      <c r="BK77" s="89"/>
-      <c r="BL77" s="89"/>
-      <c r="BM77" s="89"/>
-      <c r="BN77" s="89"/>
-      <c r="BO77" s="89"/>
-      <c r="BP77" s="89"/>
-      <c r="BQ77" s="89"/>
-      <c r="BR77" s="89"/>
-      <c r="BS77" s="89"/>
-      <c r="BT77" s="89"/>
-      <c r="BU77" s="89"/>
-      <c r="BV77" s="89"/>
+      <c r="BH77" s="146"/>
+      <c r="BI77" s="146"/>
+      <c r="BJ77" s="146"/>
+      <c r="BK77" s="146"/>
+      <c r="BL77" s="146"/>
+      <c r="BM77" s="146"/>
+      <c r="BN77" s="146"/>
+      <c r="BO77" s="146"/>
+      <c r="BP77" s="146"/>
+      <c r="BQ77" s="146"/>
+      <c r="BR77" s="146"/>
+      <c r="BS77" s="146"/>
+      <c r="BT77" s="146"/>
+      <c r="BU77" s="146"/>
+      <c r="BV77" s="146"/>
       <c r="BW77" s="10"/>
       <c r="BX77" s="80"/>
-      <c r="BY77" s="89"/>
-      <c r="BZ77" s="89"/>
-      <c r="CA77" s="89"/>
-      <c r="CB77" s="89"/>
-      <c r="CC77" s="89"/>
-      <c r="CD77" s="89"/>
-      <c r="CE77" s="89"/>
+      <c r="BY77" s="146"/>
+      <c r="BZ77" s="146"/>
+      <c r="CA77" s="146"/>
+      <c r="CB77" s="146"/>
+      <c r="CC77" s="146"/>
+      <c r="CD77" s="146"/>
+      <c r="CE77" s="146"/>
       <c r="CF77" s="80"/>
     </row>
     <row r="78" spans="2:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -10703,30 +10682,30 @@
       <c r="BB78" s="7"/>
       <c r="BC78" s="7"/>
       <c r="BG78" s="7"/>
-      <c r="BH78" s="89"/>
-      <c r="BI78" s="89"/>
-      <c r="BJ78" s="89"/>
-      <c r="BK78" s="89"/>
-      <c r="BL78" s="89"/>
-      <c r="BM78" s="89"/>
-      <c r="BN78" s="89"/>
-      <c r="BO78" s="89"/>
-      <c r="BP78" s="89"/>
-      <c r="BQ78" s="89"/>
-      <c r="BR78" s="89"/>
-      <c r="BS78" s="89"/>
-      <c r="BT78" s="89"/>
-      <c r="BU78" s="89"/>
-      <c r="BV78" s="89"/>
+      <c r="BH78" s="146"/>
+      <c r="BI78" s="146"/>
+      <c r="BJ78" s="146"/>
+      <c r="BK78" s="146"/>
+      <c r="BL78" s="146"/>
+      <c r="BM78" s="146"/>
+      <c r="BN78" s="146"/>
+      <c r="BO78" s="146"/>
+      <c r="BP78" s="146"/>
+      <c r="BQ78" s="146"/>
+      <c r="BR78" s="146"/>
+      <c r="BS78" s="146"/>
+      <c r="BT78" s="146"/>
+      <c r="BU78" s="146"/>
+      <c r="BV78" s="146"/>
       <c r="BW78" s="10"/>
       <c r="BX78" s="80"/>
-      <c r="BY78" s="89"/>
-      <c r="BZ78" s="89"/>
-      <c r="CA78" s="89"/>
-      <c r="CB78" s="89"/>
-      <c r="CC78" s="89"/>
-      <c r="CD78" s="89"/>
-      <c r="CE78" s="89"/>
+      <c r="BY78" s="146"/>
+      <c r="BZ78" s="146"/>
+      <c r="CA78" s="146"/>
+      <c r="CB78" s="146"/>
+      <c r="CC78" s="146"/>
+      <c r="CD78" s="146"/>
+      <c r="CE78" s="146"/>
       <c r="CF78" s="80"/>
     </row>
     <row r="79" spans="2:84" x14ac:dyDescent="0.3">
@@ -10754,13 +10733,13 @@
       <c r="BV79" s="7"/>
       <c r="BW79" s="10"/>
       <c r="BX79" s="7"/>
-      <c r="BY79" s="89"/>
-      <c r="BZ79" s="89"/>
-      <c r="CA79" s="89"/>
-      <c r="CB79" s="89"/>
-      <c r="CC79" s="89"/>
-      <c r="CD79" s="89"/>
-      <c r="CE79" s="89"/>
+      <c r="BY79" s="146"/>
+      <c r="BZ79" s="146"/>
+      <c r="CA79" s="146"/>
+      <c r="CB79" s="146"/>
+      <c r="CC79" s="146"/>
+      <c r="CD79" s="146"/>
+      <c r="CE79" s="146"/>
       <c r="CF79" s="7"/>
     </row>
     <row r="80" spans="2:84" x14ac:dyDescent="0.3">
@@ -10795,44 +10774,44 @@
       <c r="BE81" s="6"/>
       <c r="BG81" s="6"/>
       <c r="BH81" s="33" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="BI81" s="6"/>
       <c r="BJ81" s="33" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="BK81" s="6"/>
       <c r="BL81" s="33" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="BM81" s="7"/>
       <c r="BN81" s="33" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="BO81" s="6"/>
       <c r="BP81" s="33" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="BQ81" s="6"/>
       <c r="BR81" s="33" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="BS81" s="6"/>
       <c r="BT81" s="33" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="BU81" s="6"/>
       <c r="BV81" s="33" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="BW81" s="10"/>
       <c r="BX81" s="33" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="BZ81" s="7"/>
       <c r="CA81" s="69"/>
       <c r="CB81" s="33" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="CC81" s="7"/>
       <c r="CD81" s="7"/>
@@ -10846,7 +10825,7 @@
       <c r="BI82" s="6"/>
       <c r="BJ82" s="17"/>
       <c r="BK82" s="6"/>
-      <c r="BL82" s="112"/>
+      <c r="BL82" s="98"/>
       <c r="BM82" s="7"/>
       <c r="BN82" s="17"/>
       <c r="BO82" s="6"/>
@@ -10862,7 +10841,7 @@
       <c r="BY82" s="7"/>
       <c r="BZ82" s="7"/>
       <c r="CA82" s="69"/>
-      <c r="CB82" s="113"/>
+      <c r="CB82" s="124"/>
       <c r="CC82" s="7"/>
       <c r="CD82" s="7"/>
       <c r="CE82" s="7"/>
@@ -10875,7 +10854,7 @@
       <c r="BI83" s="6"/>
       <c r="BJ83" s="17"/>
       <c r="BK83" s="6"/>
-      <c r="BL83" s="112"/>
+      <c r="BL83" s="98"/>
       <c r="BM83" s="7"/>
       <c r="BN83" s="17"/>
       <c r="BO83" s="6"/>
@@ -10891,7 +10870,7 @@
       <c r="BY83" s="7"/>
       <c r="BZ83" s="7"/>
       <c r="CA83" s="69"/>
-      <c r="CB83" s="113"/>
+      <c r="CB83" s="124"/>
       <c r="CC83" s="7"/>
       <c r="CD83" s="7"/>
       <c r="CE83" s="7"/>
@@ -10977,10 +10956,10 @@
       <c r="BW86" s="10"/>
       <c r="BX86" s="17"/>
       <c r="BY86" s="7"/>
-      <c r="BZ86" s="115" t="s">
-        <v>62</v>
-      </c>
-      <c r="CA86" s="116"/>
+      <c r="BZ86" s="127" t="s">
+        <v>56</v>
+      </c>
+      <c r="CA86" s="128"/>
       <c r="CB86" s="32"/>
       <c r="CC86" s="7"/>
       <c r="CD86" s="7"/>
@@ -11008,8 +10987,8 @@
       <c r="BW87" s="10"/>
       <c r="BX87" s="17"/>
       <c r="BY87" s="7"/>
-      <c r="BZ87" s="115"/>
-      <c r="CA87" s="116"/>
+      <c r="BZ87" s="127"/>
+      <c r="CA87" s="128"/>
       <c r="CB87" s="32"/>
       <c r="CC87" s="7"/>
       <c r="CD87" s="7"/>
@@ -11040,10 +11019,10 @@
       <c r="BZ88" s="7"/>
       <c r="CA88" s="69"/>
       <c r="CB88" s="2"/>
-      <c r="CC88" s="117" t="s">
-        <v>63</v>
-      </c>
-      <c r="CD88" s="118"/>
+      <c r="CC88" s="129" t="s">
+        <v>57</v>
+      </c>
+      <c r="CD88" s="130"/>
       <c r="CE88" s="7"/>
       <c r="CF88" s="7"/>
     </row>
@@ -11071,8 +11050,8 @@
       <c r="BZ89" s="7"/>
       <c r="CA89" s="69"/>
       <c r="CB89" s="3"/>
-      <c r="CC89" s="119"/>
-      <c r="CD89" s="118"/>
+      <c r="CC89" s="131"/>
+      <c r="CD89" s="130"/>
       <c r="CE89" s="7"/>
       <c r="CF89" s="7"/>
       <c r="CJ89" t="s">
@@ -11314,23 +11293,23 @@
     <row r="98" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG98" s="7"/>
       <c r="BH98" s="39"/>
-      <c r="BI98" s="114" t="s">
+      <c r="BI98" s="125" t="s">
         <v>40</v>
       </c>
-      <c r="BJ98" s="114"/>
-      <c r="BK98" s="114"/>
-      <c r="BL98" s="114"/>
-      <c r="BM98" s="114"/>
-      <c r="BN98" s="114"/>
-      <c r="BO98" s="114"/>
-      <c r="BP98" s="114"/>
-      <c r="BQ98" s="114"/>
-      <c r="BR98" s="114"/>
-      <c r="BS98" s="114"/>
-      <c r="BT98" s="114"/>
-      <c r="BU98" s="114"/>
-      <c r="BV98" s="114"/>
-      <c r="BW98" s="114"/>
+      <c r="BJ98" s="125"/>
+      <c r="BK98" s="125"/>
+      <c r="BL98" s="125"/>
+      <c r="BM98" s="125"/>
+      <c r="BN98" s="125"/>
+      <c r="BO98" s="125"/>
+      <c r="BP98" s="125"/>
+      <c r="BQ98" s="125"/>
+      <c r="BR98" s="125"/>
+      <c r="BS98" s="125"/>
+      <c r="BT98" s="125"/>
+      <c r="BU98" s="125"/>
+      <c r="BV98" s="125"/>
+      <c r="BW98" s="125"/>
       <c r="BX98" s="40"/>
       <c r="BY98" s="7"/>
       <c r="BZ98" s="7"/>
@@ -11344,21 +11323,21 @@
     <row r="99" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG99" s="7"/>
       <c r="BH99" s="39"/>
-      <c r="BI99" s="114"/>
-      <c r="BJ99" s="114"/>
-      <c r="BK99" s="114"/>
-      <c r="BL99" s="114"/>
-      <c r="BM99" s="114"/>
-      <c r="BN99" s="114"/>
-      <c r="BO99" s="114"/>
-      <c r="BP99" s="114"/>
-      <c r="BQ99" s="114"/>
-      <c r="BR99" s="114"/>
-      <c r="BS99" s="114"/>
-      <c r="BT99" s="114"/>
-      <c r="BU99" s="114"/>
-      <c r="BV99" s="114"/>
-      <c r="BW99" s="114"/>
+      <c r="BI99" s="125"/>
+      <c r="BJ99" s="125"/>
+      <c r="BK99" s="125"/>
+      <c r="BL99" s="125"/>
+      <c r="BM99" s="125"/>
+      <c r="BN99" s="125"/>
+      <c r="BO99" s="125"/>
+      <c r="BP99" s="125"/>
+      <c r="BQ99" s="125"/>
+      <c r="BR99" s="125"/>
+      <c r="BS99" s="125"/>
+      <c r="BT99" s="125"/>
+      <c r="BU99" s="125"/>
+      <c r="BV99" s="125"/>
+      <c r="BW99" s="125"/>
       <c r="BX99" s="40"/>
       <c r="BY99" s="7"/>
       <c r="BZ99" s="7"/>
@@ -11372,21 +11351,21 @@
     <row r="100" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG100" s="7"/>
       <c r="BH100" s="39"/>
-      <c r="BI100" s="114"/>
-      <c r="BJ100" s="114"/>
-      <c r="BK100" s="114"/>
-      <c r="BL100" s="114"/>
-      <c r="BM100" s="114"/>
-      <c r="BN100" s="114"/>
-      <c r="BO100" s="114"/>
-      <c r="BP100" s="114"/>
-      <c r="BQ100" s="114"/>
-      <c r="BR100" s="114"/>
-      <c r="BS100" s="114"/>
-      <c r="BT100" s="114"/>
-      <c r="BU100" s="114"/>
-      <c r="BV100" s="114"/>
-      <c r="BW100" s="114"/>
+      <c r="BI100" s="125"/>
+      <c r="BJ100" s="125"/>
+      <c r="BK100" s="125"/>
+      <c r="BL100" s="125"/>
+      <c r="BM100" s="125"/>
+      <c r="BN100" s="125"/>
+      <c r="BO100" s="125"/>
+      <c r="BP100" s="125"/>
+      <c r="BQ100" s="125"/>
+      <c r="BR100" s="125"/>
+      <c r="BS100" s="125"/>
+      <c r="BT100" s="125"/>
+      <c r="BU100" s="125"/>
+      <c r="BV100" s="125"/>
+      <c r="BW100" s="125"/>
       <c r="BX100" s="40"/>
       <c r="BY100" s="7"/>
       <c r="BZ100" s="7"/>
@@ -11400,21 +11379,21 @@
     <row r="101" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG101" s="7"/>
       <c r="BH101" s="39"/>
-      <c r="BI101" s="114"/>
-      <c r="BJ101" s="114"/>
-      <c r="BK101" s="114"/>
-      <c r="BL101" s="114"/>
-      <c r="BM101" s="114"/>
-      <c r="BN101" s="114"/>
-      <c r="BO101" s="114"/>
-      <c r="BP101" s="114"/>
-      <c r="BQ101" s="114"/>
-      <c r="BR101" s="114"/>
-      <c r="BS101" s="114"/>
-      <c r="BT101" s="114"/>
-      <c r="BU101" s="114"/>
-      <c r="BV101" s="114"/>
-      <c r="BW101" s="114"/>
+      <c r="BI101" s="125"/>
+      <c r="BJ101" s="125"/>
+      <c r="BK101" s="125"/>
+      <c r="BL101" s="125"/>
+      <c r="BM101" s="125"/>
+      <c r="BN101" s="125"/>
+      <c r="BO101" s="125"/>
+      <c r="BP101" s="125"/>
+      <c r="BQ101" s="125"/>
+      <c r="BR101" s="125"/>
+      <c r="BS101" s="125"/>
+      <c r="BT101" s="125"/>
+      <c r="BU101" s="125"/>
+      <c r="BV101" s="125"/>
+      <c r="BW101" s="125"/>
       <c r="BX101" s="40"/>
       <c r="BY101" s="7"/>
       <c r="BZ101" s="7"/>
@@ -11428,21 +11407,21 @@
     <row r="102" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG102" s="7"/>
       <c r="BH102" s="39"/>
-      <c r="BI102" s="114"/>
-      <c r="BJ102" s="114"/>
-      <c r="BK102" s="114"/>
-      <c r="BL102" s="114"/>
-      <c r="BM102" s="114"/>
-      <c r="BN102" s="114"/>
-      <c r="BO102" s="114"/>
-      <c r="BP102" s="114"/>
-      <c r="BQ102" s="114"/>
-      <c r="BR102" s="114"/>
-      <c r="BS102" s="114"/>
-      <c r="BT102" s="114"/>
-      <c r="BU102" s="114"/>
-      <c r="BV102" s="114"/>
-      <c r="BW102" s="114"/>
+      <c r="BI102" s="125"/>
+      <c r="BJ102" s="125"/>
+      <c r="BK102" s="125"/>
+      <c r="BL102" s="125"/>
+      <c r="BM102" s="125"/>
+      <c r="BN102" s="125"/>
+      <c r="BO102" s="125"/>
+      <c r="BP102" s="125"/>
+      <c r="BQ102" s="125"/>
+      <c r="BR102" s="125"/>
+      <c r="BS102" s="125"/>
+      <c r="BT102" s="125"/>
+      <c r="BU102" s="125"/>
+      <c r="BV102" s="125"/>
+      <c r="BW102" s="125"/>
       <c r="BX102" s="40"/>
       <c r="BY102" s="7"/>
       <c r="BZ102" s="7"/>
@@ -11687,15 +11666,15 @@
       <c r="BM111" s="45"/>
       <c r="BN111" s="45"/>
       <c r="BO111" s="45"/>
-      <c r="BP111" s="133" t="s">
+      <c r="BP111" s="145" t="s">
         <v>41</v>
       </c>
-      <c r="BQ111" s="133"/>
-      <c r="BR111" s="133"/>
-      <c r="BS111" s="133"/>
-      <c r="BT111" s="133"/>
-      <c r="BU111" s="133"/>
-      <c r="BV111" s="133"/>
+      <c r="BQ111" s="145"/>
+      <c r="BR111" s="145"/>
+      <c r="BS111" s="145"/>
+      <c r="BT111" s="145"/>
+      <c r="BU111" s="145"/>
+      <c r="BV111" s="145"/>
       <c r="BW111" s="56"/>
       <c r="BX111" s="11"/>
       <c r="BY111" s="45"/>
@@ -11717,13 +11696,13 @@
       <c r="BM112" s="45"/>
       <c r="BN112" s="45"/>
       <c r="BO112" s="45"/>
-      <c r="BP112" s="133"/>
-      <c r="BQ112" s="133"/>
-      <c r="BR112" s="133"/>
-      <c r="BS112" s="133"/>
-      <c r="BT112" s="133"/>
-      <c r="BU112" s="133"/>
-      <c r="BV112" s="133"/>
+      <c r="BP112" s="145"/>
+      <c r="BQ112" s="145"/>
+      <c r="BR112" s="145"/>
+      <c r="BS112" s="145"/>
+      <c r="BT112" s="145"/>
+      <c r="BU112" s="145"/>
+      <c r="BV112" s="145"/>
       <c r="BW112" s="56"/>
       <c r="BX112" s="11"/>
       <c r="BY112" s="45"/>
@@ -11745,13 +11724,13 @@
       <c r="BM113" s="45"/>
       <c r="BN113" s="45"/>
       <c r="BO113" s="45"/>
-      <c r="BP113" s="133"/>
-      <c r="BQ113" s="133"/>
-      <c r="BR113" s="133"/>
-      <c r="BS113" s="133"/>
-      <c r="BT113" s="133"/>
-      <c r="BU113" s="133"/>
-      <c r="BV113" s="133"/>
+      <c r="BP113" s="145"/>
+      <c r="BQ113" s="145"/>
+      <c r="BR113" s="145"/>
+      <c r="BS113" s="145"/>
+      <c r="BT113" s="145"/>
+      <c r="BU113" s="145"/>
+      <c r="BV113" s="145"/>
       <c r="BW113" s="56"/>
       <c r="BX113" s="11"/>
       <c r="BY113" s="45"/>
@@ -11773,13 +11752,13 @@
       <c r="BM114" s="45"/>
       <c r="BN114" s="45"/>
       <c r="BO114" s="45"/>
-      <c r="BP114" s="133"/>
-      <c r="BQ114" s="133"/>
-      <c r="BR114" s="133"/>
-      <c r="BS114" s="133"/>
-      <c r="BT114" s="133"/>
-      <c r="BU114" s="133"/>
-      <c r="BV114" s="133"/>
+      <c r="BP114" s="145"/>
+      <c r="BQ114" s="145"/>
+      <c r="BR114" s="145"/>
+      <c r="BS114" s="145"/>
+      <c r="BT114" s="145"/>
+      <c r="BU114" s="145"/>
+      <c r="BV114" s="145"/>
       <c r="BW114" s="56"/>
       <c r="BX114" s="11"/>
       <c r="BY114" s="45"/>
@@ -11801,13 +11780,13 @@
       <c r="BM115" s="45"/>
       <c r="BN115" s="45"/>
       <c r="BO115" s="45"/>
-      <c r="BP115" s="133"/>
-      <c r="BQ115" s="133"/>
-      <c r="BR115" s="133"/>
-      <c r="BS115" s="133"/>
-      <c r="BT115" s="133"/>
-      <c r="BU115" s="133"/>
-      <c r="BV115" s="133"/>
+      <c r="BP115" s="145"/>
+      <c r="BQ115" s="145"/>
+      <c r="BR115" s="145"/>
+      <c r="BS115" s="145"/>
+      <c r="BT115" s="145"/>
+      <c r="BU115" s="145"/>
+      <c r="BV115" s="145"/>
       <c r="BW115" s="56"/>
       <c r="BX115" s="11"/>
       <c r="BY115" s="45"/>
@@ -12017,16 +11996,16 @@
     </row>
     <row r="123" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG123" s="7"/>
-      <c r="BH123" s="90" t="s">
-        <v>43</v>
+      <c r="BH123" s="126" t="s">
+        <v>74</v>
       </c>
       <c r="BI123" s="6"/>
-      <c r="BJ123" s="90" t="s">
-        <v>44</v>
+      <c r="BJ123" s="126" t="s">
+        <v>75</v>
       </c>
       <c r="BK123" s="6"/>
-      <c r="BL123" s="90" t="s">
-        <v>51</v>
+      <c r="BL123" s="126" t="s">
+        <v>76</v>
       </c>
       <c r="BM123" s="7"/>
       <c r="BN123" s="17"/>
@@ -12035,16 +12014,16 @@
       <c r="BQ123" s="6"/>
       <c r="BR123" s="17"/>
       <c r="BS123" s="6"/>
-      <c r="BT123" s="90" t="s">
-        <v>45</v>
+      <c r="BT123" s="126" t="s">
+        <v>77</v>
       </c>
       <c r="BU123" s="6"/>
-      <c r="BV123" s="90" t="s">
-        <v>46</v>
+      <c r="BV123" s="126" t="s">
+        <v>78</v>
       </c>
       <c r="BW123" s="10"/>
-      <c r="BX123" s="90" t="s">
-        <v>50</v>
+      <c r="BX123" s="126" t="s">
+        <v>79</v>
       </c>
       <c r="BY123" s="7"/>
       <c r="BZ123" s="7"/>
@@ -12057,11 +12036,11 @@
     </row>
     <row r="124" spans="59:84" ht="25.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="BG124" s="7"/>
-      <c r="BH124" s="90"/>
+      <c r="BH124" s="126"/>
       <c r="BI124" s="6"/>
-      <c r="BJ124" s="90"/>
+      <c r="BJ124" s="126"/>
       <c r="BK124" s="6"/>
-      <c r="BL124" s="90"/>
+      <c r="BL124" s="126"/>
       <c r="BM124" s="34"/>
       <c r="BN124" s="17"/>
       <c r="BP124" s="79" t="s">
@@ -12070,11 +12049,11 @@
       <c r="BQ124" s="6"/>
       <c r="BR124" s="17"/>
       <c r="BS124" s="6"/>
-      <c r="BT124" s="90"/>
+      <c r="BT124" s="126"/>
       <c r="BU124" s="6"/>
-      <c r="BV124" s="90"/>
+      <c r="BV124" s="126"/>
       <c r="BW124" s="10"/>
-      <c r="BX124" s="90"/>
+      <c r="BX124" s="126"/>
       <c r="BY124" s="7"/>
       <c r="BZ124" s="7"/>
       <c r="CA124" s="69"/>
@@ -12086,11 +12065,11 @@
     </row>
     <row r="125" spans="59:84" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="BG125" s="7"/>
-      <c r="BH125" s="90"/>
+      <c r="BH125" s="126"/>
       <c r="BI125" s="6"/>
-      <c r="BJ125" s="90"/>
+      <c r="BJ125" s="126"/>
       <c r="BK125" s="6"/>
-      <c r="BL125" s="90"/>
+      <c r="BL125" s="126"/>
       <c r="BM125" s="7"/>
       <c r="BN125" s="17"/>
       <c r="BO125" s="6"/>
@@ -12098,11 +12077,11 @@
       <c r="BQ125" s="6"/>
       <c r="BR125" s="17"/>
       <c r="BS125" s="6"/>
-      <c r="BT125" s="90"/>
+      <c r="BT125" s="126"/>
       <c r="BU125" s="6"/>
-      <c r="BV125" s="90"/>
+      <c r="BV125" s="126"/>
       <c r="BW125" s="10"/>
-      <c r="BX125" s="90"/>
+      <c r="BX125" s="126"/>
       <c r="BY125" s="7"/>
       <c r="BZ125" s="7"/>
       <c r="CA125" s="69"/>
@@ -12271,11 +12250,11 @@
       <c r="BV131" s="7"/>
       <c r="BW131" s="10"/>
       <c r="BX131" s="7"/>
-      <c r="BY131" s="124" t="s">
-        <v>52</v>
-      </c>
-      <c r="BZ131" s="125"/>
-      <c r="CA131" s="126"/>
+      <c r="BY131" s="136" t="s">
+        <v>46</v>
+      </c>
+      <c r="BZ131" s="137"/>
+      <c r="CA131" s="138"/>
       <c r="CB131" s="69"/>
       <c r="CC131" s="60"/>
       <c r="CD131" s="61"/>
@@ -12290,28 +12269,28 @@
       <c r="BK132" s="7"/>
       <c r="BL132" s="7"/>
       <c r="BM132" s="7"/>
-      <c r="BN132" s="120" t="s">
-        <v>71</v>
-      </c>
-      <c r="BO132" s="121"/>
-      <c r="BP132" s="121"/>
-      <c r="BQ132" s="121"/>
-      <c r="BR132" s="122"/>
+      <c r="BN132" s="132" t="s">
+        <v>80</v>
+      </c>
+      <c r="BO132" s="133"/>
+      <c r="BP132" s="133"/>
+      <c r="BQ132" s="133"/>
+      <c r="BR132" s="134"/>
       <c r="BS132" s="7"/>
       <c r="BT132" s="7"/>
       <c r="BU132" s="7"/>
       <c r="BV132" s="7"/>
       <c r="BW132" s="10"/>
       <c r="BX132" s="7"/>
-      <c r="BY132" s="127"/>
-      <c r="BZ132" s="128"/>
-      <c r="CA132" s="129"/>
+      <c r="BY132" s="139"/>
+      <c r="BZ132" s="140"/>
+      <c r="CA132" s="141"/>
       <c r="CB132" s="69"/>
-      <c r="CC132" s="109" t="s">
-        <v>47</v>
-      </c>
-      <c r="CD132" s="110"/>
-      <c r="CE132" s="111"/>
+      <c r="CC132" s="121" t="s">
+        <v>43</v>
+      </c>
+      <c r="CD132" s="122"/>
+      <c r="CE132" s="123"/>
       <c r="CF132" s="7"/>
     </row>
     <row r="133" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -12322,24 +12301,24 @@
       <c r="BK133" s="7"/>
       <c r="BL133" s="7"/>
       <c r="BM133" s="7"/>
-      <c r="BN133" s="123"/>
-      <c r="BO133" s="121"/>
-      <c r="BP133" s="121"/>
-      <c r="BQ133" s="121"/>
-      <c r="BR133" s="122"/>
+      <c r="BN133" s="135"/>
+      <c r="BO133" s="133"/>
+      <c r="BP133" s="133"/>
+      <c r="BQ133" s="133"/>
+      <c r="BR133" s="134"/>
       <c r="BS133" s="7"/>
       <c r="BT133" s="7"/>
       <c r="BU133" s="7"/>
       <c r="BV133" s="7"/>
       <c r="BW133" s="10"/>
       <c r="BX133" s="7"/>
-      <c r="BY133" s="127"/>
-      <c r="BZ133" s="128"/>
-      <c r="CA133" s="129"/>
+      <c r="BY133" s="139"/>
+      <c r="BZ133" s="140"/>
+      <c r="CA133" s="141"/>
       <c r="CB133" s="69"/>
-      <c r="CC133" s="109"/>
-      <c r="CD133" s="110"/>
-      <c r="CE133" s="111"/>
+      <c r="CC133" s="121"/>
+      <c r="CD133" s="122"/>
+      <c r="CE133" s="123"/>
       <c r="CF133" s="7"/>
     </row>
     <row r="134" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -12350,24 +12329,24 @@
       <c r="BK134" s="7"/>
       <c r="BL134" s="7"/>
       <c r="BM134" s="7"/>
-      <c r="BN134" s="123"/>
-      <c r="BO134" s="121"/>
-      <c r="BP134" s="121"/>
-      <c r="BQ134" s="121"/>
-      <c r="BR134" s="122"/>
+      <c r="BN134" s="135"/>
+      <c r="BO134" s="133"/>
+      <c r="BP134" s="133"/>
+      <c r="BQ134" s="133"/>
+      <c r="BR134" s="134"/>
       <c r="BS134" s="7"/>
       <c r="BT134" s="7"/>
       <c r="BU134" s="7"/>
       <c r="BV134" s="7"/>
       <c r="BW134" s="10"/>
       <c r="BX134" s="7"/>
-      <c r="BY134" s="127"/>
-      <c r="BZ134" s="128"/>
-      <c r="CA134" s="129"/>
+      <c r="BY134" s="139"/>
+      <c r="BZ134" s="140"/>
+      <c r="CA134" s="141"/>
       <c r="CB134" s="69"/>
-      <c r="CC134" s="109"/>
-      <c r="CD134" s="110"/>
-      <c r="CE134" s="111"/>
+      <c r="CC134" s="121"/>
+      <c r="CD134" s="122"/>
+      <c r="CE134" s="123"/>
       <c r="CF134" s="7"/>
     </row>
     <row r="135" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -12378,24 +12357,24 @@
       <c r="BK135" s="7"/>
       <c r="BL135" s="7"/>
       <c r="BM135" s="7"/>
-      <c r="BN135" s="123"/>
-      <c r="BO135" s="121"/>
-      <c r="BP135" s="121"/>
-      <c r="BQ135" s="121"/>
-      <c r="BR135" s="122"/>
+      <c r="BN135" s="135"/>
+      <c r="BO135" s="133"/>
+      <c r="BP135" s="133"/>
+      <c r="BQ135" s="133"/>
+      <c r="BR135" s="134"/>
       <c r="BS135" s="7"/>
       <c r="BT135" s="7"/>
       <c r="BU135" s="7"/>
       <c r="BV135" s="7"/>
       <c r="BW135" s="10"/>
       <c r="BX135" s="7"/>
-      <c r="BY135" s="127"/>
-      <c r="BZ135" s="128"/>
-      <c r="CA135" s="129"/>
+      <c r="BY135" s="139"/>
+      <c r="BZ135" s="140"/>
+      <c r="CA135" s="141"/>
       <c r="CB135" s="69"/>
-      <c r="CC135" s="109"/>
-      <c r="CD135" s="110"/>
-      <c r="CE135" s="111"/>
+      <c r="CC135" s="121"/>
+      <c r="CD135" s="122"/>
+      <c r="CE135" s="123"/>
       <c r="CF135" s="7"/>
     </row>
     <row r="136" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -12406,24 +12385,24 @@
       <c r="BK136" s="7"/>
       <c r="BL136" s="7"/>
       <c r="BM136" s="7"/>
-      <c r="BN136" s="123"/>
-      <c r="BO136" s="121"/>
-      <c r="BP136" s="121"/>
-      <c r="BQ136" s="121"/>
-      <c r="BR136" s="122"/>
+      <c r="BN136" s="135"/>
+      <c r="BO136" s="133"/>
+      <c r="BP136" s="133"/>
+      <c r="BQ136" s="133"/>
+      <c r="BR136" s="134"/>
       <c r="BS136" s="7"/>
       <c r="BT136" s="7"/>
       <c r="BU136" s="7"/>
       <c r="BV136" s="7"/>
       <c r="BW136" s="10"/>
       <c r="BX136" s="7"/>
-      <c r="BY136" s="127"/>
-      <c r="BZ136" s="128"/>
-      <c r="CA136" s="129"/>
+      <c r="BY136" s="139"/>
+      <c r="BZ136" s="140"/>
+      <c r="CA136" s="141"/>
       <c r="CB136" s="69"/>
-      <c r="CC136" s="109"/>
-      <c r="CD136" s="110"/>
-      <c r="CE136" s="111"/>
+      <c r="CC136" s="121"/>
+      <c r="CD136" s="122"/>
+      <c r="CE136" s="123"/>
       <c r="CF136" s="7"/>
     </row>
     <row r="137" spans="59:84 1257:1257" x14ac:dyDescent="0.3">
@@ -12445,9 +12424,9 @@
       <c r="BV137" s="7"/>
       <c r="BW137" s="10"/>
       <c r="BX137" s="7"/>
-      <c r="BY137" s="130"/>
-      <c r="BZ137" s="131"/>
-      <c r="CA137" s="132"/>
+      <c r="BY137" s="142"/>
+      <c r="BZ137" s="143"/>
+      <c r="CA137" s="144"/>
       <c r="CB137" s="69"/>
       <c r="CC137" s="63"/>
       <c r="CD137" s="64"/>
@@ -12621,23 +12600,44 @@
     </row>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="R62:V62"/>
-    <mergeCell ref="U44:X45"/>
-    <mergeCell ref="U49:X51"/>
-    <mergeCell ref="U52:X54"/>
-    <mergeCell ref="U37:V40"/>
-    <mergeCell ref="U46:W46"/>
-    <mergeCell ref="T40:T49"/>
-    <mergeCell ref="E34:I35"/>
-    <mergeCell ref="N33:P34"/>
-    <mergeCell ref="T38:T39"/>
-    <mergeCell ref="S34:U34"/>
-    <mergeCell ref="AP45:AT46"/>
-    <mergeCell ref="AE34:AI35"/>
-    <mergeCell ref="O45:O46"/>
-    <mergeCell ref="O41:O42"/>
-    <mergeCell ref="O43:O44"/>
-    <mergeCell ref="AS34:AU34"/>
+    <mergeCell ref="CR32:CX33"/>
+    <mergeCell ref="DD10:DD24"/>
+    <mergeCell ref="DF26:DK27"/>
+    <mergeCell ref="CQ17:CQ30"/>
+    <mergeCell ref="BY76:CE79"/>
+    <mergeCell ref="BH123:BH125"/>
+    <mergeCell ref="AN63:AX64"/>
+    <mergeCell ref="AN65:AX66"/>
+    <mergeCell ref="AN61:AX62"/>
+    <mergeCell ref="AO57:AO58"/>
+    <mergeCell ref="AO55:AO56"/>
+    <mergeCell ref="CC132:CE136"/>
+    <mergeCell ref="BL82:BL83"/>
+    <mergeCell ref="CB82:CB83"/>
+    <mergeCell ref="BI98:BW102"/>
+    <mergeCell ref="BX123:BX125"/>
+    <mergeCell ref="BL123:BL125"/>
+    <mergeCell ref="BZ86:CA87"/>
+    <mergeCell ref="CC88:CD89"/>
+    <mergeCell ref="BV123:BV125"/>
+    <mergeCell ref="BT123:BT125"/>
+    <mergeCell ref="BJ123:BJ125"/>
+    <mergeCell ref="BN132:BR136"/>
+    <mergeCell ref="BY131:CA137"/>
+    <mergeCell ref="BP111:BV115"/>
+    <mergeCell ref="BH76:BV78"/>
+    <mergeCell ref="O47:O48"/>
+    <mergeCell ref="O49:O50"/>
+    <mergeCell ref="P48:R49"/>
+    <mergeCell ref="AC39:AC40"/>
+    <mergeCell ref="AK39:AK40"/>
+    <mergeCell ref="N60:P61"/>
+    <mergeCell ref="R60:V61"/>
+    <mergeCell ref="O55:O56"/>
+    <mergeCell ref="O57:O58"/>
+    <mergeCell ref="T51:T55"/>
+    <mergeCell ref="O51:O52"/>
+    <mergeCell ref="O53:O54"/>
     <mergeCell ref="AP48:AR49"/>
     <mergeCell ref="AO49:AO50"/>
     <mergeCell ref="AM33:AQ34"/>
@@ -12654,44 +12654,23 @@
     <mergeCell ref="AO47:AO48"/>
     <mergeCell ref="AO51:AO52"/>
     <mergeCell ref="AO53:AO54"/>
-    <mergeCell ref="N60:P61"/>
-    <mergeCell ref="R60:V61"/>
-    <mergeCell ref="O55:O56"/>
-    <mergeCell ref="O57:O58"/>
-    <mergeCell ref="T51:T55"/>
-    <mergeCell ref="O51:O52"/>
-    <mergeCell ref="O53:O54"/>
-    <mergeCell ref="O47:O48"/>
-    <mergeCell ref="O49:O50"/>
-    <mergeCell ref="P48:R49"/>
-    <mergeCell ref="AC39:AC40"/>
-    <mergeCell ref="AK39:AK40"/>
-    <mergeCell ref="AO55:AO56"/>
-    <mergeCell ref="CC132:CE136"/>
-    <mergeCell ref="BL82:BL83"/>
-    <mergeCell ref="CB82:CB83"/>
-    <mergeCell ref="BI98:BW102"/>
-    <mergeCell ref="BX123:BX125"/>
-    <mergeCell ref="BL123:BL125"/>
-    <mergeCell ref="BZ86:CA87"/>
-    <mergeCell ref="CC88:CD89"/>
-    <mergeCell ref="BV123:BV125"/>
-    <mergeCell ref="BT123:BT125"/>
-    <mergeCell ref="BJ123:BJ125"/>
-    <mergeCell ref="BN132:BR136"/>
-    <mergeCell ref="BY131:CA137"/>
-    <mergeCell ref="BP111:BV115"/>
-    <mergeCell ref="BH76:BV78"/>
-    <mergeCell ref="BH123:BH125"/>
-    <mergeCell ref="AN63:AX64"/>
-    <mergeCell ref="AN65:AX66"/>
-    <mergeCell ref="AN61:AX62"/>
-    <mergeCell ref="AO57:AO58"/>
-    <mergeCell ref="CR32:CX33"/>
-    <mergeCell ref="DD10:DD24"/>
-    <mergeCell ref="DF26:DK27"/>
-    <mergeCell ref="CQ17:CQ30"/>
-    <mergeCell ref="BY76:CE79"/>
+    <mergeCell ref="E34:I35"/>
+    <mergeCell ref="N33:P34"/>
+    <mergeCell ref="T38:T39"/>
+    <mergeCell ref="S34:U34"/>
+    <mergeCell ref="AP45:AT46"/>
+    <mergeCell ref="AE34:AI35"/>
+    <mergeCell ref="O45:O46"/>
+    <mergeCell ref="O41:O42"/>
+    <mergeCell ref="O43:O44"/>
+    <mergeCell ref="AS34:AU34"/>
+    <mergeCell ref="R62:V62"/>
+    <mergeCell ref="U44:X45"/>
+    <mergeCell ref="U49:X51"/>
+    <mergeCell ref="U52:X54"/>
+    <mergeCell ref="U37:V40"/>
+    <mergeCell ref="U46:W46"/>
+    <mergeCell ref="T40:T49"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>